<commit_message>
Bump plugin to 0.9.0: statement_short column in checklist template; re-sync review generator (v0.3.0)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/checklists/eval_checklist.xlsx
+++ b/tests/fixtures/checklists/eval_checklist.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Architecture, Compute &amp; Infrast" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Enterprise-grade Security, Perm" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Scalable Performance, Stability" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture, Compute &amp; Infrast" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enterprise-grade Security, Perm" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scalable Performance, Stability" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z6"/>
+  <dimension ref="A1:AA6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -444,26 +444,27 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="50" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
     <col width="40" customWidth="1" min="13" max="13"/>
     <col width="40" customWidth="1" min="14" max="14"/>
-    <col width="36" customWidth="1" min="15" max="15"/>
-    <col width="24" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="24" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="40" customWidth="1" min="21" max="21"/>
-    <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="40" customWidth="1" min="23" max="23"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="40" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
     <col width="40" customWidth="1" min="24" max="24"/>
-    <col width="16" customWidth="1" min="25" max="25"/>
-    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="40" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -499,100 +500,105 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>statement_short</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>parameter_hint</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>operator</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>expected_value</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>expected_condition_notes</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>supporting_evidence</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>contradicting_evidence</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>insufficient_evidence_handling</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>rationale</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>dataiku_concepts</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>source_document</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>source_page</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>source_section</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>ambiguity_notes</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>validation_status</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>evidence_found</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>validated_at</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>validated_by</t>
         </is>
@@ -629,62 +635,67 @@
           <t>Production-grade Dataiku deployments should separate experimental/design work from production runs by leveraging dedicated automation nodes; reviewers should discuss the Design -&gt; Deployer -&gt; Automation Node architecture with the customer and flag gaps, even though standing up new nodes is out of scope for the review itself.</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n"/>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Separate production workloads onto dedicated automation nodes rather than running everything on the design node.</t>
+        </is>
+      </c>
       <c r="H2" s="3" t="n"/>
       <c r="I2" s="3" t="n"/>
       <c r="J2" s="3" t="n"/>
       <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>Diagnosis shows a distinct automation node (or nodes) separate from the design node, with a deployer configured and bundles being pushed from design to automation.</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>Only a single design node is used to run both experimentation and production workloads, with no automation node or deployer in use.</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>If the diagnosis file does not expose node topology/roles, flag needs_manual_review and recommend discussing the Design -&gt; Deployer -&gt; Automation architecture directly with the customer.</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>Mixing experimental and production work on the same node risks instability and is not considered production-ready.</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>Design node, Automation node, Deployer, Bundles</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>architecture_compute_cost</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
+      <c r="S2" s="3" t="inlineStr">
         <is>
           <t>1, 2</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>Dataiku Deployment Infrastructure | MUST HAVE; Dataiku Deployment Infrastructure | MUST HAVE</t>
         </is>
       </c>
-      <c r="T2" s="3" t="inlineStr">
+      <c r="U2" s="3" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="U2" s="3" t="n"/>
       <c r="V2" s="3" t="n"/>
       <c r="W2" s="3" t="n"/>
       <c r="X2" s="3" t="n"/>
       <c r="Y2" s="3" t="n"/>
       <c r="Z2" s="3" t="n"/>
+      <c r="AA2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -717,62 +728,67 @@
           <t>Dataiku recommends customers stay reasonably current on DSS versions to benefit from continuous platform improvements; reviewers should identify and recommend an upgrade if appropriate, but the upgrade itself is a separate service-catalog engagement and should not be performed during the review.</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n"/>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Recommend upgrading DSS to a reasonably current version via a separate service engagement.</t>
+        </is>
+      </c>
       <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="n"/>
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Diagnosis shows a DSS version reasonably close to the latest generally available release.</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Diagnosis shows a DSS version many releases behind current, or a version approaching/at end-of-life.</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>If the diagnosis file lacks version information or there is no context on Dataiku's release cadence, flag needs_manual_review and recommend checking DSS release notes for the customer's version.</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>Dataiku regularly enriches the platform, so staying current continuously brings value and new opportunities to customers.</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>DSS version, Upgrade</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="R3" s="3" t="inlineStr">
         <is>
           <t>architecture_compute_cost</t>
         </is>
       </c>
-      <c r="R3" s="3" t="inlineStr">
+      <c r="S3" s="3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="S3" s="3" t="inlineStr">
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>Dataiku Version | NICE TO HAVE</t>
         </is>
       </c>
-      <c r="T3" s="3" t="inlineStr">
+      <c r="U3" s="3" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="U3" s="3" t="n"/>
       <c r="V3" s="3" t="n"/>
       <c r="W3" s="3" t="n"/>
       <c r="X3" s="3" t="n"/>
       <c r="Y3" s="3" t="n"/>
       <c r="Z3" s="3" t="n"/>
+      <c r="AA3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -805,62 +821,67 @@
           <t>DSS should run on SSD drives rather than legacy rotational hard drives, since rotational disks can significantly degrade performance, especially on larger, multi-user instances (potentially causing a non-workable experience); reviewers should identify currently used disk types and recommend migration to SSD where feasible, noting this is typically easier on cloud than on-premise deployments.</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n"/>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Run DSS on SSD storage instead of rotational hard drives for performance.</t>
+        </is>
+      </c>
       <c r="H4" s="3" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
       <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Diagnosis or infrastructure metadata indicates SSD-backed storage underlying the DATADIR.</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Diagnosis or infrastructure metadata indicates rotational HDD storage is in use, particularly on a larger or many-user instance.</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>If the diagnosis file does not report the underlying disk/storage medium, flag needs_manual_review and ask the infrastructure team/customer directly.</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Rotational hard drives can severely impact performance and, on larger instances with many users, may lead to a non-workable experience.</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>Disk I/O, SSD, DATADIR</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr">
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>architecture_compute_cost</t>
         </is>
       </c>
-      <c r="R4" s="3" t="inlineStr">
+      <c r="S4" s="3" t="inlineStr">
         <is>
           <t>2, 3</t>
         </is>
       </c>
-      <c r="S4" s="3" t="inlineStr">
+      <c r="T4" s="3" t="inlineStr">
         <is>
           <t>Use of SSDs | MUST HAVE; Use of SSDs | MUST HAVE</t>
         </is>
       </c>
-      <c r="T4" s="3" t="inlineStr">
+      <c r="U4" s="3" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="U4" s="3" t="n"/>
       <c r="V4" s="3" t="n"/>
       <c r="W4" s="3" t="n"/>
       <c r="X4" s="3" t="n"/>
       <c r="Y4" s="3" t="n"/>
       <c r="Z4" s="3" t="n"/>
+      <c r="AA4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -895,76 +916,81 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
+          <t>Configure at least one valid containerized execution config when using Elastic Compute.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
           <t>general-settings.json &gt; containerSettings</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>exists</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>valid containerized execution configuration present</t>
         </is>
       </c>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Required only when the customer uses Elastic Compute/Kubernetes for offloaded workloads.</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>containerSettings block is present with at least one named config with reasonable memory requests/limits.</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>containerSettings is missing or empty while the instance shows evidence of Kubernetes-based execution elsewhere in the diagnosis.</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>If the diagnosis file does not clarify whether Elastic Compute is used, flag needs_manual_review.</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr">
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>A valid container exec config is required to run workloads in Kubernetes.</t>
         </is>
       </c>
-      <c r="P5" s="3" t="inlineStr">
+      <c r="Q5" s="3" t="inlineStr">
         <is>
           <t>Containerized execution, containerSettings, Elastic Compute</t>
         </is>
       </c>
-      <c r="Q5" s="3" t="inlineStr">
+      <c r="R5" s="3" t="inlineStr">
         <is>
           <t>architecture_compute_cost</t>
         </is>
       </c>
-      <c r="R5" s="3" t="inlineStr">
+      <c r="S5" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="S5" s="3" t="inlineStr">
+      <c r="T5" s="3" t="inlineStr">
         <is>
           <t>Containerized execution configs | MUST HAVE if using Elastic Compute</t>
         </is>
       </c>
-      <c r="T5" s="3" t="inlineStr">
+      <c r="U5" s="3" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="U5" s="3" t="n"/>
       <c r="V5" s="3" t="n"/>
       <c r="W5" s="3" t="n"/>
       <c r="X5" s="3" t="n"/>
       <c r="Y5" s="3" t="n"/>
       <c r="Z5" s="3" t="n"/>
+      <c r="AA5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -999,72 +1025,77 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
+          <t>Configure at least one valid Kubernetes cluster when using Elastic Compute.</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
           <t>{DATADIR}/config/clusters</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>exists</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>at least one valid cluster configuration present</t>
         </is>
       </c>
-      <c r="J6" s="3" t="n"/>
       <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="L6" s="3" t="n"/>
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>The clusters config/directory contains at least one properly defined cluster, consistent with other evidence of elastic-compute usage (spark/container jobs running on Kubernetes).</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>No cluster configuration is present despite evidence of Kubernetes-based workloads elsewhere in the diagnosis.</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="O6" s="3" t="inlineStr">
         <is>
           <t>If the diagnosis file does not clarify whether Elastic Compute is used at all, flag needs_manual_review.</t>
         </is>
       </c>
-      <c r="O6" s="3" t="inlineStr">
+      <c r="P6" s="3" t="inlineStr">
         <is>
           <t>A valid cluster is required to offload computation to Kubernetes.</t>
         </is>
       </c>
-      <c r="P6" s="3" t="inlineStr">
+      <c r="Q6" s="3" t="inlineStr">
         <is>
           <t>Cluster, Managed cluster, Unmanaged cluster, Elastic AI</t>
         </is>
       </c>
-      <c r="Q6" s="3" t="inlineStr">
+      <c r="R6" s="3" t="inlineStr">
         <is>
           <t>architecture_compute_cost</t>
         </is>
       </c>
-      <c r="R6" s="3" t="inlineStr">
+      <c r="S6" s="3" t="inlineStr">
         <is>
           <t>12, 13</t>
         </is>
       </c>
-      <c r="S6" s="3" t="inlineStr">
+      <c r="T6" s="3" t="inlineStr">
         <is>
           <t>Cluster configurations | MUST HAVE if using Elastic Compute; Cluster configurations | MUST HAVE if using Elastic Compute</t>
         </is>
       </c>
-      <c r="T6" s="3" t="inlineStr">
+      <c r="U6" s="3" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="U6" s="3" t="n"/>
       <c r="V6" s="3" t="n"/>
       <c r="W6" s="3" t="n"/>
       <c r="X6" s="3" t="n"/>
       <c r="Y6" s="3" t="n"/>
       <c r="Z6" s="3" t="n"/>
+      <c r="AA6" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1077,7 +1108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z3"/>
+  <dimension ref="A1:AA3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1086,26 +1117,27 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="50" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
     <col width="40" customWidth="1" min="13" max="13"/>
     <col width="40" customWidth="1" min="14" max="14"/>
-    <col width="36" customWidth="1" min="15" max="15"/>
-    <col width="24" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="24" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="40" customWidth="1" min="21" max="21"/>
-    <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="40" customWidth="1" min="23" max="23"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="40" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
     <col width="40" customWidth="1" min="24" max="24"/>
-    <col width="16" customWidth="1" min="25" max="25"/>
-    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="40" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1141,100 +1173,105 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>statement_short</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>parameter_hint</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>operator</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>expected_value</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>expected_condition_notes</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>supporting_evidence</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>contradicting_evidence</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>insufficient_evidence_handling</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>rationale</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>dataiku_concepts</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>source_document</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>source_page</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>source_section</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>ambiguity_notes</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>validation_status</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>evidence_found</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>validated_at</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>validated_by</t>
         </is>
@@ -1273,76 +1310,81 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
+          <t>Enable cgroups with a memory limit sized per the recommended heuristic for instance RAM.</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
           <t>{DATA_DIR}/config/general-settings.json &gt; cgroupSettings.enabled</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>equals</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>Additional checks required: cgroupSettings &gt; cgroups memory limit target should be set and sized per the documented heuristic (approx. 50-75% of physical memory depending on total RAM); no single literal field given for the limit value itself, so compare against the formula in evaluation_guidance.</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>general-settings.json shows cgroupSettings.enabled: true, targets set for each category under cgroups, and a memory limit configured on memory cgroups (e.g., memory/DSS) that approximates the documented formula based on total instance memory (e.g., ~75% for &gt;120GB, ~66% for 60-120GB, total-20GB for 30-60GB, ~50% below 30GB). Front-end equivalent: Administration &gt; Settings &gt; Resource Control &gt; cgroups shows 'Enable cgroups support' selected with placements and memory limits configured.</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>cgroupSettings.enabled is false/absent, no memory limit is set on memory cgroups, or the configured limit is far below the heuristic (e.g., unlimited or near-total memory), risking instability.</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>If cgroupSettings or category placements are not visible in the diagnosis file, flag as needs_manual_review; also check whether the instance was recently reprovisioned (Cloud Stacks) or upgraded, as cgroup limits/placements may not auto-update and new placements may need to be added post-upgrade.</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>A memory cgroup limit prevents runaway processes from destabilizing or degrading the DSS instance; sizing per the heuristic balances safety with usable memory.</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>cgroups, memory limits, Resource Control</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>security_permissions_compliance</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
+      <c r="S2" s="3" t="inlineStr">
         <is>
           <t>3, 4, 5</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>CGroups | MUST HAVE; CGroups | MUST HAVE (Review steps); CGroups | MUST HAVE (Notes)</t>
         </is>
       </c>
-      <c r="T2" s="3" t="inlineStr">
+      <c r="U2" s="3" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="U2" s="3" t="n"/>
       <c r="V2" s="3" t="n"/>
       <c r="W2" s="3" t="n"/>
       <c r="X2" s="3" t="n"/>
       <c r="Y2" s="3" t="n"/>
       <c r="Z2" s="3" t="n"/>
+      <c r="AA2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1377,76 +1419,81 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
+          <t>Verify HTTPS access to DSS is configured natively or via a reverse proxy.</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
           <t>install.ini &gt; [server] section (HTTPS settings) or /data/dataiku/dss_data/run/nodes-directory.json</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>exists</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>HTTPS enabled (natively or via reverse proxy)</t>
         </is>
       </c>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>No single literal key name given for the HTTPS flag itself; pointer is to the file/section where it should be inspected.</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>install.ini [server] section shows native HTTPS parameters configured, or nodes-directory.json shows HTTPS URLs/ports for nodes, or customer confirms a reverse proxy terminates HTTPS in front of DSS.</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Only HTTP is configured with no reverse proxy in front, and install.ini/nodes-directory.json show no HTTPS-related configuration.</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>If the diagnosis file does not include install.ini or nodes-directory.json content, or if reverse-proxy setup is external to DSS, flag as needs_manual_review and confirm directly with the customer.</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>HTTPS protects data in transit and is recommended practice for securing access to DSS.</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>HTTPS, reverse proxy, install.ini, nodes-directory.json</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="R3" s="3" t="inlineStr">
         <is>
           <t>security_permissions_compliance</t>
         </is>
       </c>
-      <c r="R3" s="3" t="inlineStr">
+      <c r="S3" s="3" t="inlineStr">
         <is>
           <t>5, 6</t>
         </is>
       </c>
-      <c r="S3" s="3" t="inlineStr">
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>HTTPS | NICE TO HAVE; HTTPS | NICE TO HAVE (Review steps)</t>
         </is>
       </c>
-      <c r="T3" s="3" t="inlineStr">
+      <c r="U3" s="3" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="U3" s="3" t="n"/>
       <c r="V3" s="3" t="n"/>
       <c r="W3" s="3" t="n"/>
       <c r="X3" s="3" t="n"/>
       <c r="Y3" s="3" t="n"/>
       <c r="Z3" s="3" t="n"/>
+      <c r="AA3" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1459,7 +1506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z5"/>
+  <dimension ref="A1:AA5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1468,26 +1515,27 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="50" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
     <col width="40" customWidth="1" min="13" max="13"/>
     <col width="40" customWidth="1" min="14" max="14"/>
-    <col width="36" customWidth="1" min="15" max="15"/>
-    <col width="24" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="24" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="40" customWidth="1" min="21" max="21"/>
-    <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="40" customWidth="1" min="23" max="23"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="40" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
     <col width="40" customWidth="1" min="24" max="24"/>
-    <col width="16" customWidth="1" min="25" max="25"/>
-    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="40" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1523,100 +1571,105 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>statement_short</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>parameter_hint</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>operator</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>expected_value</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>expected_condition_notes</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>supporting_evidence</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>contradicting_evidence</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>insufficient_evidence_handling</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>rationale</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>dataiku_concepts</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>source_document</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>source_page</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>source_section</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>ambiguity_notes</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>validation_status</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>evidence_found</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>validated_at</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>validated_by</t>
         </is>
@@ -1653,62 +1706,67 @@
           <t>Review recent backend.log files (including rotated/zipped logs) for ERROR or FATAL level entries indicating systemic issues such as repeating stack traces, connection failures, or plugin crashes; investigate patterns that recur frequently even without explicit user complaints.</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n"/>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Review backend.log for recurring ERROR/FATAL entries indicating systemic stability issues.</t>
+        </is>
+      </c>
       <c r="H2" s="3" t="n"/>
       <c r="I2" s="3" t="n"/>
       <c r="J2" s="3" t="n"/>
       <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>backend.log and rotated logs show few or no ERROR/FATAL entries, or only isolated non-recurring errors; AI Log Analysis in DiagParser3 shows no systemic issue flagged.</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>Frequent recurring ERROR/FATAL entries (e.g., the same stack trace dozens of times per day), repeated connection failures, or plugin crashes.</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>If logs aren't included or available in the diagnosis bundle, flag needs_manual_review and request the backend.log files directly.</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>A high volume of repeated errors often points to a systemic issue that needs to be addressed before it impacts instance stability.</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>backend.log, AI Log Analysis, DiagParser3</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>scalable_performance_ops</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
+      <c r="S2" s="3" t="inlineStr">
         <is>
           <t>6, 7</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>Backend.log Errors | MUST HAVE; Backend.log Errors | MUST HAVE</t>
         </is>
       </c>
-      <c r="T2" s="3" t="inlineStr">
+      <c r="U2" s="3" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="U2" s="3" t="n"/>
       <c r="V2" s="3" t="n"/>
       <c r="W2" s="3" t="n"/>
       <c r="X2" s="3" t="n"/>
       <c r="Y2" s="3" t="n"/>
       <c r="Z2" s="3" t="n"/>
+      <c r="AA2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1743,80 +1801,85 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
+          <t>Size backend.xmx per the memory heuristic, at least 3x the config folder size.</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
           <t>install.ini &gt; backend.xmx</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>greater_than_or_equal</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>per Cloud Stacks heuristic tier (4g/8g/16g based on system RAM) and &gt;=3x config folder size</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Also verify jek.xmx/fek.xmx are not oversized, and that xmx avoids the 32GB&lt;=xmx&lt;48GB dead zone (jump to 48GB instead) due to Java Ordinary Object Pointer behavior.</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>install.ini backend.xmx matches or exceeds the recommended tier for system memory, is &gt;=3x config folder size, and avoids the 32-48GB dead zone; no OutOfMemoryError entries in backend.log.</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>backend.xmx set below the recommended heuristic, falls in the 32GB-48GB dead zone, or backend.log shows recurring 'OutOfMemoryError: Java heap space' / 'OutOfMemoryError: GC Overhead limit exceeded' entries.</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>If install.ini or system memory info is not present in the diagnosis, flag needs_manual_review and request system specs and install.ini contents.</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>Insufficient or misconfigured heap sizing leads to OutOfMemory errors and instability; oversizing into the 32-48GB range paradoxically reduces available memory due to JVM pointer compression behavior.</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>backend.xmx, jek.xmx, fek.xmx, JVM memory, OutOfMemoryError</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="R3" s="3" t="inlineStr">
         <is>
           <t>scalable_performance_ops</t>
         </is>
       </c>
-      <c r="R3" s="3" t="inlineStr">
+      <c r="S3" s="3" t="inlineStr">
         <is>
           <t>7, 8</t>
         </is>
       </c>
-      <c r="S3" s="3" t="inlineStr">
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>Backend Xmx | MUST HAVE; Backend Xmx | MUST HAVE</t>
         </is>
       </c>
-      <c r="T3" s="3" t="inlineStr">
+      <c r="U3" s="3" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="U3" s="3" t="n"/>
       <c r="V3" s="3" t="n"/>
       <c r="W3" s="3" t="n"/>
       <c r="X3" s="3" t="n"/>
       <c r="Y3" s="3" t="n"/>
       <c r="Z3" s="3" t="n"/>
+      <c r="AA3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1851,76 +1914,81 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
+          <t>Size Max Jobs and Max Activities via the memory framework; never set Max Jobs to zero.</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
           <t>general-settings.json &gt; maxRunningJobs</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>not_equals</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Also verify general-settings.json &gt; maxRunningActivities falls within 30-50, and maxRunningActivitiesPerJob is at the default of 5 unless justified. Front-end equivalent: Administration &gt; Settings &gt; Resources control &gt; Concurrent Activities.</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>maxRunningJobs set to a positive nonzero value derived from the 5-step memory sizing framework; maxRunningActivities within 30-50; maxRunningActivitiesPerJob at 5 (or a justified alternative).</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>maxRunningJobs is 0 or blank (critical stability risk); maxRunningActivities is outside 30-50 without justification; sizing doesn't account for available host memory, risking OOM.</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>If these general-settings.json values are missing from the diagnosis, flag needs_manual_review and check the Administration &gt; Settings &gt; Resources control UI directly.</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Improperly sized flow limits risk instance-wide Out-Of-Memory crashes; Max Jobs=0 disables protection entirely.</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>Flow limits, Max Jobs, Max Activities, CGroups, JEK, memory sizing</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr">
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>scalable_performance_ops</t>
         </is>
       </c>
-      <c r="R4" s="3" t="inlineStr">
+      <c r="S4" s="3" t="inlineStr">
         <is>
           <t>8, 9, 10, 11</t>
         </is>
       </c>
-      <c r="S4" s="3" t="inlineStr">
+      <c r="T4" s="3" t="inlineStr">
         <is>
           <t>Flow parallelism | MUST HAVE; Flow parallelism | MUST HAVE; Flow parallelism | MUST HAVE; Flow parallelism | MUST HAVE</t>
         </is>
       </c>
-      <c r="T4" s="3" t="inlineStr">
+      <c r="U4" s="3" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="U4" s="3" t="n"/>
       <c r="V4" s="3" t="n"/>
       <c r="W4" s="3" t="n"/>
       <c r="X4" s="3" t="n"/>
       <c r="Y4" s="3" t="n"/>
       <c r="Z4" s="3" t="n"/>
+      <c r="AA4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1955,76 +2023,81 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
+          <t>Remove the filesystem_root connection unless actively used, replacing it with a scoped connection.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
           <t>connections.json &gt; filesystem_root</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>not_exists</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>removed (unless replaced by a scoped connection after confirming no active project usage)</t>
         </is>
       </c>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Check usage via Administration -&gt; Monitoring before deletion.</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>filesystem_root connection absent from the connections list, or confirmed unused and removed; if it was in use, a dedicated scoped connection was created to replace it.</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>filesystem_root connection still present and either unused (should have been deleted) or in use without a safer scoped replacement.</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>If the connections list isn't in the diagnosis, flag needs_manual_review and check the Administration &gt; Connections UI directly.</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr">
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>The filesystem_root connection exposes the entire server filesystem, posing a security and stability risk.</t>
         </is>
       </c>
-      <c r="P5" s="3" t="inlineStr">
+      <c r="Q5" s="3" t="inlineStr">
         <is>
           <t>connections, filesystem_root, security</t>
         </is>
       </c>
-      <c r="Q5" s="3" t="inlineStr">
+      <c r="R5" s="3" t="inlineStr">
         <is>
           <t>scalable_performance_ops</t>
         </is>
       </c>
-      <c r="R5" s="3" t="inlineStr">
+      <c r="S5" s="3" t="inlineStr">
         <is>
           <t>14, 15</t>
         </is>
       </c>
-      <c r="S5" s="3" t="inlineStr">
+      <c r="T5" s="3" t="inlineStr">
         <is>
           <t>Remove filesystem_root connection | MUST HAVE; Remove filesystem_root connection | MUST HAVE</t>
         </is>
       </c>
-      <c r="T5" s="3" t="inlineStr">
+      <c r="U5" s="3" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="U5" s="3" t="n"/>
       <c r="V5" s="3" t="n"/>
       <c r="W5" s="3" t="n"/>
       <c r="X5" s="3" t="n"/>
       <c r="Y5" s="3" t="n"/>
       <c r="Z5" s="3" t="n"/>
+      <c r="AA5" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Release 0.24.0: fixed statuses for SCALE-007, GENAI-001, GENAI-009 calibrations to stabilise run-to-run counts
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/checklists/eval_checklist.xlsx
+++ b/tests/fixtures/checklists/eval_checklist.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture, Compute &amp; Infrast" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enterprise-grade Security, Perm" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scalable Performance, Stability" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Advanced Security Options (DSS " sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generative AI Acceleration &amp; In" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scalable Performance, Stability" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Advanced Security Options (DSS " sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1604,6 +1605,392 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:AA3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="40" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="40" customWidth="1" min="24" max="24"/>
+    <col width="40" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>check_type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>subtopic</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>statement</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>statement_short</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>parameter_hint</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>operator</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>expected_value</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>expected_condition_notes</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>supporting_evidence</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>contradicting_evidence</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>insufficient_evidence_handling</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>rationale</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>dataiku_concepts</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>source_document</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>source_page</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>source_section</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>ambiguity_notes</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>validation_status</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>evidence_found</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>validated_at</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>validated_by</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>GENAI-001</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>LLM Mesh and Agents</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Internal Code Environments for RAG, Document Extraction, PII Detection</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Ensure the internal code environments for Retrieval-Augmented Generation, document extraction, and PII detection are properly installed and set as the default code-env for each category under Administration &gt; Settings &gt; Other &gt; LLM Mesh. If a non-internal code-env is used instead, DSS surfaces a warning in the LLM Mesh settings page and in Administration &gt; Code-envs &gt; Internal envs.</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Use internal code environments as default for RAG, document extraction, and PII detection.</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; generativeAISettings &gt; defaultRetrievableKnowledgeCodeEnv</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>not_exists</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>absent (i.e., using internal default code-env, containerMode NONE)</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>If defaultRetrievableKnowledgeCodeEnv is present with a custom value and containerMode is INHERIT, a non-internal code-env is in use. Also check presidioBasedPIIDetection (PII detection) and embedDocumentsRecipeSettings (document extraction) keys for equivalent non-internal overrides.</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json generativeAISettings shows containerMode NONE with no defaultRetrievableKnowledgeCodeEnv key, and PII/doc extraction sections show no custom code-env overrides; Admin &gt; Code-envs &gt; Internal envs shows RAG/PII/Doc extraction set up as internal.</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>defaultRetrievableKnowledgeCodeEnv key present with a non-internal value, containerMode INHERIT, or a warning banner shown in Admin &gt; Settings &gt; Other &gt; LLM Mesh / Code-envs &gt; Internal envs.</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>If generativeAISettings section is absent from the diagnosis, flag needs_manual_review to check the UI directly.</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>Internal code envs bundle the correct/supported dependencies (e.g., libreoffice for document extraction); using a non-internal env can cause missing dependencies or unsupported behavior.</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>LLM Mesh, code environments, RAG, PII detection, document extraction</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>generative_ai_acceleration</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
+      <c r="T2" s="3" t="inlineStr">
+        <is>
+          <t>LLM Mesh and Agents MUST HAVE:; RAG, Doc extraction, PII detection; Instance Diags / DiagParser3</t>
+        </is>
+      </c>
+      <c r="U2" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V2" s="3" t="n"/>
+      <c r="W2" s="3" t="n"/>
+      <c r="X2" s="3" t="n"/>
+      <c r="Y2" s="3" t="n"/>
+      <c r="Z2" s="3" t="n"/>
+      <c r="AA2" s="3" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>GENAI-009</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>nice_to_have</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>qualitative_practice</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub Deployment Required Permissions</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Before a user can deploy an Agent Hub instance, they must have permissions for writing project content in the hosting project, writing isolated code execution, WebApp impersonation, and (if Quick agents are enabled) create projects; alternatively the user could be a DSS administrator, though a dedicated service account is preferred.</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Grant Agent Hub deployers write project content, isolated code execution, and webapp impersonation permissions.</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="n"/>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Administration &gt; Security &gt; Groups shows the Agent Hub deployer's group granted 'Write project content', 'Write isolated code execution', and 'WebApp impersonation' permissions (plus 'Create projects' if Quick agents are enabled), or the deployer is a DSS admin/service account.</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>The deployer's group lacks one or more of these permissions and is not an admin/service account, or logs show 'Not authorized' errors when creating the Agent Hub WebApp.</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file lacks per-user/group permission detail, flag needs_manual_review and recommend checking Administration &gt; Security &gt; Groups directly.</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>Missing permissions cause deployment failures such as 'Not authorized' errors when creating the Agent Hub WebApp.</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub, Permissions, Groups, WebApp</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>generative_ai_acceleration</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>10, 11, 12</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub NICE TO HAVE:; Writing isolated code execution; WebApp impersonation</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>Although the parent topic is tagged NICE TO HAVE, the described permission requirements are phrased as mandatory ('must have permissions') for successful deployment; classification follows the explicit heading tag.</t>
+        </is>
+      </c>
+      <c r="W3" s="3" t="n"/>
+      <c r="X3" s="3" t="n"/>
+      <c r="Y3" s="3" t="n"/>
+      <c r="Z3" s="3" t="n"/>
+      <c r="AA3" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AA5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2202,7 +2589,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Release 0.26.0: calibrations for the 11 items that varied across repeat runs, fixtures extended to 25 items
- Calibrations for SEC-002, SEC-004, SEC-006, ADVSEC-008, ADVSEC-009, SCALE-001/002/003/004,
  ARCH-006, GENAI-007. New general rule: judge only what the bundle shows; live-check aspects go
  in notes as an Action:, not in the status.
- Eval fixtures extended to 25 items covering each new calibration, in both synthetic bundles.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/checklists/eval_checklist.xlsx
+++ b/tests/fixtures/checklists/eval_checklist.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA7"/>
+  <dimension ref="A1:AA8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -888,67 +888,83 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>ARCH-008</t>
+          <t>ARCH-006</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>qualitative_practice</t>
+          <t>specific_setting</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Spark Validation</t>
+          <t>Spark Configuration</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Functional Validation of Spark Execution (Recipe &amp; Notebook)</t>
+          <t>Baseline Spark Configuration Set (High/Standard/Large-memory/High I/O)</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Reviewers should functionally validate Spark execution: run a Spark-engine recipe on Kubernetes in a test project (should succeed), and separately launch a Python/R/Scala notebook with starter Spark code and run it locally (should succeed, with Spark executor pods visible in the cluster while the code runs).</t>
+          <t>Dataiku recommends defining multiple named Spark configurations as a tunable baseline: a default Standard config for recipes and notebooks, a High config for higher parallelism, a Large memory config for the largest jobs, and an optional High I/O config for read/write-heavy workloads with a high cores-to-memory ratio.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Validate Spark execution by successfully running a test Spark recipe and notebook.</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
+          <t>Define Standard, High, Large-memory, and optional High I/O Spark configurations as a baseline.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; sparkSettings (named spark configs)</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>one_of</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Standard/High/Large-memory baseline configs, plus optional High I/O config, as documented</t>
+        </is>
+      </c>
       <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Baseline reference values: Standard config - spark.executor.instances=4, spark.executor.memory=6g, spark.executor.cores=2, spark.kubernetes.memoryOverheadFactor=0.4, spark.driver.memory=1g, spark.sql.shuffle.partitions=40, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. High config - spark.executor.instances=12, spark.executor.memory=6g, spark.executor.cores=2, spark.kubernetes.memoryOverheadFactor=0.4, spark.driver.memory=1g, spark.sql.shuffle.partitions=80, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. Large memory config - spark.executor.instances=4, spark.executor.memory=12g, spark.executor.cores=2, spark.kubernetes.memoryOverheadFactor=0.6, spark.driver.memory=3g, spark.sql.shuffle.partitions=80, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. Optional High I/O config (only if there is a use case for it) - spark.executor.instances=2, spark.executor.memory=16g, spark.executor.cores=8, spark.kubernetes.memoryOverheadFactor=0.4, spark.driver.memory=3g, spark.sql.shuffle.partitions=40, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. These values are guidance, not a requirement.</t>
+        </is>
+      </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>Job/notebook execution logs show successful completion of a Spark recipe and a Spark notebook session, and cluster monitoring shows executor pods created during notebook execution.</t>
+          <t>sparkSettings contains multiple named configs roughly matching these purposes (default/high-parallelism/large-memory, and optionally high I/O).</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>The Spark recipe or notebook execution fails, hangs, or no executor pods ever appear in the cluster.</t>
+          <t>Only a single undifferentiated spark config exists despite varied workload needs (e.g., both lightweight recipes and large jobs run identically).</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file lacks job/notebook execution logs or cluster pod visibility, flag needs_manual_review and recommend running these test steps manually.</t>
+          <t>If the diagnosis file does not list multiple sparkSettings configs or describe workload diversity, flag needs_manual_review and ask about workload variety.</t>
         </is>
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>Confirms Spark integration works end-to-end, beyond just having a syntactically valid configuration.</t>
+          <t>Different Spark workloads (lightweight recipes vs. large jobs vs. I/O-heavy jobs) benefit from different executor sizing and parallelism trade-offs.</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>Spark recipe, Spark notebook, Kubernetes executor pods</t>
+          <t>Spark executor, Spark configuration, Kubernetes</t>
         </is>
       </c>
       <c r="R5" s="3" t="inlineStr">
@@ -958,12 +974,12 @@
       </c>
       <c r="S5" s="3" t="inlineStr">
         <is>
-          <t>5, 6, 7</t>
+          <t>4, 5</t>
         </is>
       </c>
       <c r="T5" s="3" t="inlineStr">
         <is>
-          <t>Additional Spark testing; Spark on Notebook MUST HAVE; Spark on Notebook MUST HAVE</t>
+          <t>Define three spark configs - NICE TO HAVE; Special spark configs (only if there's use case for it)</t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr">
@@ -971,11 +987,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="V5" s="3" t="inlineStr">
-        <is>
-          <t>Worded for Spark on Kubernetes (executor pods). If no Kubernetes cluster is attached and Spark runs on YARN/Hadoop, the pod-based checks do not apply.</t>
-        </is>
-      </c>
+      <c r="V5" s="3" t="n"/>
       <c r="W5" s="3" t="n"/>
       <c r="X5" s="3" t="n"/>
       <c r="Y5" s="3" t="n"/>
@@ -985,7 +997,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>ARCH-010</t>
+          <t>ARCH-008</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -995,73 +1007,57 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>specific_setting</t>
+          <t>qualitative_practice</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Containerized Execution</t>
+          <t>Spark Validation</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Valid Containerized Execution Configuration</t>
+          <t>Functional Validation of Spark Execution (Recipe &amp; Notebook)</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Environments using Elastic Compute (Kubernetes) must have at least one valid containerized execution configuration set up (general-settings.json &gt; containerSettings, or Administration &gt; Settings &gt; Containerized execution); as with Spark, the specific example values are only a baseline, not a strict requirement.</t>
+          <t>Reviewers should functionally validate Spark execution: run a Spark-engine recipe on Kubernetes in a test project (should succeed), and separately launch a Python/R/Scala notebook with starter Spark code and run it locally (should succeed, with Spark executor pods visible in the cluster while the code runs).</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Configure at least one valid containerized execution config when using Elastic Compute.</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>general-settings.json &gt; containerSettings</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>exists</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>valid containerized execution configuration present</t>
-        </is>
-      </c>
+          <t>Validate Spark execution by successfully running a test Spark recipe and notebook.</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
       <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>Required only when the customer uses Elastic Compute/Kubernetes for offloaded workloads.</t>
-        </is>
-      </c>
+      <c r="L6" s="3" t="n"/>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>containerSettings block is present with at least one named config with reasonable memory requests/limits.</t>
+          <t>Job/notebook execution logs show successful completion of a Spark recipe and a Spark notebook session, and cluster monitoring shows executor pods created during notebook execution.</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>containerSettings is missing or empty while the instance shows evidence of Kubernetes-based execution elsewhere in the diagnosis.</t>
+          <t>The Spark recipe or notebook execution fails, hangs, or no executor pods ever appear in the cluster.</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not clarify whether Elastic Compute is used, flag needs_manual_review.</t>
+          <t>If the diagnosis file lacks job/notebook execution logs or cluster pod visibility, flag needs_manual_review and recommend running these test steps manually.</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>A valid container exec config is required to run workloads in Kubernetes.</t>
+          <t>Confirms Spark integration works end-to-end, beyond just having a syntactically valid configuration.</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>Containerized execution, containerSettings, Elastic Compute</t>
+          <t>Spark recipe, Spark notebook, Kubernetes executor pods</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
@@ -1071,12 +1067,12 @@
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5, 6, 7</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>Containerized execution configs | MUST HAVE if using Elastic Compute</t>
+          <t>Additional Spark testing; Spark on Notebook MUST HAVE; Spark on Notebook MUST HAVE</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
@@ -1084,7 +1080,11 @@
           <t>high</t>
         </is>
       </c>
-      <c r="V6" s="3" t="n"/>
+      <c r="V6" s="3" t="inlineStr">
+        <is>
+          <t>Worded for Spark on Kubernetes (executor pods). If no Kubernetes cluster is attached and Spark runs on YARN/Hadoop, the pod-based checks do not apply.</t>
+        </is>
+      </c>
       <c r="W6" s="3" t="n"/>
       <c r="X6" s="3" t="n"/>
       <c r="Y6" s="3" t="n"/>
@@ -1094,7 +1094,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>ARCH-013</t>
+          <t>ARCH-010</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1109,27 +1109,27 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Cluster Configuration</t>
+          <t>Containerized Execution</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Valid Cluster Configuration for Elastic Compute</t>
+          <t>Valid Containerized Execution Configuration</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Environments using Elastic Compute must have at least one valid cluster configured (found under {DATADIR}/config/clusters or Administration &gt; Clusters); Dataiku does not mandate the specific example configuration, only that a workable cluster exists.</t>
+          <t>Environments using Elastic Compute (Kubernetes) must have at least one valid containerized execution configuration set up (general-settings.json &gt; containerSettings, or Administration &gt; Settings &gt; Containerized execution); as with Spark, the specific example values are only a baseline, not a strict requirement.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Configure at least one valid Kubernetes cluster when using Elastic Compute.</t>
+          <t>Configure at least one valid containerized execution config when using Elastic Compute.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>{DATADIR}/config/clusters</t>
+          <t>general-settings.json &gt; containerSettings</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -1139,34 +1139,38 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>at least one valid cluster configuration present</t>
+          <t>valid containerized execution configuration present</t>
         </is>
       </c>
       <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Required only when the customer uses Elastic Compute/Kubernetes for offloaded workloads.</t>
+        </is>
+      </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>The clusters config/directory contains at least one properly defined cluster, consistent with other evidence of elastic-compute usage (spark/container jobs running on Kubernetes).</t>
+          <t>containerSettings block is present with at least one named config with reasonable memory requests/limits.</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>No cluster configuration is present despite evidence of Kubernetes-based workloads elsewhere in the diagnosis.</t>
+          <t>containerSettings is missing or empty while the instance shows evidence of Kubernetes-based execution elsewhere in the diagnosis.</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not clarify whether Elastic Compute is used at all, flag needs_manual_review.</t>
+          <t>If the diagnosis file does not clarify whether Elastic Compute is used, flag needs_manual_review.</t>
         </is>
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>A valid cluster is required to offload computation to Kubernetes.</t>
+          <t>A valid container exec config is required to run workloads in Kubernetes.</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>Cluster, Managed cluster, Unmanaged cluster, Elastic AI</t>
+          <t>Containerized execution, containerSettings, Elastic Compute</t>
         </is>
       </c>
       <c r="R7" s="3" t="inlineStr">
@@ -1176,12 +1180,12 @@
       </c>
       <c r="S7" s="3" t="inlineStr">
         <is>
-          <t>12, 13</t>
+          <t>8</t>
         </is>
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>Cluster configurations | MUST HAVE if using Elastic Compute; Cluster configurations | MUST HAVE if using Elastic Compute</t>
+          <t>Containerized execution configs | MUST HAVE if using Elastic Compute</t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr">
@@ -1195,6 +1199,111 @@
       <c r="Y7" s="3" t="n"/>
       <c r="Z7" s="3" t="n"/>
       <c r="AA7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-013</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Cluster Configuration</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Valid Cluster Configuration for Elastic Compute</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Environments using Elastic Compute must have at least one valid cluster configured (found under {DATADIR}/config/clusters or Administration &gt; Clusters); Dataiku does not mandate the specific example configuration, only that a workable cluster exists.</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Configure at least one valid Kubernetes cluster when using Elastic Compute.</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>{DATADIR}/config/clusters</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>exists</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>at least one valid cluster configuration present</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="n"/>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>The clusters config/directory contains at least one properly defined cluster, consistent with other evidence of elastic-compute usage (spark/container jobs running on Kubernetes).</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>No cluster configuration is present despite evidence of Kubernetes-based workloads elsewhere in the diagnosis.</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not clarify whether Elastic Compute is used at all, flag needs_manual_review.</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>A valid cluster is required to offload computation to Kubernetes.</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>Cluster, Managed cluster, Unmanaged cluster, Elastic AI</t>
+        </is>
+      </c>
+      <c r="R8" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S8" s="3" t="inlineStr">
+        <is>
+          <t>12, 13</t>
+        </is>
+      </c>
+      <c r="T8" s="3" t="inlineStr">
+        <is>
+          <t>Cluster configurations | MUST HAVE if using Elastic Compute; Cluster configurations | MUST HAVE if using Elastic Compute</t>
+        </is>
+      </c>
+      <c r="U8" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V8" s="3" t="n"/>
+      <c r="W8" s="3" t="n"/>
+      <c r="X8" s="3" t="n"/>
+      <c r="Y8" s="3" t="n"/>
+      <c r="Z8" s="3" t="n"/>
+      <c r="AA8" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1207,7 +1316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA3"/>
+  <dimension ref="A1:AA4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1379,7 +1488,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>SEC-004</t>
+          <t>SEC-002</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -1394,27 +1503,27 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>CGroups</t>
+          <t>User Isolation Framework</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>CGroups Enabled with Memory Limit per Sizing Heuristic</t>
+          <t>User Isolation Framework (UIF) Enabled with Appropriate Impersonation Rules</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Ensure cgroups support is enabled and a memory limit is configured for all memory cgroups, sized according to the recommended heuristic (e.g., 32GB VM -&gt; 10g, 64GB -&gt; 38g, 96GB -&gt; 60g, 128GB+ -&gt; 75% of physical memory), with cgroup placements set for all categories.</t>
+          <t>Ensure the User Isolation Framework (UIF) is installed and enabled, with impersonation active and sensible impersonation rules in place (a one-to-one mapping or regex pattern ensuring all DSS users map to identities other than the dataiku service account). For Kubernetes workloads, one namespace per user is recommended; for Hadoop workloads, Sentry/Ranger should be used to manage access. Also check for any Sanity Check warnings regarding UIF.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Enable cgroups with a memory limit sized per the recommended heuristic for instance RAM.</t>
+          <t>Enable User Isolation Framework with impersonation rules mapping all users away from the service account.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>{DATA_DIR}/config/general-settings.json &gt; cgroupSettings.enabled</t>
+          <t>{DATA_DIR}/config/general-settings.json &gt; impersonation.enabled</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -1428,34 +1537,30 @@
         </is>
       </c>
       <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>Additional checks required: cgroupSettings &gt; cgroups memory limit target should be set and sized per the documented heuristic (approx. 50-75% of physical memory depending on total RAM); no single literal field given for the limit value itself, so compare against the formula in evaluation_guidance.</t>
-        </is>
-      </c>
+      <c r="L2" s="3" t="n"/>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json shows cgroupSettings.enabled: true, targets set for each category under cgroups, and a memory limit configured on memory cgroups (e.g., memory/DSS) that approximates the documented formula based on total instance memory (e.g., ~75% for &gt;120GB, ~66% for 60-120GB, total-20GB for 30-60GB, ~50% below 30GB). Front-end equivalent: Administration &gt; Settings &gt; Resource Control &gt; cgroups shows 'Enable cgroups support' selected with placements and memory limits configured.</t>
+          <t>general-settings.json shows impersonation.enabled: true with userRules configured as a one-to-one mapping or regex rule mapping DSS users to non-service-account identities; no Sanity Check warnings about UIF; for K8s workloads a per-user namespace strategy is evident; for Hadoop workloads Sentry/Ranger integration is present.</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>cgroupSettings.enabled is false/absent, no memory limit is set on memory cgroups, or the configured limit is far below the heuristic (e.g., unlimited or near-total memory), risking instability.</t>
+          <t>impersonation.enabled is false or absent, userRules are missing/overly permissive (e.g., mapping to the dataiku service account), Sanity Check warnings reference UIF, or Kubernetes/Hadoop workloads lack namespace-per-user/Sentry-Ranger controls.</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>If cgroupSettings or category placements are not visible in the diagnosis file, flag as needs_manual_review; also check whether the instance was recently reprovisioned (Cloud Stacks) or upgraded, as cgroup limits/placements may not auto-update and new placements may need to be added post-upgrade.</t>
+          <t>If the diagnosis file lacks general-settings.json impersonation details or workload-specific config, flag as needs_manual_review, noting that longstanding instances without UIF require careful, considerate customer messaging and that disabling/downgrading UIF is not supported.</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>A memory cgroup limit prevents runaway processes from destabilizing or degrading the DSS instance; sizing per the heuristic balances safety with usable memory.</t>
+          <t>UIF and correct impersonation rules are required for proper user isolation and security; without them workloads may run under a shared service account, creating security risk and instability in multi-user environments.</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>cgroups, memory limits, Resource Control</t>
+          <t>User Isolation Framework, impersonation, Kubernetes namespaces, Hadoop Sentry/Ranger</t>
         </is>
       </c>
       <c r="R2" s="3" t="inlineStr">
@@ -1465,12 +1570,12 @@
       </c>
       <c r="S2" s="3" t="inlineStr">
         <is>
-          <t>3, 4, 5</t>
+          <t>2, 3</t>
         </is>
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>CGroups | MUST HAVE; CGroups | MUST HAVE (Review steps); CGroups | MUST HAVE (Notes)</t>
+          <t>User Isolation Framework | MUST HAVE; User Isolation Framework | MUST HAVE (Front End/Back End/Notes)</t>
         </is>
       </c>
       <c r="U2" s="3" t="inlineStr">
@@ -1488,12 +1593,12 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>SEC-006</t>
+          <t>SEC-004</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>nice_to_have</t>
+          <t>must_have</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -1503,68 +1608,68 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>HTTPS Configuration</t>
+          <t>CGroups</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>HTTPS Access Configured for DSS</t>
+          <t>CGroups Enabled with Memory Limit per Sizing Heuristic</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Verify with the customer whether HTTPS access to DSS is configured, either natively via DSS configuration or through a reverse proxy. For custom installations, inspect the [server] section of install.ini; for Cloud Stacks (Fleet Manager) installations, inspect nodes-directory.json in the Instance Diag.</t>
+          <t>Ensure cgroups support is enabled and a memory limit is configured for all memory cgroups, sized according to the recommended heuristic (e.g., 32GB VM -&gt; 10g, 64GB -&gt; 38g, 96GB -&gt; 60g, 128GB+ -&gt; 75% of physical memory), with cgroup placements set for all categories.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Verify HTTPS access to DSS is configured natively or via a reverse proxy.</t>
+          <t>Enable cgroups with a memory limit sized per the recommended heuristic for instance RAM.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>install.ini &gt; [server] section (HTTPS settings) or /data/dataiku/dss_data/run/nodes-directory.json</t>
+          <t>{DATA_DIR}/config/general-settings.json &gt; cgroupSettings.enabled</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>exists</t>
+          <t>equals</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>HTTPS enabled (natively or via reverse proxy)</t>
+          <t>true</t>
         </is>
       </c>
       <c r="K3" s="3" t="n"/>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>No single literal key name given for the HTTPS flag itself; pointer is to the file/section where it should be inspected.</t>
+          <t>Additional checks required: cgroupSettings &gt; cgroups memory limit target should be set and sized per the documented heuristic (approx. 50-75% of physical memory depending on total RAM); no single literal field given for the limit value itself, so compare against the formula in evaluation_guidance.</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>install.ini [server] section shows native HTTPS parameters configured, or nodes-directory.json shows HTTPS URLs/ports for nodes, or customer confirms a reverse proxy terminates HTTPS in front of DSS.</t>
+          <t>general-settings.json shows cgroupSettings.enabled: true, targets set for each category under cgroups, and a memory limit configured on memory cgroups (e.g., memory/DSS) that approximates the documented formula based on total instance memory (e.g., ~75% for &gt;120GB, ~66% for 60-120GB, total-20GB for 30-60GB, ~50% below 30GB). Front-end equivalent: Administration &gt; Settings &gt; Resource Control &gt; cgroups shows 'Enable cgroups support' selected with placements and memory limits configured.</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>Only HTTP is configured with no reverse proxy in front, and install.ini/nodes-directory.json show no HTTPS-related configuration.</t>
+          <t>cgroupSettings.enabled is false/absent, no memory limit is set on memory cgroups, or the configured limit is far below the heuristic (e.g., unlimited or near-total memory), risking instability.</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not include install.ini or nodes-directory.json content, or if reverse-proxy setup is external to DSS, flag as needs_manual_review and confirm directly with the customer.</t>
+          <t>If cgroupSettings or category placements are not visible in the diagnosis file, flag as needs_manual_review; also check whether the instance was recently reprovisioned (Cloud Stacks) or upgraded, as cgroup limits/placements may not auto-update and new placements may need to be added post-upgrade.</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>HTTPS protects data in transit and is recommended practice for securing access to DSS.</t>
+          <t>A memory cgroup limit prevents runaway processes from destabilizing or degrading the DSS instance; sizing per the heuristic balances safety with usable memory.</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>HTTPS, reverse proxy, install.ini, nodes-directory.json</t>
+          <t>cgroups, memory limits, Resource Control</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
@@ -1574,17 +1679,17 @@
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
-          <t>5, 6</t>
+          <t>3, 4, 5</t>
         </is>
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>HTTPS | NICE TO HAVE; HTTPS | NICE TO HAVE (Review steps)</t>
+          <t>CGroups | MUST HAVE; CGroups | MUST HAVE (Review steps); CGroups | MUST HAVE (Notes)</t>
         </is>
       </c>
       <c r="U3" s="3" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="V3" s="3" t="n"/>
@@ -1593,6 +1698,115 @@
       <c r="Y3" s="3" t="n"/>
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>SEC-006</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>nice_to_have</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>HTTPS Configuration</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>HTTPS Access Configured for DSS</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Verify with the customer whether HTTPS access to DSS is configured, either natively via DSS configuration or through a reverse proxy. For custom installations, inspect the [server] section of install.ini; for Cloud Stacks (Fleet Manager) installations, inspect nodes-directory.json in the Instance Diag.</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Verify HTTPS access to DSS is configured natively or via a reverse proxy.</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>install.ini &gt; [server] section (HTTPS settings) or /data/dataiku/dss_data/run/nodes-directory.json</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>exists</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>HTTPS enabled (natively or via reverse proxy)</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>No single literal key name given for the HTTPS flag itself; pointer is to the file/section where it should be inspected.</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>install.ini [server] section shows native HTTPS parameters configured, or nodes-directory.json shows HTTPS URLs/ports for nodes, or customer confirms a reverse proxy terminates HTTPS in front of DSS.</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Only HTTP is configured with no reverse proxy in front, and install.ini/nodes-directory.json show no HTTPS-related configuration.</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not include install.ini or nodes-directory.json content, or if reverse-proxy setup is external to DSS, flag as needs_manual_review and confirm directly with the customer.</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>HTTPS protects data in transit and is recommended practice for securing access to DSS.</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>HTTPS, reverse proxy, install.ini, nodes-directory.json</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>security_permissions_compliance</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>5, 6</t>
+        </is>
+      </c>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>HTTPS | NICE TO HAVE; HTTPS | NICE TO HAVE (Review steps)</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V4" s="3" t="n"/>
+      <c r="W4" s="3" t="n"/>
+      <c r="X4" s="3" t="n"/>
+      <c r="Y4" s="3" t="n"/>
+      <c r="Z4" s="3" t="n"/>
+      <c r="AA4" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1605,7 +1819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA3"/>
+  <dimension ref="A1:AA4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1886,67 +2100,75 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>GENAI-009</t>
+          <t>GENAI-007</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>nice_to_have</t>
+          <t>must_have</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>qualitative_practice</t>
+          <t>specific_setting</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Agent Hub</t>
+          <t>Cobuild</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Agent Hub Deployment Required Permissions</t>
+          <t>Cobuild Default LLM Configuration</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Before a user can deploy an Agent Hub instance, they must have permissions for writing project content in the hosting project, writing isolated code execution, WebApp impersonation, and (if Quick agents are enabled) create projects; alternatively the user could be a DSS administrator, though a dedicated service account is preferred.</t>
+          <t>Administrators must configure default LLM settings for Cobuild (agent-building tools) upon activation of AI Assistants, including defaultEmbeddingLLMId, defaultLLMId, and defaultImageGenerationLLMId under agentBuildingSettings; if unset, Cobuild's building-agent tools will fail and instruct users to contact an administrator.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Grant Agent Hub deployers write project content, isolated code execution, and webapp impersonation permissions.</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
+          <t>Configure default embedding, LLM, and image-generation models for Cobuild agent building.</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; aiDrivenAnalyticsSettings.agentBuildingSettings.{defaultEmbeddingLLMId, defaultLLMId, defaultImageGenerationLLMId}</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>exists</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>all three fields populated with valid LLM IDs</t>
+        </is>
+      </c>
       <c r="K3" s="3" t="n"/>
       <c r="L3" s="3" t="n"/>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Administration &gt; Security &gt; Groups shows the Agent Hub deployer's group granted 'Write project content', 'Write isolated code execution', and 'WebApp impersonation' permissions (plus 'Create projects' if Quick agents are enabled), or the deployer is a DSS admin/service account.</t>
+          <t>agentBuildingSettings block shows non-empty defaultEmbeddingLLMId, defaultLLMId, and defaultImageGenerationLLMId values.</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>The deployer's group lacks one or more of these permissions and is not an admin/service account, or logs show 'Not authorized' errors when creating the Agent Hub WebApp.</t>
+          <t>One or more of these fields is missing or empty while Cobuild/AI Assistants is enabled.</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file lacks per-user/group permission detail, flag needs_manual_review and recommend checking Administration &gt; Security &gt; Groups directly.</t>
-        </is>
-      </c>
-      <c r="P3" s="3" t="inlineStr">
-        <is>
-          <t>Missing permissions cause deployment failures such as 'Not authorized' errors when creating the Agent Hub WebApp.</t>
-        </is>
-      </c>
+          <t>If aiDrivenAnalyticsSettings is absent from the diagnosis, flag needs_manual_review to confirm whether Cobuild/AI Assistants is enabled for this customer.</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="n"/>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>Agent Hub, Permissions, Groups, WebApp</t>
+          <t>Cobuild, AI Assistants, Agent building</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
@@ -1956,29 +2178,122 @@
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
-          <t>10, 11, 12</t>
+          <t>7, 8, 9</t>
         </is>
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>Agent Hub NICE TO HAVE:; Writing isolated code execution; WebApp impersonation</t>
+          <t>Cobuild; Cobuild; Instance Diags / DiagParser3</t>
         </is>
       </c>
       <c r="U3" s="3" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="V3" s="3" t="inlineStr">
-        <is>
-          <t>Although the parent topic is tagged NICE TO HAVE, the described permission requirements are phrased as mandatory ('must have permissions') for successful deployment; classification follows the explicit heading tag.</t>
-        </is>
-      </c>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V3" s="3" t="n"/>
       <c r="W3" s="3" t="n"/>
       <c r="X3" s="3" t="n"/>
       <c r="Y3" s="3" t="n"/>
       <c r="Z3" s="3" t="n"/>
       <c r="AA3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>GENAI-009</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>nice_to_have</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>qualitative_practice</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub Deployment Required Permissions</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Before a user can deploy an Agent Hub instance, they must have permissions for writing project content in the hosting project, writing isolated code execution, WebApp impersonation, and (if Quick agents are enabled) create projects; alternatively the user could be a DSS administrator, though a dedicated service account is preferred.</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Grant Agent Hub deployers write project content, isolated code execution, and webapp impersonation permissions.</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Administration &gt; Security &gt; Groups shows the Agent Hub deployer's group granted 'Write project content', 'Write isolated code execution', and 'WebApp impersonation' permissions (plus 'Create projects' if Quick agents are enabled), or the deployer is a DSS admin/service account.</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>The deployer's group lacks one or more of these permissions and is not an admin/service account, or logs show 'Not authorized' errors when creating the Agent Hub WebApp.</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file lacks per-user/group permission detail, flag needs_manual_review and recommend checking Administration &gt; Security &gt; Groups directly.</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>Missing permissions cause deployment failures such as 'Not authorized' errors when creating the Agent Hub WebApp.</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub, Permissions, Groups, WebApp</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>generative_ai_acceleration</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>10, 11, 12</t>
+        </is>
+      </c>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub NICE TO HAVE:; Writing isolated code execution; WebApp impersonation</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V4" s="3" t="inlineStr">
+        <is>
+          <t>Although the parent topic is tagged NICE TO HAVE, the described permission requirements are phrased as mandatory ('must have permissions') for successful deployment; classification follows the explicit heading tag.</t>
+        </is>
+      </c>
+      <c r="W4" s="3" t="n"/>
+      <c r="X4" s="3" t="n"/>
+      <c r="Y4" s="3" t="n"/>
+      <c r="Z4" s="3" t="n"/>
+      <c r="AA4" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1986,6 +2301,1034 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AA9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="40" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="40" customWidth="1" min="24" max="24"/>
+    <col width="40" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>check_type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>subtopic</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>statement</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>statement_short</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>parameter_hint</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>operator</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>expected_value</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>expected_condition_notes</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>supporting_evidence</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>contradicting_evidence</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>insufficient_evidence_handling</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>rationale</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>dataiku_concepts</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>source_document</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>source_page</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>source_section</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>ambiguity_notes</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>validation_status</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>evidence_found</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>validated_at</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>validated_by</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>SCALE-001</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Runtime Database</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>External PostgreSQL Runtime Database</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>The default H2 runtime database is not production-ready and should be replaced with an external PostgreSQL database (or DCS-managed internal PostgreSQL) for scalability and resilience. When PostgreSQL is used, connection pooling and backup practices must also be verified.</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Replace the default H2 runtime database with external PostgreSQL for production readiness.</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; internalDatabase.type</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>equals</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>PostgreSQL</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Also verify maxPooledExternalConnections (general-settings.json) is at least 2x the postgresql.conf max_connections value (Cloud Stacks default max_connections=500), and that a backup process synced with DSS backups exists.</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json shows internalDatabase.type = PostgreSQL (external or DCS-managed); maxPooledExternalConnections &gt;= 2x postgres max_connections; documented backup process aligned with DSS backups.</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>internalDatabase field absent or shows internal H2 in use without an external Postgres configured; maxPooledExternalConnections too low relative to max_connections; no DB backup process.</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>If general-settings.json is unavailable or DB type cannot be determined, flag needs_manual_review and request the customer's postgresql.conf max_connections value and backup policy.</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>H2 does not scale well and complicates backup/resilience; PostgreSQL is required for production readiness.</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>runtime database, PostgreSQL, H2, backup</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>scalable_performance_ops</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
+      <c r="T2" s="3" t="inlineStr">
+        <is>
+          <t>Postgres runtime database | MUST HAVE; Postgres runtime database | MUST HAVE</t>
+        </is>
+      </c>
+      <c r="U2" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V2" s="3" t="n"/>
+      <c r="W2" s="3" t="n"/>
+      <c r="X2" s="3" t="n"/>
+      <c r="Y2" s="3" t="n"/>
+      <c r="Z2" s="3" t="n"/>
+      <c r="AA2" s="3" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>SCALE-002</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>nice_to_have</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Metastore Configuration</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Appropriate Metastore Configured</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>An appropriate metastore should be configured based on environment: Hive for standard Hadoop clusters, Glue when properly integrated on AWS, or the DSS internal metastore otherwise. Confirm the configured flavor matches the environment and that managed datasets sync correctly.</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Configure the metastore flavor (Hive, Glue, or internal) appropriate to the environment.</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; metastoreCatalogsSettings.flavor</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>one_of</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Hive (Hadoop cluster) | Glue (AWS with proper integration) | DSS internal (otherwise)</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Correct value is context-dependent on infrastructure; also verify via Administration &gt; Settings &gt; Metastore catalogs UI.</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>flavor value matches environment type (Hive for Hadoop, Glue for properly-integrated AWS, else DSS internal); a test dataset sync confirms managed datasets sync to the metastore.</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>flavor mismatched with environment (e.g., Glue configured without proper AWS integration, or DSS internal used when Hive/Glue would be appropriate); sync test fails.</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>If environment type or metastoreCatalogsSettings is not present in the diagnosis, flag needs_manual_review and confirm with the customer during interview.</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>Correct metastore selection ensures managed dataset metadata is properly synced and available for query engines.</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>metastore, Hive, Glue, managed datasets</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>scalable_performance_ops</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>2, 3</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>Metastore is configured | NICE TO HAVE; Metastore is configured | NICE TO HAVE</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>Expected flavor value is not a fixed constant but depends on customer's infrastructure, so the check requires contextual knowledge of the environment.</t>
+        </is>
+      </c>
+      <c r="W3" s="3" t="n"/>
+      <c r="X3" s="3" t="n"/>
+      <c r="Y3" s="3" t="n"/>
+      <c r="Z3" s="3" t="n"/>
+      <c r="AA3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>SCALE-003</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>nice_to_have</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Graphics Export</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Graphics Export (PDF/Image) Configuration</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Check whether PDF/image export from the Flow is configured; if not configured, discuss with the client whether this feature should be enabled.</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Check whether Flow PDF/image export is configured and discuss enabling it if not.</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; graphicsExportsEnabled</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>equals</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Desired state is contextual on client needs; can also confirm via the Flow Actions &gt; Export to PDF/Image UI option.</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>graphicsExportsEnabled=true in general-settings.json, or the Export to PDF/Image option is visible in the Flow Actions menu.</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>graphicsExportsEnabled=false with no documented discussion or decision with the client about whether the feature is desired.</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>If the field is absent from the diagnosis, flag needs_manual_review and verify via the UI or ask the customer.</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>Feature must be explicitly configured; disabling it may be acceptable if the client doesn't need it, hence nice to have.</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>graphics export, Flow</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>scalable_performance_ops</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>Graphics export configured | NICE TO HAVE</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V4" s="3" t="n"/>
+      <c r="W4" s="3" t="n"/>
+      <c r="X4" s="3" t="n"/>
+      <c r="Y4" s="3" t="n"/>
+      <c r="Z4" s="3" t="n"/>
+      <c r="AA4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>SCALE-004</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>qualitative_practice</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Maintenance &amp; Cleanup</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Admin Project for Garbage Collection</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>An admin project should be set up to automatically clean up accumulated logs and idle Jupyter kernels on a schedule, per the Setup Maintenance Jobs wiki.</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Set up a scheduled admin project to clean up logs and idle Jupyter kernels.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n"/>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Presence of a dedicated admin/maintenance project with scenarios scheduled to clean logs and idle kernels; scenario run history shows regular execution.</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>No maintenance project exists, or disk usage/log data shows unbounded growth of logs or idle Jupyter kernels.</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis doesn't include a project list or scenario details, flag needs_manual_review and ask the customer to confirm existence of a scheduled cleanup project.</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>Without cleanup, logs and idle kernels accumulate over time causing resource exhaustion.</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>admin project, garbage collection, scenarios, disk usage</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>scalable_performance_ops</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>3, 4</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="inlineStr">
+        <is>
+          <t>Admin project - garbage collection | MUST HAVE; Admin project - garbage collection | MUST HAVE</t>
+        </is>
+      </c>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V5" s="3" t="n"/>
+      <c r="W5" s="3" t="n"/>
+      <c r="X5" s="3" t="n"/>
+      <c r="Y5" s="3" t="n"/>
+      <c r="Z5" s="3" t="n"/>
+      <c r="AA5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>SCALE-007</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>qualitative_practice</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Log Monitoring</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Backend.log Error Review</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Review recent backend.log files (including rotated/zipped logs) for ERROR or FATAL level entries indicating systemic issues such as repeating stack traces, connection failures, or plugin crashes; investigate patterns that recur frequently even without explicit user complaints.</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Review backend.log for recurring ERROR/FATAL entries indicating systemic stability issues.</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="n"/>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>backend.log and rotated logs show few or no ERROR/FATAL entries, or only isolated non-recurring errors; AI Log Analysis in DiagParser3 shows no systemic issue flagged.</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>Frequent recurring ERROR/FATAL entries (e.g., the same stack trace dozens of times per day), repeated connection failures, or plugin crashes.</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>If logs aren't included or available in the diagnosis bundle, flag needs_manual_review and request the backend.log files directly.</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>A high volume of repeated errors often points to a systemic issue that needs to be addressed before it impacts instance stability.</t>
+        </is>
+      </c>
+      <c r="Q6" s="3" t="inlineStr">
+        <is>
+          <t>backend.log, AI Log Analysis, DiagParser3</t>
+        </is>
+      </c>
+      <c r="R6" s="3" t="inlineStr">
+        <is>
+          <t>scalable_performance_ops</t>
+        </is>
+      </c>
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>6, 7</t>
+        </is>
+      </c>
+      <c r="T6" s="3" t="inlineStr">
+        <is>
+          <t>Backend.log Errors | MUST HAVE; Backend.log Errors | MUST HAVE</t>
+        </is>
+      </c>
+      <c r="U6" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V6" s="3" t="n"/>
+      <c r="W6" s="3" t="n"/>
+      <c r="X6" s="3" t="n"/>
+      <c r="Y6" s="3" t="n"/>
+      <c r="Z6" s="3" t="n"/>
+      <c r="AA6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>SCALE-008</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Memory Sizing</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Backend Xmx Sizing</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>backend.xmx must be appropriately sized for the deployment based on system memory (Cloud Stacks heuristic: 4g for &gt;12GB RAM, 8g for &gt;30GB RAM, 16g for &gt;95GB RAM, more for larger deployments), and should be at least 3x the size of the configuration folder. jek.xmx and fek.xmx should also be checked to ensure they haven't been oversized, and backend.log should be checked for OutOfMemoryError entries.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Size backend.xmx per the memory heuristic, at least 3x the config folder size.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>install.ini &gt; backend.xmx</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>greater_than_or_equal</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>per Cloud Stacks heuristic tier (4g/8g/16g based on system RAM) and &gt;=3x config folder size</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Also verify jek.xmx/fek.xmx are not oversized, and that xmx avoids the 32GB&lt;=xmx&lt;48GB dead zone (jump to 48GB instead) due to Java Ordinary Object Pointer behavior.</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>install.ini backend.xmx matches or exceeds the recommended tier for system memory, is &gt;=3x config folder size, and avoids the 32-48GB dead zone; no OutOfMemoryError entries in backend.log.</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>backend.xmx set below the recommended heuristic, falls in the 32GB-48GB dead zone, or backend.log shows recurring 'OutOfMemoryError: Java heap space' / 'OutOfMemoryError: GC Overhead limit exceeded' entries.</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>If install.ini or system memory info is not present in the diagnosis, flag needs_manual_review and request system specs and install.ini contents.</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>Insufficient or misconfigured heap sizing leads to OutOfMemory errors and instability; oversizing into the 32-48GB range paradoxically reduces available memory due to JVM pointer compression behavior.</t>
+        </is>
+      </c>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>backend.xmx, jek.xmx, fek.xmx, JVM memory, OutOfMemoryError</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>scalable_performance_ops</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>7, 8</t>
+        </is>
+      </c>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>Backend Xmx | MUST HAVE; Backend Xmx | MUST HAVE</t>
+        </is>
+      </c>
+      <c r="U7" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V7" s="3" t="n"/>
+      <c r="W7" s="3" t="n"/>
+      <c r="X7" s="3" t="n"/>
+      <c r="Y7" s="3" t="n"/>
+      <c r="Z7" s="3" t="n"/>
+      <c r="AA7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>SCALE-009</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Flow Parallelism Limits</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Flow Limits Sizing (Max Jobs, Max Activities)</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Configure Flow concurrency limits using the 5-step sizing framework: reserve OS/backend.xmx memory, allocate roughly 70% of remaining memory to CGroups (less if offloading heavy workloads to EKS/Kubernetes), size Max Jobs from the remaining JEK memory, set the global Max Activities limit (30-50) as a backstop above Max Jobs, and leave Max Activities per Job at the default of 5. Max Jobs must never be set to 0, as this disables the limit entirely and risks crashing the instance via OOM.</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Size Max Jobs and Max Activities via the memory framework; never set Max Jobs to zero.</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; maxRunningJobs</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>not_equals</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>Also verify general-settings.json &gt; maxRunningActivities falls within 30-50, and maxRunningActivitiesPerJob is at the default of 5 unless justified. Front-end equivalent: Administration &gt; Settings &gt; Resources control &gt; Concurrent Activities.</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>maxRunningJobs set to a positive nonzero value derived from the 5-step memory sizing framework; maxRunningActivities within 30-50; maxRunningActivitiesPerJob at 5 (or a justified alternative).</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>maxRunningJobs is 0 or blank (critical stability risk); maxRunningActivities is outside 30-50 without justification; sizing doesn't account for available host memory, risking OOM.</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>If these general-settings.json values are missing from the diagnosis, flag needs_manual_review and check the Administration &gt; Settings &gt; Resources control UI directly.</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>Improperly sized flow limits risk instance-wide Out-Of-Memory crashes; Max Jobs=0 disables protection entirely.</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>Flow limits, Max Jobs, Max Activities, CGroups, JEK, memory sizing</t>
+        </is>
+      </c>
+      <c r="R8" s="3" t="inlineStr">
+        <is>
+          <t>scalable_performance_ops</t>
+        </is>
+      </c>
+      <c r="S8" s="3" t="inlineStr">
+        <is>
+          <t>8, 9, 10, 11</t>
+        </is>
+      </c>
+      <c r="T8" s="3" t="inlineStr">
+        <is>
+          <t>Flow parallelism | MUST HAVE; Flow parallelism | MUST HAVE; Flow parallelism | MUST HAVE; Flow parallelism | MUST HAVE</t>
+        </is>
+      </c>
+      <c r="U8" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V8" s="3" t="n"/>
+      <c r="W8" s="3" t="n"/>
+      <c r="X8" s="3" t="n"/>
+      <c r="Y8" s="3" t="n"/>
+      <c r="Z8" s="3" t="n"/>
+      <c r="AA8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>SCALE-011</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Connections Hygiene</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Remove filesystem_root Connection</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>The default filesystem_root connection pointing to the server's root filesystem should be removed unless actively used by a project; if in use, propose a dedicated scoped connection to the specific path before removing filesystem_root.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Remove the filesystem_root connection unless actively used, replacing it with a scoped connection.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>connections.json &gt; filesystem_root</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>not_exists</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>removed (unless replaced by a scoped connection after confirming no active project usage)</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="n"/>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>Check usage via Administration -&gt; Monitoring before deletion.</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>filesystem_root connection absent from the connections list, or confirmed unused and removed; if it was in use, a dedicated scoped connection was created to replace it.</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>filesystem_root connection still present and either unused (should have been deleted) or in use without a safer scoped replacement.</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>If the connections list isn't in the diagnosis, flag needs_manual_review and check the Administration &gt; Connections UI directly.</t>
+        </is>
+      </c>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>The filesystem_root connection exposes the entire server filesystem, posing a security and stability risk.</t>
+        </is>
+      </c>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>connections, filesystem_root, security</t>
+        </is>
+      </c>
+      <c r="R9" s="3" t="inlineStr">
+        <is>
+          <t>scalable_performance_ops</t>
+        </is>
+      </c>
+      <c r="S9" s="3" t="inlineStr">
+        <is>
+          <t>14, 15</t>
+        </is>
+      </c>
+      <c r="T9" s="3" t="inlineStr">
+        <is>
+          <t>Remove filesystem_root connection | MUST HAVE; Remove filesystem_root connection | MUST HAVE</t>
+        </is>
+      </c>
+      <c r="U9" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V9" s="3" t="n"/>
+      <c r="W9" s="3" t="n"/>
+      <c r="X9" s="3" t="n"/>
+      <c r="Y9" s="3" t="n"/>
+      <c r="Z9" s="3" t="n"/>
+      <c r="AA9" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2163,7 +3506,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>SCALE-007</t>
+          <t>ADVSEC-003</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -2173,80 +3516,100 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>qualitative_practice</t>
+          <t>specific_setting</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Log Monitoring</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Backend.log Error Review</t>
+          <t>Expiring sessions</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Review recent backend.log files (including rotated/zipped logs) for ERROR or FATAL level entries indicating systemic issues such as repeating stack traces, connection failures, or plugin crashes; investigate patterns that recur frequently even without explicit user complaints.</t>
+          <t>DSS can be configured to expire user sessions after a maximum duration since login and/or after a period of inactivity, via Administration &gt; Settings &gt; Security &amp; Audit &gt; User login &amp; provisioning &gt; Session management ('Maximum session duration' and 'Idle timeout'), noting this can cause lost work if a session expires mid-edit.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Review backend.log for recurring ERROR/FATAL entries indicating systemic stability issues.</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
+          <t>Configure maximum session duration and idle timeout to automatically expire user sessions.</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; security.sessionsMaxTotalTimeMinutes / security.sessionsMaxIdleTimeMinutes (UI: Administration &gt; Settings &gt; Security &amp; Audit &gt; User login &amp; provisioning &gt; Session management)</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>exists</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>either value set to a finite number of minutes greater than 0</t>
+        </is>
+      </c>
       <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>In general-settings.json a value of 0 means unlimited (the default). The source does not mandate a specific threshold; treat as satisfied if either or both values are greater than 0.</t>
+        </is>
+      </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>backend.log and rotated logs show few or no ERROR/FATAL entries, or only isolated non-recurring errors; AI Log Analysis in DiagParser3 shows no systemic issue flagged.</t>
+          <t>general-settings.json security.sessionsMaxTotalTimeMinutes and/or security.sessionsMaxIdleTimeMinutes is greater than 0.</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>Frequent recurring ERROR/FATAL entries (e.g., the same stack trace dozens of times per day), repeated connection failures, or plugin crashes.</t>
+          <t>Both keys are 0 (unlimited) or absent.</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>If logs aren't included or available in the diagnosis bundle, flag needs_manual_review and request the backend.log files directly.</t>
+          <t>Flag needs_manual_review only if general-settings.json or its security block is not in the diagnosis; otherwise decide from the two keys. Note the source's caveat that expiring sessions can lose in-progress work.</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>A high volume of repeated errors often points to a systemic issue that needs to be addressed before it impacts instance stability.</t>
+          <t>Session expiration limits how long a stolen or abandoned session remains valid, though the source warns it can cause lost in-progress work (including complications with open Jupyter notebooks).</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>backend.log, AI Log Analysis, DiagParser3</t>
+          <t>session management, user login &amp; provisioning</t>
         </is>
       </c>
       <c r="R2" s="3" t="inlineStr">
         <is>
-          <t>scalable_performance_ops</t>
+          <t>advanced_security_options</t>
         </is>
       </c>
       <c r="S2" s="3" t="inlineStr">
         <is>
-          <t>6, 7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>Backend.log Errors | MUST HAVE; Backend.log Errors | MUST HAVE</t>
+          <t>Expiring sessions</t>
         </is>
       </c>
       <c r="U2" s="3" t="inlineStr">
         <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="V2" s="3" t="n"/>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V2" s="3" t="inlineStr">
+        <is>
+          <t>The source gives only the UI path and no numeric threshold; the file keys were verified against sample bundles, not the source documents.</t>
+        </is>
+      </c>
       <c r="W2" s="3" t="n"/>
       <c r="X2" s="3" t="n"/>
       <c r="Y2" s="3" t="n"/>
@@ -2256,12 +3619,12 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>SCALE-008</t>
+          <t>ADVSEC-006</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -2271,87 +3634,83 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Memory Sizing</t>
+          <t>Session &amp; Logout UX</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Backend Xmx Sizing</t>
+          <t>Redirecting to a custom URL after logout</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>backend.xmx must be appropriately sized for the deployment based on system memory (Cloud Stacks heuristic: 4g for &gt;12GB RAM, 8g for &gt;30GB RAM, 16g for &gt;95GB RAM, more for larger deployments), and should be at least 3x the size of the configuration folder. jek.xmx and fek.xmx should also be checked to ensure they haven't been oversized, and backend.log should be checked for OutOfMemoryError entries.</t>
+          <t>By default, users are redirected to a standard DSS-hosted page after logout; administrators can configure security.postLogoutBehavior (CUSTOM_URL for a GET redirect or CUSTOM_URL_POST for a POST request aligned with OpenID Connect RP-Initiated Logout) together with security.postLogoutCustomURL (must be an http/https URL) in general-settings.json to redirect users elsewhere, with DSS validating these settings on save/load and falling back to the default page on invalid values.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Size backend.xmx per the memory heuristic, at least 3x the config folder size.</t>
+          <t>Configure postLogoutBehavior and postLogoutCustomURL to redirect users after logout.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>install.ini &gt; backend.xmx</t>
+          <t>general-settings.json &gt; security.postLogoutBehavior / security.postLogoutCustomURL</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>greater_than_or_equal</t>
+          <t>one_of</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>per Cloud Stacks heuristic tier (4g/8g/16g based on system RAM) and &gt;=3x config folder size</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
+          <t>CUSTOM_URL, CUSTOM_URL_POST</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="n"/>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>Also verify jek.xmx/fek.xmx are not oversized, and that xmx avoids the 32GB&lt;=xmx&lt;48GB dead zone (jump to 48GB instead) due to Java Ordinary Object Pointer behavior.</t>
+          <t>postLogoutCustomURL is required and must be an http/https URL when postLogoutBehavior is CUSTOM_URL or CUSTOM_URL_POST; DSS validates these settings on save and on load, falling back to the default DSS logged-out page if invalid.</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>install.ini backend.xmx matches or exceeds the recommended tier for system memory, is &gt;=3x config folder size, and avoids the 32-48GB dead zone; no OutOfMemoryError entries in backend.log.</t>
+          <t>general-settings.json "security" object contains postLogoutBehavior set to CUSTOM_URL or CUSTOM_URL_POST along with a valid http/https postLogoutCustomURL.</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>backend.xmx set below the recommended heuristic, falls in the 32GB-48GB dead zone, or backend.log shows recurring 'OutOfMemoryError: Java heap space' / 'OutOfMemoryError: GC Overhead limit exceeded' entries.</t>
+          <t>The keys are absent (default DSS logged-out page used) or postLogoutCustomURL is invalid, in which case DSS falls back to default behavior anyway.</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>If install.ini or system memory info is not present in the diagnosis, flag needs_manual_review and request system specs and install.ini contents.</t>
+          <t>If general-settings.json content is not present in the diagnosis, flag as needs_manual_review; absence means the default logout page is used, which is not a security concern.</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>Insufficient or misconfigured heap sizing leads to OutOfMemory errors and instability; oversizing into the 32-48GB range paradoxically reduces available memory due to JVM pointer compression behavior.</t>
+          <t>Allows organizations to redirect users to a branded or external page after logout instead of the DSS default logged-out page.</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>backend.xmx, jek.xmx, fek.xmx, JVM memory, OutOfMemoryError</t>
+          <t>general-settings.json, security settings, logout, OpenID Connect</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
         <is>
-          <t>scalable_performance_ops</t>
+          <t>advanced_security_options</t>
         </is>
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
-          <t>7, 8</t>
+          <t>4, 5</t>
         </is>
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>Backend Xmx | MUST HAVE; Backend Xmx | MUST HAVE</t>
+          <t>Redirecting to a custom URL after logout; Redirecting to a custom URL after logout</t>
         </is>
       </c>
       <c r="U3" s="3" t="inlineStr">
@@ -2369,7 +3728,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>SCALE-009</t>
+          <t>ADVSEC-008</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -2384,83 +3743,83 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Flow Parallelism Limits</t>
+          <t>Data Exfiltration Controls</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Flow Limits Sizing (Max Jobs, Max Activities)</t>
+          <t>Restricting exports</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Configure Flow concurrency limits using the 5-step sizing framework: reserve OS/backend.xmx memory, allocate roughly 70% of remaining memory to CGroups (less if offloading heavy workloads to EKS/Kubernetes), size Max Jobs from the remaining JEK memory, set the global Max Activities limit (30-50) as a backstop above Max Jobs, and leave Max Activities per Job at the default of 5. Max Jobs must never be set to 0, as this disables the limit entirely and risks crashing the instance via OOM.</t>
+          <t>DSS can globally restrict export/copy features (regardless of project-level permissions) via a set of escalating dip.properties keys: disableAllDatasetExports, disableAllDataExports (implies the former), disableAllExports (implies both former), plus the independent disableCopySampleToClipboard and disableSQLNotebookCopyResultToClipboard keys for clipboard copying; the source explicitly warns this is only a 'best-effort' restriction since any user who can see data can still exfiltrate it, e.g. via copy/paste.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Size Max Jobs and Max Activities via the memory framework; never set Max Jobs to zero.</t>
+          <t>Disable export and clipboard-copy keys in dip.properties to limit data exfiltration risk.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; maxRunningJobs</t>
+          <t>dip.properties &gt; dku.exports.disable*</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>not_equals</t>
+          <t>one_of</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>dku.exports.disableAllDatasetExports=true; dku.exports.disableAllDataExports=true; dku.exports.disableAllExports=true; dku.exports.disableCopySampleToClipboard=true; dku.exports.disableSQLNotebookCopyResultToClipboard=true</t>
         </is>
       </c>
       <c r="K4" s="3" t="n"/>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>Also verify general-settings.json &gt; maxRunningActivities falls within 30-50, and maxRunningActivitiesPerJob is at the default of 5 unless justified. Front-end equivalent: Administration &gt; Settings &gt; Resources control &gt; Concurrent Activities.</t>
+          <t>dku.exports.disableAllDatasetExports=true disables 'Download' export of datasets to files (CSV, Excel, Tableau Hyper, etc.), plus including datasets in project exports/bundle downloads and attaching datasets to emails in scenarios; other exports (ML data, schema, SQL queries, prepared data) remain possible. dku.exports.disableAllDataExports=true implies the previous key and additionally disables exports of prepared data or SQL query results, downloading files/zips from managed folders, and including datasets or managed folders in project exports/bundle downloads or scenario email attachments; ML data and schema exports remain possible. dku.exports.disableAllExports=true implies both previous keys and additionally disables exports of ML data and schemas, so essentially all dataset, prepared-data, SQL-query, ML data/schema, and managed-folder exports, downloads, bundle inclusions, and email attachments are disabled. dku.exports.disableCopySampleToClipboard=true disables copying data samples to the clipboard everywhere except SQL notebooks (default false, i.e. enabled). dku.exports.disableSQLNotebookCopyResultToClipboard=true disables copying results to the clipboard specifically in SQL notebooks (default false, i.e. enabled).</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>maxRunningJobs set to a positive nonzero value derived from the 5-step memory sizing framework; maxRunningActivities within 30-50; maxRunningActivitiesPerJob at 5 (or a justified alternative).</t>
+          <t>dip.properties contains one or more of the five dku.exports.disable* keys set to true, at a scope level (dataset/data/all) matching the organization's data-exfiltration risk tolerance.</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>maxRunningJobs is 0 or blank (critical stability risk); maxRunningActivities is outside 30-50 without justification; sizing doesn't account for available host memory, risking OOM.</t>
+          <t>None of the dku.exports.disable* keys are present or set to true, meaning full export and clipboard-copy capabilities remain available to any user with data-view permission.</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>If these general-settings.json values are missing from the diagnosis, flag needs_manual_review and check the Administration &gt; Settings &gt; Resources control UI directly.</t>
+          <t>dip.properties content is often not fully captured in diagnostics; if absent, flag as needs_manual_review. Importantly, even when these settings are enabled, treat this only as a risk-reduction control, not a guarantee: the source explicitly states export restriction is inherently 'best-effort' since a user who can view data can still exfiltrate it by other means (e.g., copy/paste).</t>
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>Improperly sized flow limits risk instance-wide Out-Of-Memory crashes; Max Jobs=0 disables protection entirely.</t>
+          <t>Restricting export and clipboard-copy features reduces (but per the source's own warning, does not eliminate) the ability of authorized viewers to exfiltrate data out of DSS.</t>
         </is>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Flow limits, Max Jobs, Max Activities, CGroups, JEK, memory sizing</t>
+          <t>dip.properties, exports, data exfiltration</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>scalable_performance_ops</t>
+          <t>advanced_security_options</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>8, 9, 10, 11</t>
+          <t>6, 7, 8</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>Flow parallelism | MUST HAVE; Flow parallelism | MUST HAVE; Flow parallelism | MUST HAVE; Flow parallelism | MUST HAVE</t>
+          <t>Restricting exports; Restricting exports; Restricting exports</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
@@ -2478,7 +3837,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>SCALE-011</t>
+          <t>ADVSEC-009</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -2493,83 +3852,83 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Connections Hygiene</t>
+          <t>Transport &amp; Browser Hardening</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Remove filesystem_root Connection</t>
+          <t>Setting security-related HTTP headers</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>The default filesystem_root connection pointing to the server's root filesystem should be removed unless actively used by a project; if in use, propose a dedicated scoped connection to the specific path before removing filesystem_root.</t>
+          <t>DSS supports configuring standard security-related HTTP response headers (X-Frame-Options, Content-Security-Policy, X-XSS-Protection, X-Content-Type-Options, Strict-Transport-Security, Referrer-Policy, Permissions-Policy, Cross-Origin-Embedder-Policy, Cross-Origin-Opener-Policy, Cross-Origin-Resource-Policy) in the [server] section of install.ini, requiring a `dssadmin regenerate-config` run and a DSS restart to take effect.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Remove the filesystem_root connection unless actively used, replacing it with a scoped connection.</t>
+          <t>Configure restrictive security HTTP headers like CSP, X-Frame-Options, and HSTS in install.ini.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>connections.json &gt; filesystem_root</t>
+          <t>install.ini &gt; [server] content-security-policy / x-frame-options / x-content-type-options / x-xss-protection / hsts-max-age / referrer-policy / permissions-policy / cross-origin-embedder-policy / cross-origin-opener-policy / cross-origin-resource-policy</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>not_exists</t>
+          <t>exists</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>removed (unless replaced by a scoped connection after confirming no active project usage)</t>
+          <t>restrictive values configured for each applicable header (e.g., x-frame-options=SAMEORIGIN, x-content-type-options=nosniff, hsts-max-age set to a non-zero value, a content-security-policy restricting sources)</t>
         </is>
       </c>
       <c r="K5" s="3" t="n"/>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>Check usage via Administration -&gt; Monitoring before deletion.</t>
+          <t>The source provides an example syntax but does not mandate one canonical value set for every header; presence of a restrictive, deliberately-chosen value for each relevant header indicates the practice is followed.</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>filesystem_root connection absent from the connections list, or confirmed unused and removed; if it was in use, a dedicated scoped connection was created to replace it.</t>
+          <t>install.ini's [server] section contains one or more of these header keys with restrictive values (e.g., SAMEORIGIN/DENY for x-frame-options, nosniff for x-content-type-options, a non-trivial content-security-policy, hsts-max-age set).</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>filesystem_root connection still present and either unused (should have been deleted) or in use without a safer scoped replacement.</t>
+          <t>The [server] section lacks these header keys entirely, meaning DSS is not emitting these security headers (browser defaults/no explicit protection).</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>If the connections list isn't in the diagnosis, flag needs_manual_review and check the Administration &gt; Connections UI directly.</t>
+          <t>install.ini is a server-level config file often not captured in diagnostics; if absent, flag as needs_manual_review, since the default state (no headers configured) cannot otherwise be confirmed.</t>
         </is>
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>The filesystem_root connection exposes the entire server filesystem, posing a security and stability risk.</t>
+          <t>Configuring these headers hardens the DSS Web application against clickjacking, XSS, MIME-sniffing, protocol downgrade, and cross-origin data leakage attacks.</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>connections, filesystem_root, security</t>
+          <t>install.ini, HTTP security headers, CSP, HSTS</t>
         </is>
       </c>
       <c r="R5" s="3" t="inlineStr">
         <is>
-          <t>scalable_performance_ops</t>
+          <t>advanced_security_options</t>
         </is>
       </c>
       <c r="S5" s="3" t="inlineStr">
         <is>
-          <t>14, 15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="T5" s="3" t="inlineStr">
         <is>
-          <t>Remove filesystem_root connection | MUST HAVE; Remove filesystem_root connection | MUST HAVE</t>
+          <t>Setting security-related HTTP headers</t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr">
@@ -2587,406 +3946,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AA3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="50" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="40" customWidth="1" min="14" max="14"/>
-    <col width="40" customWidth="1" min="15" max="15"/>
-    <col width="36" customWidth="1" min="16" max="16"/>
-    <col width="24" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="24" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="40" customWidth="1" min="22" max="22"/>
-    <col width="16" customWidth="1" min="23" max="23"/>
-    <col width="40" customWidth="1" min="24" max="24"/>
-    <col width="40" customWidth="1" min="25" max="25"/>
-    <col width="16" customWidth="1" min="26" max="26"/>
-    <col width="20" customWidth="1" min="27" max="27"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>priority</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>check_type</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>subtopic</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>statement</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>statement_short</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>parameter_hint</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>operator</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>expected_value</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>expected_condition_notes</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>supporting_evidence</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>contradicting_evidence</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>insufficient_evidence_handling</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>rationale</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>dataiku_concepts</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>source_document</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>source_page</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>source_section</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>confidence</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>ambiguity_notes</t>
-        </is>
-      </c>
-      <c r="W1" s="2" t="inlineStr">
-        <is>
-          <t>validation_status</t>
-        </is>
-      </c>
-      <c r="X1" s="2" t="inlineStr">
-        <is>
-          <t>evidence_found</t>
-        </is>
-      </c>
-      <c r="Y1" s="2" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-      <c r="Z1" s="2" t="inlineStr">
-        <is>
-          <t>validated_at</t>
-        </is>
-      </c>
-      <c r="AA1" s="2" t="inlineStr">
-        <is>
-          <t>validated_by</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>ADVSEC-003</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>must_have</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>specific_setting</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Session Management</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Expiring sessions</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>DSS can be configured to expire user sessions after a maximum duration since login and/or after a period of inactivity, via Administration &gt; Settings &gt; Security &amp; Audit &gt; User login &amp; provisioning &gt; Session management ('Maximum session duration' and 'Idle timeout'), noting this can cause lost work if a session expires mid-edit.</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Configure maximum session duration and idle timeout to automatically expire user sessions.</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>general-settings.json &gt; security.sessionsMaxTotalTimeMinutes / security.sessionsMaxIdleTimeMinutes (UI: Administration &gt; Settings &gt; Security &amp; Audit &gt; User login &amp; provisioning &gt; Session management)</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>exists</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>either value set to a finite number of minutes greater than 0</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>In general-settings.json a value of 0 means unlimited (the default). The source does not mandate a specific threshold; treat as satisfied if either or both values are greater than 0.</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>general-settings.json security.sessionsMaxTotalTimeMinutes and/or security.sessionsMaxIdleTimeMinutes is greater than 0.</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>Both keys are 0 (unlimited) or absent.</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>Flag needs_manual_review only if general-settings.json or its security block is not in the diagnosis; otherwise decide from the two keys. Note the source's caveat that expiring sessions can lose in-progress work.</t>
-        </is>
-      </c>
-      <c r="P2" s="3" t="inlineStr">
-        <is>
-          <t>Session expiration limits how long a stolen or abandoned session remains valid, though the source warns it can cause lost in-progress work (including complications with open Jupyter notebooks).</t>
-        </is>
-      </c>
-      <c r="Q2" s="3" t="inlineStr">
-        <is>
-          <t>session management, user login &amp; provisioning</t>
-        </is>
-      </c>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>advanced_security_options</t>
-        </is>
-      </c>
-      <c r="S2" s="3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="T2" s="3" t="inlineStr">
-        <is>
-          <t>Expiring sessions</t>
-        </is>
-      </c>
-      <c r="U2" s="3" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="V2" s="3" t="inlineStr">
-        <is>
-          <t>The source gives only the UI path and no numeric threshold; the file keys were verified against sample bundles, not the source documents.</t>
-        </is>
-      </c>
-      <c r="W2" s="3" t="n"/>
-      <c r="X2" s="3" t="n"/>
-      <c r="Y2" s="3" t="n"/>
-      <c r="Z2" s="3" t="n"/>
-      <c r="AA2" s="3" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>ADVSEC-006</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>nice_to_have</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>specific_setting</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Session &amp; Logout UX</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Redirecting to a custom URL after logout</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>By default, users are redirected to a standard DSS-hosted page after logout; administrators can configure security.postLogoutBehavior (CUSTOM_URL for a GET redirect or CUSTOM_URL_POST for a POST request aligned with OpenID Connect RP-Initiated Logout) together with security.postLogoutCustomURL (must be an http/https URL) in general-settings.json to redirect users elsewhere, with DSS validating these settings on save/load and falling back to the default page on invalid values.</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Configure postLogoutBehavior and postLogoutCustomURL to redirect users after logout.</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>general-settings.json &gt; security.postLogoutBehavior / security.postLogoutCustomURL</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>one_of</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>CUSTOM_URL, CUSTOM_URL_POST</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>postLogoutCustomURL is required and must be an http/https URL when postLogoutBehavior is CUSTOM_URL or CUSTOM_URL_POST; DSS validates these settings on save and on load, falling back to the default DSS logged-out page if invalid.</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>general-settings.json "security" object contains postLogoutBehavior set to CUSTOM_URL or CUSTOM_URL_POST along with a valid http/https postLogoutCustomURL.</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>The keys are absent (default DSS logged-out page used) or postLogoutCustomURL is invalid, in which case DSS falls back to default behavior anyway.</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>If general-settings.json content is not present in the diagnosis, flag as needs_manual_review; absence means the default logout page is used, which is not a security concern.</t>
-        </is>
-      </c>
-      <c r="P3" s="3" t="inlineStr">
-        <is>
-          <t>Allows organizations to redirect users to a branded or external page after logout instead of the DSS default logged-out page.</t>
-        </is>
-      </c>
-      <c r="Q3" s="3" t="inlineStr">
-        <is>
-          <t>general-settings.json, security settings, logout, OpenID Connect</t>
-        </is>
-      </c>
-      <c r="R3" s="3" t="inlineStr">
-        <is>
-          <t>advanced_security_options</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="inlineStr">
-        <is>
-          <t>4, 5</t>
-        </is>
-      </c>
-      <c r="T3" s="3" t="inlineStr">
-        <is>
-          <t>Redirecting to a custom URL after logout; Redirecting to a custom URL after logout</t>
-        </is>
-      </c>
-      <c r="U3" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="V3" s="3" t="n"/>
-      <c r="W3" s="3" t="n"/>
-      <c r="X3" s="3" t="n"/>
-      <c r="Y3" s="3" t="n"/>
-      <c r="Z3" s="3" t="n"/>
-      <c r="AA3" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Release 0.28.0: reader 0.10.0, calibrations for SEC-001/SEC-009/ARCH-004/SCALE-010, fixtures and tests
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/checklists/eval_checklist.xlsx
+++ b/tests/fixtures/checklists/eval_checklist.xlsx
@@ -1316,7 +1316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA4"/>
+  <dimension ref="A1:AA6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1488,79 +1488,67 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>SEC-002</t>
+          <t>SEC-001</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>specific_setting</t>
+          <t>qualitative_practice</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>User Isolation Framework</t>
+          <t>Instance Identification</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>User Isolation Framework (UIF) Enabled with Appropriate Impersonation Rules</t>
+          <t>Verify/Capture Instance IDs</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Ensure the User Isolation Framework (UIF) is installed and enabled, with impersonation active and sensible impersonation rules in place (a one-to-one mapping or regex pattern ensuring all DSS users map to identities other than the dataiku service account). For Kubernetes workloads, one namespace per user is recommended; for Hadoop workloads, Sentry/Ranger should be used to manage access. Also check for any Sanity Check warnings regarding UIF.</t>
+          <t>For an established platform, confirm that each node's instance ID (found in {DATA_DIR}/install.ini) is accurately recorded in the platform's tracking/tooling system.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Enable User Isolation Framework with impersonation rules mapping all users away from the service account.</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>{DATA_DIR}/config/general-settings.json &gt; impersonation.enabled</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>equals</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
+          <t>Confirm each node's instance ID is accurately recorded in platform tracking tooling.</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n"/>
       <c r="K2" s="3" t="n"/>
       <c r="L2" s="3" t="n"/>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json shows impersonation.enabled: true with userRules configured as a one-to-one mapping or regex rule mapping DSS users to non-service-account identities; no Sanity Check warnings about UIF; for K8s workloads a per-user namespace strategy is evident; for Hadoop workloads Sentry/Ranger integration is present.</t>
+          <t>Platform tooling/documentation shows an instance ID for each node matching the value found in {DATA_DIR}/install.ini on that node.</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>impersonation.enabled is false or absent, userRules are missing/overly permissive (e.g., mapping to the dataiku service account), Sanity Check warnings reference UIF, or Kubernetes/Hadoop workloads lack namespace-per-user/Sentry-Ranger controls.</t>
+          <t>Instance IDs are missing, blank, or mismatched between install.ini and the platform tooling records.</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file lacks general-settings.json impersonation details or workload-specific config, flag as needs_manual_review, noting that longstanding instances without UIF require careful, considerate customer messaging and that disabling/downgrading UIF is not supported.</t>
+          <t>A diagnosis file alone can show the instance ID value in install.ini but cannot confirm whether it is accurately recorded in external platform tooling; flag as needs_manual_review to cross-check against the tooling record.</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>UIF and correct impersonation rules are required for proper user isolation and security; without them workloads may run under a shared service account, creating security risk and instability in multi-user environments.</t>
+          <t>Accurate instance ID records ensure the platform tooling correctly tracks and manages each node.</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>User Isolation Framework, impersonation, Kubernetes namespaces, Hadoop Sentry/Ranger</t>
+          <t>install.ini, instance tracking</t>
         </is>
       </c>
       <c r="R2" s="3" t="inlineStr">
@@ -1570,20 +1558,24 @@
       </c>
       <c r="S2" s="3" t="inlineStr">
         <is>
-          <t>2, 3</t>
+          <t>1, 2</t>
         </is>
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>User Isolation Framework | MUST HAVE; User Isolation Framework | MUST HAVE (Front End/Back End/Notes)</t>
+          <t>Verify/Capture Instance IDs | NICE TO HAVE; DiagParser3</t>
         </is>
       </c>
       <c r="U2" s="3" t="inlineStr">
         <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="V2" s="3" t="n"/>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V2" s="3" t="inlineStr">
+        <is>
+          <t>No literal JSON field/diag pointer given beyond the file path itself; this is more a documentation-accuracy check than a technical setting.</t>
+        </is>
+      </c>
       <c r="W2" s="3" t="n"/>
       <c r="X2" s="3" t="n"/>
       <c r="Y2" s="3" t="n"/>
@@ -1593,7 +1585,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>SEC-004</t>
+          <t>SEC-002</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1608,27 +1600,27 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>CGroups</t>
+          <t>User Isolation Framework</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>CGroups Enabled with Memory Limit per Sizing Heuristic</t>
+          <t>User Isolation Framework (UIF) Enabled with Appropriate Impersonation Rules</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Ensure cgroups support is enabled and a memory limit is configured for all memory cgroups, sized according to the recommended heuristic (e.g., 32GB VM -&gt; 10g, 64GB -&gt; 38g, 96GB -&gt; 60g, 128GB+ -&gt; 75% of physical memory), with cgroup placements set for all categories.</t>
+          <t>Ensure the User Isolation Framework (UIF) is installed and enabled, with impersonation active and sensible impersonation rules in place (a one-to-one mapping or regex pattern ensuring all DSS users map to identities other than the dataiku service account). For Kubernetes workloads, one namespace per user is recommended; for Hadoop workloads, Sentry/Ranger should be used to manage access. Also check for any Sanity Check warnings regarding UIF.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Enable cgroups with a memory limit sized per the recommended heuristic for instance RAM.</t>
+          <t>Enable User Isolation Framework with impersonation rules mapping all users away from the service account.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>{DATA_DIR}/config/general-settings.json &gt; cgroupSettings.enabled</t>
+          <t>{DATA_DIR}/config/general-settings.json &gt; impersonation.enabled</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -1642,34 +1634,30 @@
         </is>
       </c>
       <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>Additional checks required: cgroupSettings &gt; cgroups memory limit target should be set and sized per the documented heuristic (approx. 50-75% of physical memory depending on total RAM); no single literal field given for the limit value itself, so compare against the formula in evaluation_guidance.</t>
-        </is>
-      </c>
+      <c r="L3" s="3" t="n"/>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json shows cgroupSettings.enabled: true, targets set for each category under cgroups, and a memory limit configured on memory cgroups (e.g., memory/DSS) that approximates the documented formula based on total instance memory (e.g., ~75% for &gt;120GB, ~66% for 60-120GB, total-20GB for 30-60GB, ~50% below 30GB). Front-end equivalent: Administration &gt; Settings &gt; Resource Control &gt; cgroups shows 'Enable cgroups support' selected with placements and memory limits configured.</t>
+          <t>general-settings.json shows impersonation.enabled: true with userRules configured as a one-to-one mapping or regex rule mapping DSS users to non-service-account identities; no Sanity Check warnings about UIF; for K8s workloads a per-user namespace strategy is evident; for Hadoop workloads Sentry/Ranger integration is present.</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>cgroupSettings.enabled is false/absent, no memory limit is set on memory cgroups, or the configured limit is far below the heuristic (e.g., unlimited or near-total memory), risking instability.</t>
+          <t>impersonation.enabled is false or absent, userRules are missing/overly permissive (e.g., mapping to the dataiku service account), Sanity Check warnings reference UIF, or Kubernetes/Hadoop workloads lack namespace-per-user/Sentry-Ranger controls.</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>If cgroupSettings or category placements are not visible in the diagnosis file, flag as needs_manual_review; also check whether the instance was recently reprovisioned (Cloud Stacks) or upgraded, as cgroup limits/placements may not auto-update and new placements may need to be added post-upgrade.</t>
+          <t>If the diagnosis file lacks general-settings.json impersonation details or workload-specific config, flag as needs_manual_review, noting that longstanding instances without UIF require careful, considerate customer messaging and that disabling/downgrading UIF is not supported.</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>A memory cgroup limit prevents runaway processes from destabilizing or degrading the DSS instance; sizing per the heuristic balances safety with usable memory.</t>
+          <t>UIF and correct impersonation rules are required for proper user isolation and security; without them workloads may run under a shared service account, creating security risk and instability in multi-user environments.</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>cgroups, memory limits, Resource Control</t>
+          <t>User Isolation Framework, impersonation, Kubernetes namespaces, Hadoop Sentry/Ranger</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
@@ -1679,12 +1667,12 @@
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
-          <t>3, 4, 5</t>
+          <t>2, 3</t>
         </is>
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>CGroups | MUST HAVE; CGroups | MUST HAVE (Review steps); CGroups | MUST HAVE (Notes)</t>
+          <t>User Isolation Framework | MUST HAVE; User Isolation Framework | MUST HAVE (Front End/Back End/Notes)</t>
         </is>
       </c>
       <c r="U3" s="3" t="inlineStr">
@@ -1702,12 +1690,12 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>SEC-006</t>
+          <t>SEC-004</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>nice_to_have</t>
+          <t>must_have</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -1717,68 +1705,68 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>HTTPS Configuration</t>
+          <t>CGroups</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>HTTPS Access Configured for DSS</t>
+          <t>CGroups Enabled with Memory Limit per Sizing Heuristic</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Verify with the customer whether HTTPS access to DSS is configured, either natively via DSS configuration or through a reverse proxy. For custom installations, inspect the [server] section of install.ini; for Cloud Stacks (Fleet Manager) installations, inspect nodes-directory.json in the Instance Diag.</t>
+          <t>Ensure cgroups support is enabled and a memory limit is configured for all memory cgroups, sized according to the recommended heuristic (e.g., 32GB VM -&gt; 10g, 64GB -&gt; 38g, 96GB -&gt; 60g, 128GB+ -&gt; 75% of physical memory), with cgroup placements set for all categories.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Verify HTTPS access to DSS is configured natively or via a reverse proxy.</t>
+          <t>Enable cgroups with a memory limit sized per the recommended heuristic for instance RAM.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>install.ini &gt; [server] section (HTTPS settings) or /data/dataiku/dss_data/run/nodes-directory.json</t>
+          <t>{DATA_DIR}/config/general-settings.json &gt; cgroupSettings.enabled</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>exists</t>
+          <t>equals</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>HTTPS enabled (natively or via reverse proxy)</t>
+          <t>true</t>
         </is>
       </c>
       <c r="K4" s="3" t="n"/>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>No single literal key name given for the HTTPS flag itself; pointer is to the file/section where it should be inspected.</t>
+          <t>Additional checks required: cgroupSettings &gt; cgroups memory limit target should be set and sized per the documented heuristic (approx. 50-75% of physical memory depending on total RAM); no single literal field given for the limit value itself, so compare against the formula in evaluation_guidance.</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>install.ini [server] section shows native HTTPS parameters configured, or nodes-directory.json shows HTTPS URLs/ports for nodes, or customer confirms a reverse proxy terminates HTTPS in front of DSS.</t>
+          <t>general-settings.json shows cgroupSettings.enabled: true, targets set for each category under cgroups, and a memory limit configured on memory cgroups (e.g., memory/DSS) that approximates the documented formula based on total instance memory (e.g., ~75% for &gt;120GB, ~66% for 60-120GB, total-20GB for 30-60GB, ~50% below 30GB). Front-end equivalent: Administration &gt; Settings &gt; Resource Control &gt; cgroups shows 'Enable cgroups support' selected with placements and memory limits configured.</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>Only HTTP is configured with no reverse proxy in front, and install.ini/nodes-directory.json show no HTTPS-related configuration.</t>
+          <t>cgroupSettings.enabled is false/absent, no memory limit is set on memory cgroups, or the configured limit is far below the heuristic (e.g., unlimited or near-total memory), risking instability.</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not include install.ini or nodes-directory.json content, or if reverse-proxy setup is external to DSS, flag as needs_manual_review and confirm directly with the customer.</t>
+          <t>If cgroupSettings or category placements are not visible in the diagnosis file, flag as needs_manual_review; also check whether the instance was recently reprovisioned (Cloud Stacks) or upgraded, as cgroup limits/placements may not auto-update and new placements may need to be added post-upgrade.</t>
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>HTTPS protects data in transit and is recommended practice for securing access to DSS.</t>
+          <t>A memory cgroup limit prevents runaway processes from destabilizing or degrading the DSS instance; sizing per the heuristic balances safety with usable memory.</t>
         </is>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>HTTPS, reverse proxy, install.ini, nodes-directory.json</t>
+          <t>cgroups, memory limits, Resource Control</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
@@ -1788,17 +1776,17 @@
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>5, 6</t>
+          <t>3, 4, 5</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>HTTPS | NICE TO HAVE; HTTPS | NICE TO HAVE (Review steps)</t>
+          <t>CGroups | MUST HAVE; CGroups | MUST HAVE (Review steps); CGroups | MUST HAVE (Notes)</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="V4" s="3" t="n"/>
@@ -1807,6 +1795,224 @@
       <c r="Y4" s="3" t="n"/>
       <c r="Z4" s="3" t="n"/>
       <c r="AA4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>SEC-006</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>nice_to_have</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>HTTPS Configuration</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>HTTPS Access Configured for DSS</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Verify with the customer whether HTTPS access to DSS is configured, either natively via DSS configuration or through a reverse proxy. For custom installations, inspect the [server] section of install.ini; for Cloud Stacks (Fleet Manager) installations, inspect nodes-directory.json in the Instance Diag.</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Verify HTTPS access to DSS is configured natively or via a reverse proxy.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>install.ini &gt; [server] section (HTTPS settings) or /data/dataiku/dss_data/run/nodes-directory.json</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>exists</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>HTTPS enabled (natively or via reverse proxy)</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>No single literal key name given for the HTTPS flag itself; pointer is to the file/section where it should be inspected.</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>install.ini [server] section shows native HTTPS parameters configured, or nodes-directory.json shows HTTPS URLs/ports for nodes, or customer confirms a reverse proxy terminates HTTPS in front of DSS.</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>Only HTTP is configured with no reverse proxy in front, and install.ini/nodes-directory.json show no HTTPS-related configuration.</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not include install.ini or nodes-directory.json content, or if reverse-proxy setup is external to DSS, flag as needs_manual_review and confirm directly with the customer.</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>HTTPS protects data in transit and is recommended practice for securing access to DSS.</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>HTTPS, reverse proxy, install.ini, nodes-directory.json</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>security_permissions_compliance</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>5, 6</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="inlineStr">
+        <is>
+          <t>HTTPS | NICE TO HAVE; HTTPS | NICE TO HAVE (Review steps)</t>
+        </is>
+      </c>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V5" s="3" t="n"/>
+      <c r="W5" s="3" t="n"/>
+      <c r="X5" s="3" t="n"/>
+      <c r="Y5" s="3" t="n"/>
+      <c r="Z5" s="3" t="n"/>
+      <c r="AA5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>SEC-009</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>nice_to_have</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>LDAP Configuration</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>LDAP Authorized Groups Configured</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Where DSS is integrated with LDAP, ensure Authorized Groups are configured so that only members of specified groups can connect; if LDAP is enabled but no Authorized Groups are set, all LDAP users matching the User filter query can connect, which should be flagged to the customer as a recommended improvement.</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Configure LDAP Authorized Groups to restrict which LDAP users can connect to DSS.</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>{DATA_DIR}/config/general-settings.json &gt; ldapSettings.authorizedGroups</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>exists</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>non-empty (populated with one or more groups)</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Check is conditional on ldapSettings.enabled being true.</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json shows ldapSettings.enabled: true and authorizedGroups populated with one or more group entries; front-end equivalent shows Authorized groups field populated under Login (LDAP, SSO) &amp; Security &gt; Groups mapping.</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>ldapSettings.enabled is true but authorizedGroups is empty or absent, meaning all LDAP users passing the User filter can connect without group-based restriction.</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>If ldapSettings is not present or LDAP is not enabled, this check does not apply; if enabled but authorizedGroups status is unclear, flag as needs_manual_review.</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>Authorized Groups restrict which LDAP-authenticated users may connect to DSS, reducing unauthorized access risk.</t>
+        </is>
+      </c>
+      <c r="Q6" s="3" t="inlineStr">
+        <is>
+          <t>LDAP, authorizedGroups, authentication</t>
+        </is>
+      </c>
+      <c r="R6" s="3" t="inlineStr">
+        <is>
+          <t>security_permissions_compliance</t>
+        </is>
+      </c>
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>7, 8</t>
+        </is>
+      </c>
+      <c r="T6" s="3" t="inlineStr">
+        <is>
+          <t>LDAP: Authorized groups | NICE TO HAVE; LDAP: Authorized groups | NICE TO HAVE (Review steps)</t>
+        </is>
+      </c>
+      <c r="U6" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V6" s="3" t="n"/>
+      <c r="W6" s="3" t="n"/>
+      <c r="X6" s="3" t="n"/>
+      <c r="Y6" s="3" t="n"/>
+      <c r="Z6" s="3" t="n"/>
+      <c r="AA6" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2306,7 +2512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA9"/>
+  <dimension ref="A1:AA10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3217,12 +3423,12 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>SCALE-011</t>
+          <t>SCALE-010</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -3232,68 +3438,68 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Connections Hygiene</t>
+          <t>Default Connection &amp; Engine Preferences</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Remove filesystem_root Connection</t>
+          <t>Preferred Connections and Engines Settings</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>The default filesystem_root connection pointing to the server's root filesystem should be removed unless actively used by a project; if in use, propose a dedicated scoped connection to the specific path before removing filesystem_root.</t>
+          <t>Default dataset creation settings and recipe engine preferences (preferedConnection, forcedPreferedConnection, preferedUploadConnection, preferedStorageFormats) are blank by default and should remain so unless a specific use case justifies setting them; in particular, preferred engine should almost always be left blank for v12+ instances since altering it can cause breaking changes.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Remove the filesystem_root connection unless actively used, replacing it with a scoped connection.</t>
+          <t>Leave default connection and engine preferences blank unless a specific use case justifies them.</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>connections.json &gt; filesystem_root</t>
+          <t>general-settings.json &gt; defaultDatasetCreationSettings / recipeEnginesPreferences (preferedConnection, forcedPreferedConnection, preferedUploadConnection, preferedStorageFormats)</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>not_exists</t>
+          <t>equals</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>removed (unless replaced by a scoped connection after confirming no active project usage)</t>
+          <t>unset/blank unless justified specific use case</t>
         </is>
       </c>
       <c r="K9" s="3" t="n"/>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>Check usage via Administration -&gt; Monitoring before deletion.</t>
+          <t>These keys may be entirely absent from general-settings.json if left blank, which is the expected default state.</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>filesystem_root connection absent from the connections list, or confirmed unused and removed; if it was in use, a dedicated scoped connection was created to replace it.</t>
+          <t>Keys absent or blank in general-settings.json, or if set, a documented specific use case justifies the value (e.g., not forcing storage to a local server).</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>filesystem_root connection still present and either unused (should have been deleted) or in use without a safer scoped replacement.</t>
+          <t>preferedConnection/forcedPreferedConnection set to force local server storage, or preferred engine changed without clear justification, especially on v12+ instances.</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>If the connections list isn't in the diagnosis, flag needs_manual_review and check the Administration &gt; Connections UI directly.</t>
+          <t>If this section of general-settings.json is missing from the diagnosis, flag needs_manual_review and check the Administration &gt; Settings &gt; Engines &amp; connections UI.</t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>The filesystem_root connection exposes the entire server filesystem, posing a security and stability risk.</t>
+          <t>These settings default to blank for good reason; forcing values can cause breaking changes or performance issues (e.g., forcing local storage).</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>connections, filesystem_root, security</t>
+          <t>default dataset creation, recipe engine preferences, connections</t>
         </is>
       </c>
       <c r="R9" s="3" t="inlineStr">
@@ -3303,25 +3509,138 @@
       </c>
       <c r="S9" s="3" t="inlineStr">
         <is>
-          <t>14, 15</t>
+          <t>12, 13, 14</t>
         </is>
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>Remove filesystem_root connection | MUST HAVE; Remove filesystem_root connection | MUST HAVE</t>
+          <t>Preferreds and Defaults | NICE TO HAVE; Preferreds and Defaults | NICE TO HAVE; Preferreds and Defaults | NICE TO HAVE</t>
         </is>
       </c>
       <c r="U9" s="3" t="inlineStr">
         <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="V9" s="3" t="n"/>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V9" s="3" t="inlineStr">
+        <is>
+          <t>Expected value is contextual ('reasonable values' if set), not a fixed constant, so the check requires judgment.</t>
+        </is>
+      </c>
       <c r="W9" s="3" t="n"/>
       <c r="X9" s="3" t="n"/>
       <c r="Y9" s="3" t="n"/>
       <c r="Z9" s="3" t="n"/>
       <c r="AA9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>SCALE-011</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Connections Hygiene</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Remove filesystem_root Connection</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>The default filesystem_root connection pointing to the server's root filesystem should be removed unless actively used by a project; if in use, propose a dedicated scoped connection to the specific path before removing filesystem_root.</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Remove the filesystem_root connection unless actively used, replacing it with a scoped connection.</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>connections.json &gt; filesystem_root</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>not_exists</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>removed (unless replaced by a scoped connection after confirming no active project usage)</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>Check usage via Administration -&gt; Monitoring before deletion.</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>filesystem_root connection absent from the connections list, or confirmed unused and removed; if it was in use, a dedicated scoped connection was created to replace it.</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>filesystem_root connection still present and either unused (should have been deleted) or in use without a safer scoped replacement.</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>If the connections list isn't in the diagnosis, flag needs_manual_review and check the Administration &gt; Connections UI directly.</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>The filesystem_root connection exposes the entire server filesystem, posing a security and stability risk.</t>
+        </is>
+      </c>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>connections, filesystem_root, security</t>
+        </is>
+      </c>
+      <c r="R10" s="3" t="inlineStr">
+        <is>
+          <t>scalable_performance_ops</t>
+        </is>
+      </c>
+      <c r="S10" s="3" t="inlineStr">
+        <is>
+          <t>14, 15</t>
+        </is>
+      </c>
+      <c r="T10" s="3" t="inlineStr">
+        <is>
+          <t>Remove filesystem_root connection | MUST HAVE; Remove filesystem_root connection | MUST HAVE</t>
+        </is>
+      </c>
+      <c r="U10" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V10" s="3" t="n"/>
+      <c r="W10" s="3" t="n"/>
+      <c r="X10" s="3" t="n"/>
+      <c r="Y10" s="3" t="n"/>
+      <c r="Z10" s="3" t="n"/>
+      <c r="AA10" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Release 0.28.1: SEC-010 calibration (SSO disabled = Fail, SSO+LDAP enabled = Pass, otherwise Needs Review), fixtures
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/checklists/eval_checklist.xlsx
+++ b/tests/fixtures/checklists/eval_checklist.xlsx
@@ -1316,7 +1316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA6"/>
+  <dimension ref="A1:AA7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2013,6 +2013,103 @@
       <c r="Y6" s="3" t="n"/>
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>SEC-010</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>nice_to_have</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>qualitative_practice</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Single Sign-On</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>SSO Enablement Reviewed</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Verify whether SSO is enabled for the DSS instance; if not, discuss with the customer whether enabling SSO would benefit their deployment.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Verify whether SSO is enabled and discuss potential benefits with the customer.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>Configuration or documentation indicates SSO is enabled and integrated with the customer's identity provider.</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>SSO is not configured and there is no record of a discussion with the customer about its potential benefits.</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>Diagnosis files may not clearly expose SSO configuration; if unclear, flag as needs_manual_review and recommend confirming SSO status directly with the customer/admin settings.</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>SSO can improve authentication security and user experience by centralizing identity management.</t>
+        </is>
+      </c>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>SSO, authentication</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>security_permissions_compliance</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>SSO | NICE TO HAVE</t>
+        </is>
+      </c>
+      <c r="U7" s="3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="V7" s="3" t="inlineStr">
+        <is>
+          <t>No literal field path or diag pointer is given for SSO status in this document.</t>
+        </is>
+      </c>
+      <c r="W7" s="3" t="n"/>
+      <c r="X7" s="3" t="n"/>
+      <c r="Y7" s="3" t="n"/>
+      <c r="Z7" s="3" t="n"/>
+      <c r="AA7" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Release 0.29.0: reader 0.11.0 (byo_llm), calibrations for ARCH-003/SEC-005/GENAI-005/GENAI-006, fixtures and tests
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/checklists/eval_checklist.xlsx
+++ b/tests/fixtures/checklists/eval_checklist.xlsx
@@ -437,6 +437,982 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:AA9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="40" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="40" customWidth="1" min="24" max="24"/>
+    <col width="40" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>check_type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>subtopic</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>statement</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>statement_short</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>parameter_hint</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>operator</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>expected_value</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>expected_condition_notes</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>supporting_evidence</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>contradicting_evidence</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>insufficient_evidence_handling</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>rationale</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>dataiku_concepts</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>source_document</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>source_page</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>source_section</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>ambiguity_notes</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>validation_status</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>evidence_found</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>validated_at</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>validated_by</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-001</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>qualitative_practice</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Deployment Infrastructure</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Separation of Design and Automation Nodes</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Production-grade Dataiku deployments should separate experimental/design work from production runs by leveraging dedicated automation nodes; reviewers should discuss the Design -&gt; Deployer -&gt; Automation Node architecture with the customer and flag gaps, even though standing up new nodes is out of scope for the review itself.</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Separate production workloads onto dedicated automation nodes rather than running everything on the design node.</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Diagnosis shows a distinct automation node (or nodes) separate from the design node, with a deployer configured and bundles being pushed from design to automation.</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Only a single design node is used to run both experimentation and production workloads, with no automation node or deployer in use.</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not expose node topology/roles, flag needs_manual_review and recommend discussing the Design -&gt; Deployer -&gt; Automation architecture directly with the customer.</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>Mixing experimental and production work on the same node risks instability and is not considered production-ready.</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>Design node, Automation node, Deployer, Bundles</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
+      <c r="T2" s="3" t="inlineStr">
+        <is>
+          <t>Dataiku Deployment Infrastructure | MUST HAVE; Dataiku Deployment Infrastructure | MUST HAVE</t>
+        </is>
+      </c>
+      <c r="U2" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V2" s="3" t="n"/>
+      <c r="W2" s="3" t="n"/>
+      <c r="X2" s="3" t="n"/>
+      <c r="Y2" s="3" t="n"/>
+      <c r="Z2" s="3" t="n"/>
+      <c r="AA2" s="3" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-002</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>nice_to_have</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>qualitative_practice</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Platform Versioning</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Regular DSS Version Upgrades</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Dataiku recommends customers stay reasonably current on DSS versions to benefit from continuous platform improvements; reviewers should identify and recommend an upgrade if appropriate, but the upgrade itself is a separate service-catalog engagement and should not be performed during the review.</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Recommend upgrading DSS to a reasonably current version via a separate service engagement.</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="n"/>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Diagnosis shows a DSS version reasonably close to the latest generally available release.</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>Diagnosis shows a DSS version many releases behind current, or a version approaching/at end-of-life.</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file lacks version information or there is no context on Dataiku's release cadence, flag needs_manual_review and recommend checking DSS release notes for the customer's version.</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>Dataiku regularly enriches the platform, so staying current continuously brings value and new opportunities to customers.</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>DSS version, Upgrade</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>Dataiku Version | NICE TO HAVE</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V3" s="3" t="n"/>
+      <c r="W3" s="3" t="n"/>
+      <c r="X3" s="3" t="n"/>
+      <c r="Y3" s="3" t="n"/>
+      <c r="Z3" s="3" t="n"/>
+      <c r="AA3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-003</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>qualitative_practice</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Operating System</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Supported Operating System Version</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>DSS should run on an operating system version officially supported by Dataiku, which mainly matters for custom installs since Cloud Stacks provides a supported OS image by default; reviewers should compare the current OS against Dataiku's supported OS list and deprecation notices and recommend upgrades if needed.</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Run DSS on an operating system version officially supported by Dataiku.</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Diagnosis or accompanying metadata shows the host OS and version currently listed as supported in Dataiku's Supported Operating Systems documentation.</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>The host OS/version is deprecated or not on Dataiku's supported list for the installed DSS version.</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not capture OS name/version, flag needs_manual_review and cross-check against Dataiku's Supported Operating Systems documentation.</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>Running on an unsupported OS risks instability and lack of vendor support.</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>Operating System, Custom install, Cloud Stacks</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>Operating System Version | MUST HAVE</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V4" s="3" t="inlineStr">
+        <is>
+          <t>The source includes an empty 'DiagParser3:' heading with no field specified underneath, so no literal parameter path could be extracted; treated as a qualitative check instead.</t>
+        </is>
+      </c>
+      <c r="W4" s="3" t="n"/>
+      <c r="X4" s="3" t="n"/>
+      <c r="Y4" s="3" t="n"/>
+      <c r="Z4" s="3" t="n"/>
+      <c r="AA4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-004</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>qualitative_practice</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>SSD Storage for DSS</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>DSS should run on SSD drives rather than legacy rotational hard drives, since rotational disks can significantly degrade performance, especially on larger, multi-user instances (potentially causing a non-workable experience); reviewers should identify currently used disk types and recommend migration to SSD where feasible, noting this is typically easier on cloud than on-premise deployments.</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Run DSS on SSD storage instead of rotational hard drives for performance.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n"/>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Diagnosis or infrastructure metadata indicates SSD-backed storage underlying the DATADIR.</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>Diagnosis or infrastructure metadata indicates rotational HDD storage is in use, particularly on a larger or many-user instance.</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not report the underlying disk/storage medium, flag needs_manual_review and ask the infrastructure team/customer directly.</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>Rotational hard drives can severely impact performance and, on larger instances with many users, may lead to a non-workable experience.</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>Disk I/O, SSD, DATADIR</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>2, 3</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="inlineStr">
+        <is>
+          <t>Use of SSDs | MUST HAVE; Use of SSDs | MUST HAVE</t>
+        </is>
+      </c>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V5" s="3" t="n"/>
+      <c r="W5" s="3" t="n"/>
+      <c r="X5" s="3" t="n"/>
+      <c r="Y5" s="3" t="n"/>
+      <c r="Z5" s="3" t="n"/>
+      <c r="AA5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-006</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>nice_to_have</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Spark Configuration</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Baseline Spark Configuration Set (High/Standard/Large-memory/High I/O)</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Dataiku recommends defining multiple named Spark configurations as a tunable baseline: a default Standard config for recipes and notebooks, a High config for higher parallelism, a Large memory config for the largest jobs, and an optional High I/O config for read/write-heavy workloads with a high cores-to-memory ratio.</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Define Standard, High, Large-memory, and optional High I/O Spark configurations as a baseline.</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; sparkSettings (named spark configs)</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>one_of</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Standard/High/Large-memory baseline configs, plus optional High I/O config, as documented</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Baseline reference values: Standard config - spark.executor.instances=4, spark.executor.memory=6g, spark.executor.cores=2, spark.kubernetes.memoryOverheadFactor=0.4, spark.driver.memory=1g, spark.sql.shuffle.partitions=40, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. High config - spark.executor.instances=12, spark.executor.memory=6g, spark.executor.cores=2, spark.kubernetes.memoryOverheadFactor=0.4, spark.driver.memory=1g, spark.sql.shuffle.partitions=80, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. Large memory config - spark.executor.instances=4, spark.executor.memory=12g, spark.executor.cores=2, spark.kubernetes.memoryOverheadFactor=0.6, spark.driver.memory=3g, spark.sql.shuffle.partitions=80, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. Optional High I/O config (only if there is a use case for it) - spark.executor.instances=2, spark.executor.memory=16g, spark.executor.cores=8, spark.kubernetes.memoryOverheadFactor=0.4, spark.driver.memory=3g, spark.sql.shuffle.partitions=40, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. These values are guidance, not a requirement.</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>sparkSettings contains multiple named configs roughly matching these purposes (default/high-parallelism/large-memory, and optionally high I/O).</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>Only a single undifferentiated spark config exists despite varied workload needs (e.g., both lightweight recipes and large jobs run identically).</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not list multiple sparkSettings configs or describe workload diversity, flag needs_manual_review and ask about workload variety.</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>Different Spark workloads (lightweight recipes vs. large jobs vs. I/O-heavy jobs) benefit from different executor sizing and parallelism trade-offs.</t>
+        </is>
+      </c>
+      <c r="Q6" s="3" t="inlineStr">
+        <is>
+          <t>Spark executor, Spark configuration, Kubernetes</t>
+        </is>
+      </c>
+      <c r="R6" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>4, 5</t>
+        </is>
+      </c>
+      <c r="T6" s="3" t="inlineStr">
+        <is>
+          <t>Define three spark configs - NICE TO HAVE; Special spark configs (only if there's use case for it)</t>
+        </is>
+      </c>
+      <c r="U6" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V6" s="3" t="n"/>
+      <c r="W6" s="3" t="n"/>
+      <c r="X6" s="3" t="n"/>
+      <c r="Y6" s="3" t="n"/>
+      <c r="Z6" s="3" t="n"/>
+      <c r="AA6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-008</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>qualitative_practice</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Spark Validation</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Functional Validation of Spark Execution (Recipe &amp; Notebook)</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Reviewers should functionally validate Spark execution: run a Spark-engine recipe on Kubernetes in a test project (should succeed), and separately launch a Python/R/Scala notebook with starter Spark code and run it locally (should succeed, with Spark executor pods visible in the cluster while the code runs).</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Validate Spark execution by successfully running a test Spark recipe and notebook.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>Job/notebook execution logs show successful completion of a Spark recipe and a Spark notebook session, and cluster monitoring shows executor pods created during notebook execution.</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>The Spark recipe or notebook execution fails, hangs, or no executor pods ever appear in the cluster.</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file lacks job/notebook execution logs or cluster pod visibility, flag needs_manual_review and recommend running these test steps manually.</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>Confirms Spark integration works end-to-end, beyond just having a syntactically valid configuration.</t>
+        </is>
+      </c>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>Spark recipe, Spark notebook, Kubernetes executor pods</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>5, 6, 7</t>
+        </is>
+      </c>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>Additional Spark testing; Spark on Notebook MUST HAVE; Spark on Notebook MUST HAVE</t>
+        </is>
+      </c>
+      <c r="U7" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V7" s="3" t="inlineStr">
+        <is>
+          <t>Worded for Spark on Kubernetes (executor pods). If no Kubernetes cluster is attached and Spark runs on YARN/Hadoop, the pod-based checks do not apply.</t>
+        </is>
+      </c>
+      <c r="W7" s="3" t="n"/>
+      <c r="X7" s="3" t="n"/>
+      <c r="Y7" s="3" t="n"/>
+      <c r="Z7" s="3" t="n"/>
+      <c r="AA7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-010</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Containerized Execution</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Valid Containerized Execution Configuration</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Environments using Elastic Compute (Kubernetes) must have at least one valid containerized execution configuration set up (general-settings.json &gt; containerSettings, or Administration &gt; Settings &gt; Containerized execution); as with Spark, the specific example values are only a baseline, not a strict requirement.</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Configure at least one valid containerized execution config when using Elastic Compute.</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; containerSettings</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>exists</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>valid containerized execution configuration present</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>Required only when the customer uses Elastic Compute/Kubernetes for offloaded workloads.</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>containerSettings block is present with at least one named config with reasonable memory requests/limits.</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>containerSettings is missing or empty while the instance shows evidence of Kubernetes-based execution elsewhere in the diagnosis.</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not clarify whether Elastic Compute is used, flag needs_manual_review.</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>A valid container exec config is required to run workloads in Kubernetes.</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>Containerized execution, containerSettings, Elastic Compute</t>
+        </is>
+      </c>
+      <c r="R8" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S8" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="T8" s="3" t="inlineStr">
+        <is>
+          <t>Containerized execution configs | MUST HAVE if using Elastic Compute</t>
+        </is>
+      </c>
+      <c r="U8" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V8" s="3" t="n"/>
+      <c r="W8" s="3" t="n"/>
+      <c r="X8" s="3" t="n"/>
+      <c r="Y8" s="3" t="n"/>
+      <c r="Z8" s="3" t="n"/>
+      <c r="AA8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-013</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Cluster Configuration</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Valid Cluster Configuration for Elastic Compute</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Environments using Elastic Compute must have at least one valid cluster configured (found under {DATADIR}/config/clusters or Administration &gt; Clusters); Dataiku does not mandate the specific example configuration, only that a workable cluster exists.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Configure at least one valid Kubernetes cluster when using Elastic Compute.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>{DATADIR}/config/clusters</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>exists</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>at least one valid cluster configuration present</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="n"/>
+      <c r="L9" s="3" t="n"/>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>The clusters config/directory contains at least one properly defined cluster, consistent with other evidence of elastic-compute usage (spark/container jobs running on Kubernetes).</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>No cluster configuration is present despite evidence of Kubernetes-based workloads elsewhere in the diagnosis.</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not clarify whether Elastic Compute is used at all, flag needs_manual_review.</t>
+        </is>
+      </c>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>A valid cluster is required to offload computation to Kubernetes.</t>
+        </is>
+      </c>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>Cluster, Managed cluster, Unmanaged cluster, Elastic AI</t>
+        </is>
+      </c>
+      <c r="R9" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S9" s="3" t="inlineStr">
+        <is>
+          <t>12, 13</t>
+        </is>
+      </c>
+      <c r="T9" s="3" t="inlineStr">
+        <is>
+          <t>Cluster configurations | MUST HAVE if using Elastic Compute; Cluster configurations | MUST HAVE if using Elastic Compute</t>
+        </is>
+      </c>
+      <c r="U9" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V9" s="3" t="n"/>
+      <c r="W9" s="3" t="n"/>
+      <c r="X9" s="3" t="n"/>
+      <c r="Y9" s="3" t="n"/>
+      <c r="Z9" s="3" t="n"/>
+      <c r="AA9" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AA8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -609,12 +1585,12 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>ARCH-001</t>
+          <t>SEC-001</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -624,22 +1600,22 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Deployment Infrastructure</t>
+          <t>Instance Identification</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Separation of Design and Automation Nodes</t>
+          <t>Verify/Capture Instance IDs</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Production-grade Dataiku deployments should separate experimental/design work from production runs by leveraging dedicated automation nodes; reviewers should discuss the Design -&gt; Deployer -&gt; Automation Node architecture with the customer and flag gaps, even though standing up new nodes is out of scope for the review itself.</t>
+          <t>For an established platform, confirm that each node's instance ID (found in {DATA_DIR}/install.ini) is accurately recorded in the platform's tracking/tooling system.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Separate production workloads onto dedicated automation nodes rather than running everything on the design node.</t>
+          <t>Confirm each node's instance ID is accurately recorded in platform tracking tooling.</t>
         </is>
       </c>
       <c r="H2" s="3" t="n"/>
@@ -649,32 +1625,32 @@
       <c r="L2" s="3" t="n"/>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>Diagnosis shows a distinct automation node (or nodes) separate from the design node, with a deployer configured and bundles being pushed from design to automation.</t>
+          <t>Platform tooling/documentation shows an instance ID for each node matching the value found in {DATA_DIR}/install.ini on that node.</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>Only a single design node is used to run both experimentation and production workloads, with no automation node or deployer in use.</t>
+          <t>Instance IDs are missing, blank, or mismatched between install.ini and the platform tooling records.</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not expose node topology/roles, flag needs_manual_review and recommend discussing the Design -&gt; Deployer -&gt; Automation architecture directly with the customer.</t>
+          <t>A diagnosis file alone can show the instance ID value in install.ini but cannot confirm whether it is accurately recorded in external platform tooling; flag as needs_manual_review to cross-check against the tooling record.</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>Mixing experimental and production work on the same node risks instability and is not considered production-ready.</t>
+          <t>Accurate instance ID records ensure the platform tooling correctly tracks and manages each node.</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>Design node, Automation node, Deployer, Bundles</t>
+          <t>install.ini, instance tracking</t>
         </is>
       </c>
       <c r="R2" s="3" t="inlineStr">
         <is>
-          <t>architecture_compute_cost</t>
+          <t>security_permissions_compliance</t>
         </is>
       </c>
       <c r="S2" s="3" t="inlineStr">
@@ -684,15 +1660,19 @@
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>Dataiku Deployment Infrastructure | MUST HAVE; Dataiku Deployment Infrastructure | MUST HAVE</t>
+          <t>Verify/Capture Instance IDs | NICE TO HAVE; DiagParser3</t>
         </is>
       </c>
       <c r="U2" s="3" t="inlineStr">
         <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="V2" s="3" t="n"/>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V2" s="3" t="inlineStr">
+        <is>
+          <t>No literal JSON field/diag pointer given beyond the file path itself; this is more a documentation-accuracy check than a technical setting.</t>
+        </is>
+      </c>
       <c r="W2" s="3" t="n"/>
       <c r="X2" s="3" t="n"/>
       <c r="Y2" s="3" t="n"/>
@@ -702,82 +1682,94 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>ARCH-002</t>
+          <t>SEC-002</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>nice_to_have</t>
+          <t>must_have</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>qualitative_practice</t>
+          <t>specific_setting</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Platform Versioning</t>
+          <t>User Isolation Framework</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Regular DSS Version Upgrades</t>
+          <t>User Isolation Framework (UIF) Enabled with Appropriate Impersonation Rules</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Dataiku recommends customers stay reasonably current on DSS versions to benefit from continuous platform improvements; reviewers should identify and recommend an upgrade if appropriate, but the upgrade itself is a separate service-catalog engagement and should not be performed during the review.</t>
+          <t>Ensure the User Isolation Framework (UIF) is installed and enabled, with impersonation active and sensible impersonation rules in place (a one-to-one mapping or regex pattern ensuring all DSS users map to identities other than the dataiku service account). For Kubernetes workloads, one namespace per user is recommended; for Hadoop workloads, Sentry/Ranger should be used to manage access. Also check for any Sanity Check warnings regarding UIF.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Recommend upgrading DSS to a reasonably current version via a separate service engagement.</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
+          <t>Enable User Isolation Framework with impersonation rules mapping all users away from the service account.</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>{DATA_DIR}/config/general-settings.json &gt; impersonation.enabled</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>equals</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="K3" s="3" t="n"/>
       <c r="L3" s="3" t="n"/>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Diagnosis shows a DSS version reasonably close to the latest generally available release.</t>
+          <t>general-settings.json shows impersonation.enabled: true with userRules configured as a one-to-one mapping or regex rule mapping DSS users to non-service-account identities; no Sanity Check warnings about UIF; for K8s workloads a per-user namespace strategy is evident; for Hadoop workloads Sentry/Ranger integration is present.</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>Diagnosis shows a DSS version many releases behind current, or a version approaching/at end-of-life.</t>
+          <t>impersonation.enabled is false or absent, userRules are missing/overly permissive (e.g., mapping to the dataiku service account), Sanity Check warnings reference UIF, or Kubernetes/Hadoop workloads lack namespace-per-user/Sentry-Ranger controls.</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file lacks version information or there is no context on Dataiku's release cadence, flag needs_manual_review and recommend checking DSS release notes for the customer's version.</t>
+          <t>If the diagnosis file lacks general-settings.json impersonation details or workload-specific config, flag as needs_manual_review, noting that longstanding instances without UIF require careful, considerate customer messaging and that disabling/downgrading UIF is not supported.</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>Dataiku regularly enriches the platform, so staying current continuously brings value and new opportunities to customers.</t>
+          <t>UIF and correct impersonation rules are required for proper user isolation and security; without them workloads may run under a shared service account, creating security risk and instability in multi-user environments.</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>DSS version, Upgrade</t>
+          <t>User Isolation Framework, impersonation, Kubernetes namespaces, Hadoop Sentry/Ranger</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
         <is>
-          <t>architecture_compute_cost</t>
+          <t>security_permissions_compliance</t>
         </is>
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2, 3</t>
         </is>
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>Dataiku Version | NICE TO HAVE</t>
+          <t>User Isolation Framework | MUST HAVE; User Isolation Framework | MUST HAVE (Front End/Back End/Notes)</t>
         </is>
       </c>
       <c r="U3" s="3" t="inlineStr">
@@ -795,7 +1787,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>ARCH-004</t>
+          <t>SEC-004</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -805,72 +1797,88 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>qualitative_practice</t>
+          <t>specific_setting</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Storage</t>
+          <t>CGroups</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>SSD Storage for DSS</t>
+          <t>CGroups Enabled with Memory Limit per Sizing Heuristic</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>DSS should run on SSD drives rather than legacy rotational hard drives, since rotational disks can significantly degrade performance, especially on larger, multi-user instances (potentially causing a non-workable experience); reviewers should identify currently used disk types and recommend migration to SSD where feasible, noting this is typically easier on cloud than on-premise deployments.</t>
+          <t>Ensure cgroups support is enabled and a memory limit is configured for all memory cgroups, sized according to the recommended heuristic (e.g., 32GB VM -&gt; 10g, 64GB -&gt; 38g, 96GB -&gt; 60g, 128GB+ -&gt; 75% of physical memory), with cgroup placements set for all categories.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Run DSS on SSD storage instead of rotational hard drives for performance.</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
+          <t>Enable cgroups with a memory limit sized per the recommended heuristic for instance RAM.</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>{DATA_DIR}/config/general-settings.json &gt; cgroupSettings.enabled</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>equals</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Additional checks required: cgroupSettings &gt; cgroups memory limit target should be set and sized per the documented heuristic (approx. 50-75% of physical memory depending on total RAM); no single literal field given for the limit value itself, so compare against the formula in evaluation_guidance.</t>
+        </is>
+      </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>Diagnosis or infrastructure metadata indicates SSD-backed storage underlying the DATADIR.</t>
+          <t>general-settings.json shows cgroupSettings.enabled: true, targets set for each category under cgroups, and a memory limit configured on memory cgroups (e.g., memory/DSS) that approximates the documented formula based on total instance memory (e.g., ~75% for &gt;120GB, ~66% for 60-120GB, total-20GB for 30-60GB, ~50% below 30GB). Front-end equivalent: Administration &gt; Settings &gt; Resource Control &gt; cgroups shows 'Enable cgroups support' selected with placements and memory limits configured.</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>Diagnosis or infrastructure metadata indicates rotational HDD storage is in use, particularly on a larger or many-user instance.</t>
+          <t>cgroupSettings.enabled is false/absent, no memory limit is set on memory cgroups, or the configured limit is far below the heuristic (e.g., unlimited or near-total memory), risking instability.</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not report the underlying disk/storage medium, flag needs_manual_review and ask the infrastructure team/customer directly.</t>
+          <t>If cgroupSettings or category placements are not visible in the diagnosis file, flag as needs_manual_review; also check whether the instance was recently reprovisioned (Cloud Stacks) or upgraded, as cgroup limits/placements may not auto-update and new placements may need to be added post-upgrade.</t>
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>Rotational hard drives can severely impact performance and, on larger instances with many users, may lead to a non-workable experience.</t>
+          <t>A memory cgroup limit prevents runaway processes from destabilizing or degrading the DSS instance; sizing per the heuristic balances safety with usable memory.</t>
         </is>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Disk I/O, SSD, DATADIR</t>
+          <t>cgroups, memory limits, Resource Control</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>architecture_compute_cost</t>
+          <t>security_permissions_compliance</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>2, 3</t>
+          <t>3, 4, 5</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>Use of SSDs | MUST HAVE; Use of SSDs | MUST HAVE</t>
+          <t>CGroups | MUST HAVE; CGroups | MUST HAVE (Review steps); CGroups | MUST HAVE (Notes)</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
@@ -888,12 +1896,12 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>ARCH-006</t>
+          <t>SEC-005</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>nice_to_have</t>
+          <t>must_have</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -903,91 +1911,95 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Spark Configuration</t>
+          <t>CGroups</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Baseline Spark Configuration Set (High/Standard/Large-memory/High I/O)</t>
+          <t>JEK-Specific CGroup Limits Left Unconfigured</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Dataiku recommends defining multiple named Spark configurations as a tunable baseline: a default Standard config for recipes and notebooks, a High config for higher parallelism, a Large memory config for the largest jobs, and an optional High I/O config for read/write-heavy workloads with a high cores-to-memory ratio.</t>
+          <t>Do not set specific cgroup limits for individual Job Execution Kernels (JEKs) unless dealing with a rare, highly specialized edge case, as this can cause unexpected execution throttles; JEK-specific cgroups should generally remain unconfigured.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Define Standard, High, Large-memory, and optional High I/O Spark configurations as a baseline.</t>
+          <t>Avoid setting JEK-specific cgroup limits except in rare specialized edge cases.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; sparkSettings (named spark configs)</t>
+          <t>general-settings.json &gt; cgroupSettings (JEK-specific cgroup entries)</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>one_of</t>
+          <t>not_exists</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Standard/High/Large-memory baseline configs, plus optional High I/O config, as documented</t>
+          <t>No JEK-specific cgroup limits configured</t>
         </is>
       </c>
       <c r="K5" s="3" t="n"/>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>Baseline reference values: Standard config - spark.executor.instances=4, spark.executor.memory=6g, spark.executor.cores=2, spark.kubernetes.memoryOverheadFactor=0.4, spark.driver.memory=1g, spark.sql.shuffle.partitions=40, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. High config - spark.executor.instances=12, spark.executor.memory=6g, spark.executor.cores=2, spark.kubernetes.memoryOverheadFactor=0.4, spark.driver.memory=1g, spark.sql.shuffle.partitions=80, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. Large memory config - spark.executor.instances=4, spark.executor.memory=12g, spark.executor.cores=2, spark.kubernetes.memoryOverheadFactor=0.6, spark.driver.memory=3g, spark.sql.shuffle.partitions=80, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. Optional High I/O config (only if there is a use case for it) - spark.executor.instances=2, spark.executor.memory=16g, spark.executor.cores=8, spark.kubernetes.memoryOverheadFactor=0.4, spark.driver.memory=3g, spark.sql.shuffle.partitions=40, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. These values are guidance, not a requirement.</t>
+          <t>No literal field path given for JEK-specific cgroup entries; conceptual pointer based on general cgroupSettings structure.</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>sparkSettings contains multiple named configs roughly matching these purposes (default/high-parallelism/large-memory, and optionally high I/O).</t>
+          <t>cgroupSettings configuration shows no per-JEK-specific memory/CPU limits distinct from the general DSS cgroup limits.</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>Only a single undifferentiated spark config exists despite varied workload needs (e.g., both lightweight recipes and large jobs run identically).</t>
+          <t>Specific cgroup limits are found configured for individual Job Kernels without documented justification for a specialized edge case.</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not list multiple sparkSettings configs or describe workload diversity, flag needs_manual_review and ask about workload variety.</t>
+          <t>If the diagnosis file does not clearly break down cgroup settings by JEK vs. general placement, flag as needs_manual_review and recommend checking internal deep-dive documentation if an exception is suspected.</t>
         </is>
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>Different Spark workloads (lightweight recipes vs. large jobs vs. I/O-heavy jobs) benefit from different executor sizing and parallelism trade-offs.</t>
+          <t>Per-JEK cgroup limits can cause unexpected execution throttling, degrading job performance.</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>Spark executor, Spark configuration, Kubernetes</t>
+          <t>cgroups, Job Execution Kernel (JEK)</t>
         </is>
       </c>
       <c r="R5" s="3" t="inlineStr">
         <is>
-          <t>architecture_compute_cost</t>
+          <t>security_permissions_compliance</t>
         </is>
       </c>
       <c r="S5" s="3" t="inlineStr">
         <is>
-          <t>4, 5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="T5" s="3" t="inlineStr">
         <is>
-          <t>Define three spark configs - NICE TO HAVE; Special spark configs (only if there's use case for it)</t>
+          <t>CGroups | MUST HAVE</t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr">
         <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="V5" s="3" t="n"/>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V5" s="3" t="inlineStr">
+        <is>
+          <t>Priority classification is inferred; this could arguably be nice_to_have as it's a caution rather than a baseline requirement, but the explicit performance-degradation risk supports must_have.</t>
+        </is>
+      </c>
       <c r="W5" s="3" t="n"/>
       <c r="X5" s="3" t="n"/>
       <c r="Y5" s="3" t="n"/>
@@ -997,94 +2009,106 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>ARCH-008</t>
+          <t>SEC-006</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>qualitative_practice</t>
+          <t>specific_setting</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Spark Validation</t>
+          <t>HTTPS Configuration</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Functional Validation of Spark Execution (Recipe &amp; Notebook)</t>
+          <t>HTTPS Access Configured for DSS</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Reviewers should functionally validate Spark execution: run a Spark-engine recipe on Kubernetes in a test project (should succeed), and separately launch a Python/R/Scala notebook with starter Spark code and run it locally (should succeed, with Spark executor pods visible in the cluster while the code runs).</t>
+          <t>Verify with the customer whether HTTPS access to DSS is configured, either natively via DSS configuration or through a reverse proxy. For custom installations, inspect the [server] section of install.ini; for Cloud Stacks (Fleet Manager) installations, inspect nodes-directory.json in the Instance Diag.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Validate Spark execution by successfully running a test Spark recipe and notebook.</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
+          <t>Verify HTTPS access to DSS is configured natively or via a reverse proxy.</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>install.ini &gt; [server] section (HTTPS settings) or /data/dataiku/dss_data/run/nodes-directory.json</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>exists</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>HTTPS enabled (natively or via reverse proxy)</t>
+        </is>
+      </c>
       <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>No single literal key name given for the HTTPS flag itself; pointer is to the file/section where it should be inspected.</t>
+        </is>
+      </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>Job/notebook execution logs show successful completion of a Spark recipe and a Spark notebook session, and cluster monitoring shows executor pods created during notebook execution.</t>
+          <t>install.ini [server] section shows native HTTPS parameters configured, or nodes-directory.json shows HTTPS URLs/ports for nodes, or customer confirms a reverse proxy terminates HTTPS in front of DSS.</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>The Spark recipe or notebook execution fails, hangs, or no executor pods ever appear in the cluster.</t>
+          <t>Only HTTP is configured with no reverse proxy in front, and install.ini/nodes-directory.json show no HTTPS-related configuration.</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file lacks job/notebook execution logs or cluster pod visibility, flag needs_manual_review and recommend running these test steps manually.</t>
+          <t>If the diagnosis file does not include install.ini or nodes-directory.json content, or if reverse-proxy setup is external to DSS, flag as needs_manual_review and confirm directly with the customer.</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>Confirms Spark integration works end-to-end, beyond just having a syntactically valid configuration.</t>
+          <t>HTTPS protects data in transit and is recommended practice for securing access to DSS.</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>Spark recipe, Spark notebook, Kubernetes executor pods</t>
+          <t>HTTPS, reverse proxy, install.ini, nodes-directory.json</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
         <is>
-          <t>architecture_compute_cost</t>
+          <t>security_permissions_compliance</t>
         </is>
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>5, 6, 7</t>
+          <t>5, 6</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>Additional Spark testing; Spark on Notebook MUST HAVE; Spark on Notebook MUST HAVE</t>
+          <t>HTTPS | NICE TO HAVE; HTTPS | NICE TO HAVE (Review steps)</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="V6" s="3" t="inlineStr">
-        <is>
-          <t>Worded for Spark on Kubernetes (executor pods). If no Kubernetes cluster is attached and Spark runs on YARN/Hadoop, the pod-based checks do not apply.</t>
-        </is>
-      </c>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V6" s="3" t="n"/>
       <c r="W6" s="3" t="n"/>
       <c r="X6" s="3" t="n"/>
       <c r="Y6" s="3" t="n"/>
@@ -1094,12 +2118,12 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>ARCH-010</t>
+          <t>SEC-009</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -1109,27 +2133,27 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Containerized Execution</t>
+          <t>LDAP Configuration</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Valid Containerized Execution Configuration</t>
+          <t>LDAP Authorized Groups Configured</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Environments using Elastic Compute (Kubernetes) must have at least one valid containerized execution configuration set up (general-settings.json &gt; containerSettings, or Administration &gt; Settings &gt; Containerized execution); as with Spark, the specific example values are only a baseline, not a strict requirement.</t>
+          <t>Where DSS is integrated with LDAP, ensure Authorized Groups are configured so that only members of specified groups can connect; if LDAP is enabled but no Authorized Groups are set, all LDAP users matching the User filter query can connect, which should be flagged to the customer as a recommended improvement.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Configure at least one valid containerized execution config when using Elastic Compute.</t>
+          <t>Configure LDAP Authorized Groups to restrict which LDAP users can connect to DSS.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; containerSettings</t>
+          <t>{DATA_DIR}/config/general-settings.json &gt; ldapSettings.authorizedGroups</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -1139,53 +2163,53 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>valid containerized execution configuration present</t>
+          <t>non-empty (populated with one or more groups)</t>
         </is>
       </c>
       <c r="K7" s="3" t="n"/>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>Required only when the customer uses Elastic Compute/Kubernetes for offloaded workloads.</t>
+          <t>Check is conditional on ldapSettings.enabled being true.</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>containerSettings block is present with at least one named config with reasonable memory requests/limits.</t>
+          <t>general-settings.json shows ldapSettings.enabled: true and authorizedGroups populated with one or more group entries; front-end equivalent shows Authorized groups field populated under Login (LDAP, SSO) &amp; Security &gt; Groups mapping.</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>containerSettings is missing or empty while the instance shows evidence of Kubernetes-based execution elsewhere in the diagnosis.</t>
+          <t>ldapSettings.enabled is true but authorizedGroups is empty or absent, meaning all LDAP users passing the User filter can connect without group-based restriction.</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not clarify whether Elastic Compute is used, flag needs_manual_review.</t>
+          <t>If ldapSettings is not present or LDAP is not enabled, this check does not apply; if enabled but authorizedGroups status is unclear, flag as needs_manual_review.</t>
         </is>
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>A valid container exec config is required to run workloads in Kubernetes.</t>
+          <t>Authorized Groups restrict which LDAP-authenticated users may connect to DSS, reducing unauthorized access risk.</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>Containerized execution, containerSettings, Elastic Compute</t>
+          <t>LDAP, authorizedGroups, authentication</t>
         </is>
       </c>
       <c r="R7" s="3" t="inlineStr">
         <is>
-          <t>architecture_compute_cost</t>
+          <t>security_permissions_compliance</t>
         </is>
       </c>
       <c r="S7" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7, 8</t>
         </is>
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>Containerized execution configs | MUST HAVE if using Elastic Compute</t>
+          <t>LDAP: Authorized groups | NICE TO HAVE; LDAP: Authorized groups | NICE TO HAVE (Review steps)</t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr">
@@ -1203,102 +2227,94 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>ARCH-013</t>
+          <t>SEC-010</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>specific_setting</t>
+          <t>qualitative_practice</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Cluster Configuration</t>
+          <t>Single Sign-On</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Valid Cluster Configuration for Elastic Compute</t>
+          <t>SSO Enablement Reviewed</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Environments using Elastic Compute must have at least one valid cluster configured (found under {DATADIR}/config/clusters or Administration &gt; Clusters); Dataiku does not mandate the specific example configuration, only that a workable cluster exists.</t>
+          <t>Verify whether SSO is enabled for the DSS instance; if not, discuss with the customer whether enabling SSO would benefit their deployment.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Configure at least one valid Kubernetes cluster when using Elastic Compute.</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>{DATADIR}/config/clusters</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>exists</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>at least one valid cluster configuration present</t>
-        </is>
-      </c>
+          <t>Verify whether SSO is enabled and discuss potential benefits with the customer.</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="n"/>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="n"/>
       <c r="K8" s="3" t="n"/>
       <c r="L8" s="3" t="n"/>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>The clusters config/directory contains at least one properly defined cluster, consistent with other evidence of elastic-compute usage (spark/container jobs running on Kubernetes).</t>
+          <t>Configuration or documentation indicates SSO is enabled and integrated with the customer's identity provider.</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>No cluster configuration is present despite evidence of Kubernetes-based workloads elsewhere in the diagnosis.</t>
+          <t>SSO is not configured and there is no record of a discussion with the customer about its potential benefits.</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not clarify whether Elastic Compute is used at all, flag needs_manual_review.</t>
+          <t>Diagnosis files may not clearly expose SSO configuration; if unclear, flag as needs_manual_review and recommend confirming SSO status directly with the customer/admin settings.</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>A valid cluster is required to offload computation to Kubernetes.</t>
+          <t>SSO can improve authentication security and user experience by centralizing identity management.</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>Cluster, Managed cluster, Unmanaged cluster, Elastic AI</t>
+          <t>SSO, authentication</t>
         </is>
       </c>
       <c r="R8" s="3" t="inlineStr">
         <is>
-          <t>architecture_compute_cost</t>
+          <t>security_permissions_compliance</t>
         </is>
       </c>
       <c r="S8" s="3" t="inlineStr">
         <is>
-          <t>12, 13</t>
+          <t>8</t>
         </is>
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>Cluster configurations | MUST HAVE if using Elastic Compute; Cluster configurations | MUST HAVE if using Elastic Compute</t>
+          <t>SSO | NICE TO HAVE</t>
         </is>
       </c>
       <c r="U8" s="3" t="inlineStr">
         <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="V8" s="3" t="n"/>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="V8" s="3" t="inlineStr">
+        <is>
+          <t>No literal field path or diag pointer is given for SSO status in this document.</t>
+        </is>
+      </c>
       <c r="W8" s="3" t="n"/>
       <c r="X8" s="3" t="n"/>
       <c r="Y8" s="3" t="n"/>
@@ -1310,13 +2326,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA7"/>
+  <dimension ref="A1:AA6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1488,94 +2504,106 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>SEC-001</t>
+          <t>GENAI-001</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>nice_to_have</t>
+          <t>must_have</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>qualitative_practice</t>
+          <t>specific_setting</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Instance Identification</t>
+          <t>LLM Mesh and Agents</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Verify/Capture Instance IDs</t>
+          <t>Internal Code Environments for RAG, Document Extraction, PII Detection</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>For an established platform, confirm that each node's instance ID (found in {DATA_DIR}/install.ini) is accurately recorded in the platform's tracking/tooling system.</t>
+          <t>Ensure the internal code environments for Retrieval-Augmented Generation, document extraction, and PII detection are properly installed and set as the default code-env for each category under Administration &gt; Settings &gt; Other &gt; LLM Mesh. If a non-internal code-env is used instead, DSS surfaces a warning in the LLM Mesh settings page and in Administration &gt; Code-envs &gt; Internal envs.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Confirm each node's instance ID is accurately recorded in platform tracking tooling.</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
+          <t>Use internal code environments as default for RAG, document extraction, and PII detection.</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; generativeAISettings &gt; defaultRetrievableKnowledgeCodeEnv</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>not_exists</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>absent (i.e., using internal default code-env, containerMode NONE)</t>
+        </is>
+      </c>
       <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>If defaultRetrievableKnowledgeCodeEnv is present with a custom value and containerMode is INHERIT, a non-internal code-env is in use. Also check presidioBasedPIIDetection (PII detection) and embedDocumentsRecipeSettings (document extraction) keys for equivalent non-internal overrides.</t>
+        </is>
+      </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>Platform tooling/documentation shows an instance ID for each node matching the value found in {DATA_DIR}/install.ini on that node.</t>
+          <t>general-settings.json generativeAISettings shows containerMode NONE with no defaultRetrievableKnowledgeCodeEnv key, and PII/doc extraction sections show no custom code-env overrides; Admin &gt; Code-envs &gt; Internal envs shows RAG/PII/Doc extraction set up as internal.</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>Instance IDs are missing, blank, or mismatched between install.ini and the platform tooling records.</t>
+          <t>defaultRetrievableKnowledgeCodeEnv key present with a non-internal value, containerMode INHERIT, or a warning banner shown in Admin &gt; Settings &gt; Other &gt; LLM Mesh / Code-envs &gt; Internal envs.</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>A diagnosis file alone can show the instance ID value in install.ini but cannot confirm whether it is accurately recorded in external platform tooling; flag as needs_manual_review to cross-check against the tooling record.</t>
+          <t>If generativeAISettings section is absent from the diagnosis, flag needs_manual_review to check the UI directly.</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>Accurate instance ID records ensure the platform tooling correctly tracks and manages each node.</t>
+          <t>Internal code envs bundle the correct/supported dependencies (e.g., libreoffice for document extraction); using a non-internal env can cause missing dependencies or unsupported behavior.</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>install.ini, instance tracking</t>
+          <t>LLM Mesh, code environments, RAG, PII detection, document extraction</t>
         </is>
       </c>
       <c r="R2" s="3" t="inlineStr">
         <is>
-          <t>security_permissions_compliance</t>
+          <t>generative_ai_acceleration</t>
         </is>
       </c>
       <c r="S2" s="3" t="inlineStr">
         <is>
-          <t>1, 2</t>
+          <t>1, 2, 3</t>
         </is>
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>Verify/Capture Instance IDs | NICE TO HAVE; DiagParser3</t>
+          <t>LLM Mesh and Agents MUST HAVE:; RAG, Doc extraction, PII detection; Instance Diags / DiagParser3</t>
         </is>
       </c>
       <c r="U2" s="3" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="V2" s="3" t="inlineStr">
-        <is>
-          <t>No literal JSON field/diag pointer given beyond the file path itself; this is more a documentation-accuracy check than a technical setting.</t>
-        </is>
-      </c>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V2" s="3" t="n"/>
       <c r="W2" s="3" t="n"/>
       <c r="X2" s="3" t="n"/>
       <c r="Y2" s="3" t="n"/>
@@ -1585,7 +2613,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>SEC-002</t>
+          <t>GENAI-005</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1600,79 +2628,75 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>User Isolation Framework</t>
+          <t>Bring Your Own LLM Mode</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>User Isolation Framework (UIF) Enabled with Appropriate Impersonation Rules</t>
+          <t>Bring Your Own LLM Mode - Reference Project &amp; Main Model</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Ensure the User Isolation Framework (UIF) is installed and enabled, with impersonation active and sensible impersonation rules in place (a one-to-one mapping or regex pattern ensuring all DSS users map to identities other than the dataiku service account). For Kubernetes workloads, one namespace per user is recommended; for Hadoop workloads, Sentry/Ranger should be used to manage access. Also check for any Sanity Check warnings regarding UIF.</t>
+          <t>When Bring Your Own LLM mode is active, a Reference project key must be set (used for LLM Mesh requests running outside a DSS project, e.g. AI Search) and a main LLM model must be configured; if unset, requests will fail.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Enable User Isolation Framework with impersonation rules mapping all users away from the service account.</t>
+          <t>Set a Reference project key and main LLM model when using Bring Your Own LLM.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>{DATA_DIR}/config/general-settings.json &gt; impersonation.enabled</t>
+          <t>general-settings.json &gt; localAIServerSettings.referenceProjectKey / mainLLMId</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>equals</t>
+          <t>exists</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>non-empty values set for both fields</t>
         </is>
       </c>
       <c r="K3" s="3" t="n"/>
       <c r="L3" s="3" t="n"/>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json shows impersonation.enabled: true with userRules configured as a one-to-one mapping or regex rule mapping DSS users to non-service-account identities; no Sanity Check warnings about UIF; for K8s workloads a per-user namespace strategy is evident; for Hadoop workloads Sentry/Ranger integration is present.</t>
+          <t>localAIServerSettings.useLocalServer=true with referenceProjectKey and mainLLMId populated (e.g., 'openai:openai-adrissi:gpt-5.5').</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>impersonation.enabled is false or absent, userRules are missing/overly permissive (e.g., mapping to the dataiku service account), Sanity Check warnings reference UIF, or Kubernetes/Hadoop workloads lack namespace-per-user/Sentry-Ranger controls.</t>
+          <t>useLocalServer=true but referenceProjectKey or mainLLMId missing or empty.</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file lacks general-settings.json impersonation details or workload-specific config, flag as needs_manual_review, noting that longstanding instances without UIF require careful, considerate customer messaging and that disabling/downgrading UIF is not supported.</t>
-        </is>
-      </c>
-      <c r="P3" s="3" t="inlineStr">
-        <is>
-          <t>UIF and correct impersonation rules are required for proper user isolation and security; without them workloads may run under a shared service account, creating security risk and instability in multi-user environments.</t>
-        </is>
-      </c>
+          <t>If localAIServerSettings is absent from the diagnosis, flag needs_manual_review to confirm whether Bring Your Own LLM mode is in use.</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="n"/>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>User Isolation Framework, impersonation, Kubernetes namespaces, Hadoop Sentry/Ranger</t>
+          <t>Bring Your Own LLM, AI Services, LLM Mesh</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
         <is>
-          <t>security_permissions_compliance</t>
+          <t>generative_ai_acceleration</t>
         </is>
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
-          <t>2, 3</t>
+          <t>5, 6</t>
         </is>
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>User Isolation Framework | MUST HAVE; User Isolation Framework | MUST HAVE (Front End/Back End/Notes)</t>
+          <t>Bring your own LLM Mode; Instance Diags / DiagParser3</t>
         </is>
       </c>
       <c r="U3" s="3" t="inlineStr">
@@ -1690,12 +2714,12 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>SEC-004</t>
+          <t>GENAI-006</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -1705,88 +2729,88 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>CGroups</t>
+          <t>Bring Your Own LLM Mode</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>CGroups Enabled with Memory Limit per Sizing Heuristic</t>
+          <t>Bring Your Own LLM - Recommended Model Versions</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Ensure cgroups support is enabled and a memory limit is configured for all memory cgroups, sized according to the recommended heuristic (e.g., 32GB VM -&gt; 10g, 64GB -&gt; 38g, 96GB -&gt; 60g, 128GB+ -&gt; 75% of physical memory), with cgroup placements set for all categories.</t>
+          <t>If the customer has activated Bring Your Own LLM Mode for AI Assistants, verify they are using recommended model versions (minimum OpenAI ChatGPT 5.2) and avoid unsupported ones (e.g., ChatGPT 5.1, which will not provide good results).</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Enable cgroups with a memory limit sized per the recommended heuristic for instance RAM.</t>
+          <t>Use at least ChatGPT 5.2 for Bring Your Own LLM; avoid version 5.1.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>{DATA_DIR}/config/general-settings.json &gt; cgroupSettings.enabled</t>
+          <t>general-settings.json &gt; localAIServerSettings.mainLLMId (and responseFormatAwareLLMId/fastLightLLMId)</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>equals</t>
+          <t>not_equals</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>ChatGPT 5.1 or earlier / unsupported model versions</t>
         </is>
       </c>
       <c r="K4" s="3" t="n"/>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>Additional checks required: cgroupSettings &gt; cgroups memory limit target should be set and sized per the documented heuristic (approx. 50-75% of physical memory depending on total RAM); no single literal field given for the limit value itself, so compare against the formula in evaluation_guidance.</t>
+          <t>Exact version comparison against the recommended minimum (ChatGPT 5.2) may require manual judgment; refer to https://doc.dataiku.com/dss/latest/ai-assistants/setup.html#bring-your-own-llm-mode.</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json shows cgroupSettings.enabled: true, targets set for each category under cgroups, and a memory limit configured on memory cgroups (e.g., memory/DSS) that approximates the documented formula based on total instance memory (e.g., ~75% for &gt;120GB, ~66% for 60-120GB, total-20GB for 30-60GB, ~50% below 30GB). Front-end equivalent: Administration &gt; Settings &gt; Resource Control &gt; cgroups shows 'Enable cgroups support' selected with placements and memory limits configured.</t>
+          <t>mainLLMId/related LLM IDs reference gpt-5.2 or later.</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>cgroupSettings.enabled is false/absent, no memory limit is set on memory cgroups, or the configured limit is far below the heuristic (e.g., unlimited or near-total memory), risking instability.</t>
+          <t>mainLLMId/related LLM IDs reference gpt-5.1 or an older/unsupported model.</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>If cgroupSettings or category placements are not visible in the diagnosis file, flag as needs_manual_review; also check whether the instance was recently reprovisioned (Cloud Stacks) or upgraded, as cgroup limits/placements may not auto-update and new placements may need to be added post-upgrade.</t>
+          <t>If the model identifier is ambiguous, non-OpenAI, or version cannot be determined, flag needs_manual_review and reference the setup documentation.</t>
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>A memory cgroup limit prevents runaway processes from destabilizing or degrading the DSS instance; sizing per the heuristic balances safety with usable memory.</t>
+          <t>Using unsupported model versions is stated to produce poor results.</t>
         </is>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>cgroups, memory limits, Resource Control</t>
+          <t>Bring Your Own LLM, Model selection, AI Assistants</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>security_permissions_compliance</t>
+          <t>generative_ai_acceleration</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>3, 4, 5</t>
+          <t>6, 7</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>CGroups | MUST HAVE; CGroups | MUST HAVE (Review steps); CGroups | MUST HAVE (Notes)</t>
+          <t>Bring your own LLM Mode; Bring your own LLM Mode</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="V4" s="3" t="n"/>
@@ -1799,12 +2823,12 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>SEC-006</t>
+          <t>GENAI-007</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>nice_to_have</t>
+          <t>must_have</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -1814,27 +2838,27 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>HTTPS Configuration</t>
+          <t>Cobuild</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>HTTPS Access Configured for DSS</t>
+          <t>Cobuild Default LLM Configuration</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Verify with the customer whether HTTPS access to DSS is configured, either natively via DSS configuration or through a reverse proxy. For custom installations, inspect the [server] section of install.ini; for Cloud Stacks (Fleet Manager) installations, inspect nodes-directory.json in the Instance Diag.</t>
+          <t>Administrators must configure default LLM settings for Cobuild (agent-building tools) upon activation of AI Assistants, including defaultEmbeddingLLMId, defaultLLMId, and defaultImageGenerationLLMId under agentBuildingSettings; if unset, Cobuild's building-agent tools will fail and instruct users to contact an administrator.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Verify HTTPS access to DSS is configured natively or via a reverse proxy.</t>
+          <t>Configure default embedding, LLM, and image-generation models for Cobuild agent building.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>install.ini &gt; [server] section (HTTPS settings) or /data/dataiku/dss_data/run/nodes-directory.json</t>
+          <t>general-settings.json &gt; aiDrivenAnalyticsSettings.agentBuildingSettings.{defaultEmbeddingLLMId, defaultLLMId, defaultImageGenerationLLMId}</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -1844,58 +2868,50 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>HTTPS enabled (natively or via reverse proxy)</t>
+          <t>all three fields populated with valid LLM IDs</t>
         </is>
       </c>
       <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>No single literal key name given for the HTTPS flag itself; pointer is to the file/section where it should be inspected.</t>
-        </is>
-      </c>
+      <c r="L5" s="3" t="n"/>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>install.ini [server] section shows native HTTPS parameters configured, or nodes-directory.json shows HTTPS URLs/ports for nodes, or customer confirms a reverse proxy terminates HTTPS in front of DSS.</t>
+          <t>agentBuildingSettings block shows non-empty defaultEmbeddingLLMId, defaultLLMId, and defaultImageGenerationLLMId values.</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>Only HTTP is configured with no reverse proxy in front, and install.ini/nodes-directory.json show no HTTPS-related configuration.</t>
+          <t>One or more of these fields is missing or empty while Cobuild/AI Assistants is enabled.</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not include install.ini or nodes-directory.json content, or if reverse-proxy setup is external to DSS, flag as needs_manual_review and confirm directly with the customer.</t>
-        </is>
-      </c>
-      <c r="P5" s="3" t="inlineStr">
-        <is>
-          <t>HTTPS protects data in transit and is recommended practice for securing access to DSS.</t>
-        </is>
-      </c>
+          <t>If aiDrivenAnalyticsSettings is absent from the diagnosis, flag needs_manual_review to confirm whether Cobuild/AI Assistants is enabled for this customer.</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="n"/>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>HTTPS, reverse proxy, install.ini, nodes-directory.json</t>
+          <t>Cobuild, AI Assistants, Agent building</t>
         </is>
       </c>
       <c r="R5" s="3" t="inlineStr">
         <is>
-          <t>security_permissions_compliance</t>
+          <t>generative_ai_acceleration</t>
         </is>
       </c>
       <c r="S5" s="3" t="inlineStr">
         <is>
-          <t>5, 6</t>
+          <t>7, 8, 9</t>
         </is>
       </c>
       <c r="T5" s="3" t="inlineStr">
         <is>
-          <t>HTTPS | NICE TO HAVE; HTTPS | NICE TO HAVE (Review steps)</t>
+          <t>Cobuild; Cobuild; Instance Diags / DiagParser3</t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="V5" s="3" t="n"/>
@@ -1908,7 +2924,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>SEC-009</t>
+          <t>GENAI-009</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1918,685 +2934,89 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>specific_setting</t>
+          <t>qualitative_practice</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>LDAP Configuration</t>
+          <t>Agent Hub</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>LDAP Authorized Groups Configured</t>
+          <t>Agent Hub Deployment Required Permissions</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Where DSS is integrated with LDAP, ensure Authorized Groups are configured so that only members of specified groups can connect; if LDAP is enabled but no Authorized Groups are set, all LDAP users matching the User filter query can connect, which should be flagged to the customer as a recommended improvement.</t>
+          <t>Before a user can deploy an Agent Hub instance, they must have permissions for writing project content in the hosting project, writing isolated code execution, WebApp impersonation, and (if Quick agents are enabled) create projects; alternatively the user could be a DSS administrator, though a dedicated service account is preferred.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Configure LDAP Authorized Groups to restrict which LDAP users can connect to DSS.</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>{DATA_DIR}/config/general-settings.json &gt; ldapSettings.authorizedGroups</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>exists</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>non-empty (populated with one or more groups)</t>
-        </is>
-      </c>
+          <t>Grant Agent Hub deployers write project content, isolated code execution, and webapp impersonation permissions.</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
       <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>Check is conditional on ldapSettings.enabled being true.</t>
-        </is>
-      </c>
+      <c r="L6" s="3" t="n"/>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json shows ldapSettings.enabled: true and authorizedGroups populated with one or more group entries; front-end equivalent shows Authorized groups field populated under Login (LDAP, SSO) &amp; Security &gt; Groups mapping.</t>
+          <t>Administration &gt; Security &gt; Groups shows the Agent Hub deployer's group granted 'Write project content', 'Write isolated code execution', and 'WebApp impersonation' permissions (plus 'Create projects' if Quick agents are enabled), or the deployer is a DSS admin/service account.</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>ldapSettings.enabled is true but authorizedGroups is empty or absent, meaning all LDAP users passing the User filter can connect without group-based restriction.</t>
+          <t>The deployer's group lacks one or more of these permissions and is not an admin/service account, or logs show 'Not authorized' errors when creating the Agent Hub WebApp.</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>If ldapSettings is not present or LDAP is not enabled, this check does not apply; if enabled but authorizedGroups status is unclear, flag as needs_manual_review.</t>
+          <t>If the diagnosis file lacks per-user/group permission detail, flag needs_manual_review and recommend checking Administration &gt; Security &gt; Groups directly.</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>Authorized Groups restrict which LDAP-authenticated users may connect to DSS, reducing unauthorized access risk.</t>
+          <t>Missing permissions cause deployment failures such as 'Not authorized' errors when creating the Agent Hub WebApp.</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>LDAP, authorizedGroups, authentication</t>
+          <t>Agent Hub, Permissions, Groups, WebApp</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
         <is>
-          <t>security_permissions_compliance</t>
+          <t>generative_ai_acceleration</t>
         </is>
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>7, 8</t>
+          <t>10, 11, 12</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>LDAP: Authorized groups | NICE TO HAVE; LDAP: Authorized groups | NICE TO HAVE (Review steps)</t>
+          <t>Agent Hub NICE TO HAVE:; Writing isolated code execution; WebApp impersonation</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="V6" s="3" t="n"/>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V6" s="3" t="inlineStr">
+        <is>
+          <t>Although the parent topic is tagged NICE TO HAVE, the described permission requirements are phrased as mandatory ('must have permissions') for successful deployment; classification follows the explicit heading tag.</t>
+        </is>
+      </c>
       <c r="W6" s="3" t="n"/>
       <c r="X6" s="3" t="n"/>
       <c r="Y6" s="3" t="n"/>
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="3" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>SEC-010</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>nice_to_have</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>qualitative_practice</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Single Sign-On</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>SSO Enablement Reviewed</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Verify whether SSO is enabled for the DSS instance; if not, discuss with the customer whether enabling SSO would benefit their deployment.</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Verify whether SSO is enabled and discuss potential benefits with the customer.</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
-      <c r="M7" s="3" t="inlineStr">
-        <is>
-          <t>Configuration or documentation indicates SSO is enabled and integrated with the customer's identity provider.</t>
-        </is>
-      </c>
-      <c r="N7" s="3" t="inlineStr">
-        <is>
-          <t>SSO is not configured and there is no record of a discussion with the customer about its potential benefits.</t>
-        </is>
-      </c>
-      <c r="O7" s="3" t="inlineStr">
-        <is>
-          <t>Diagnosis files may not clearly expose SSO configuration; if unclear, flag as needs_manual_review and recommend confirming SSO status directly with the customer/admin settings.</t>
-        </is>
-      </c>
-      <c r="P7" s="3" t="inlineStr">
-        <is>
-          <t>SSO can improve authentication security and user experience by centralizing identity management.</t>
-        </is>
-      </c>
-      <c r="Q7" s="3" t="inlineStr">
-        <is>
-          <t>SSO, authentication</t>
-        </is>
-      </c>
-      <c r="R7" s="3" t="inlineStr">
-        <is>
-          <t>security_permissions_compliance</t>
-        </is>
-      </c>
-      <c r="S7" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="T7" s="3" t="inlineStr">
-        <is>
-          <t>SSO | NICE TO HAVE</t>
-        </is>
-      </c>
-      <c r="U7" s="3" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="V7" s="3" t="inlineStr">
-        <is>
-          <t>No literal field path or diag pointer is given for SSO status in this document.</t>
-        </is>
-      </c>
-      <c r="W7" s="3" t="n"/>
-      <c r="X7" s="3" t="n"/>
-      <c r="Y7" s="3" t="n"/>
-      <c r="Z7" s="3" t="n"/>
-      <c r="AA7" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AA4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="50" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="40" customWidth="1" min="14" max="14"/>
-    <col width="40" customWidth="1" min="15" max="15"/>
-    <col width="36" customWidth="1" min="16" max="16"/>
-    <col width="24" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="24" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="40" customWidth="1" min="22" max="22"/>
-    <col width="16" customWidth="1" min="23" max="23"/>
-    <col width="40" customWidth="1" min="24" max="24"/>
-    <col width="40" customWidth="1" min="25" max="25"/>
-    <col width="16" customWidth="1" min="26" max="26"/>
-    <col width="20" customWidth="1" min="27" max="27"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>priority</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>check_type</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>subtopic</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>statement</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>statement_short</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>parameter_hint</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>operator</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>expected_value</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>expected_condition_notes</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>supporting_evidence</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>contradicting_evidence</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>insufficient_evidence_handling</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>rationale</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>dataiku_concepts</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>source_document</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>source_page</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>source_section</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>confidence</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>ambiguity_notes</t>
-        </is>
-      </c>
-      <c r="W1" s="2" t="inlineStr">
-        <is>
-          <t>validation_status</t>
-        </is>
-      </c>
-      <c r="X1" s="2" t="inlineStr">
-        <is>
-          <t>evidence_found</t>
-        </is>
-      </c>
-      <c r="Y1" s="2" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-      <c r="Z1" s="2" t="inlineStr">
-        <is>
-          <t>validated_at</t>
-        </is>
-      </c>
-      <c r="AA1" s="2" t="inlineStr">
-        <is>
-          <t>validated_by</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>GENAI-001</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>must_have</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>specific_setting</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>LLM Mesh and Agents</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Internal Code Environments for RAG, Document Extraction, PII Detection</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Ensure the internal code environments for Retrieval-Augmented Generation, document extraction, and PII detection are properly installed and set as the default code-env for each category under Administration &gt; Settings &gt; Other &gt; LLM Mesh. If a non-internal code-env is used instead, DSS surfaces a warning in the LLM Mesh settings page and in Administration &gt; Code-envs &gt; Internal envs.</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Use internal code environments as default for RAG, document extraction, and PII detection.</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>general-settings.json &gt; generativeAISettings &gt; defaultRetrievableKnowledgeCodeEnv</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>not_exists</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>absent (i.e., using internal default code-env, containerMode NONE)</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>If defaultRetrievableKnowledgeCodeEnv is present with a custom value and containerMode is INHERIT, a non-internal code-env is in use. Also check presidioBasedPIIDetection (PII detection) and embedDocumentsRecipeSettings (document extraction) keys for equivalent non-internal overrides.</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>general-settings.json generativeAISettings shows containerMode NONE with no defaultRetrievableKnowledgeCodeEnv key, and PII/doc extraction sections show no custom code-env overrides; Admin &gt; Code-envs &gt; Internal envs shows RAG/PII/Doc extraction set up as internal.</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>defaultRetrievableKnowledgeCodeEnv key present with a non-internal value, containerMode INHERIT, or a warning banner shown in Admin &gt; Settings &gt; Other &gt; LLM Mesh / Code-envs &gt; Internal envs.</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>If generativeAISettings section is absent from the diagnosis, flag needs_manual_review to check the UI directly.</t>
-        </is>
-      </c>
-      <c r="P2" s="3" t="inlineStr">
-        <is>
-          <t>Internal code envs bundle the correct/supported dependencies (e.g., libreoffice for document extraction); using a non-internal env can cause missing dependencies or unsupported behavior.</t>
-        </is>
-      </c>
-      <c r="Q2" s="3" t="inlineStr">
-        <is>
-          <t>LLM Mesh, code environments, RAG, PII detection, document extraction</t>
-        </is>
-      </c>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>generative_ai_acceleration</t>
-        </is>
-      </c>
-      <c r="S2" s="3" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
-      <c r="T2" s="3" t="inlineStr">
-        <is>
-          <t>LLM Mesh and Agents MUST HAVE:; RAG, Doc extraction, PII detection; Instance Diags / DiagParser3</t>
-        </is>
-      </c>
-      <c r="U2" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="V2" s="3" t="n"/>
-      <c r="W2" s="3" t="n"/>
-      <c r="X2" s="3" t="n"/>
-      <c r="Y2" s="3" t="n"/>
-      <c r="Z2" s="3" t="n"/>
-      <c r="AA2" s="3" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>GENAI-007</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>must_have</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>specific_setting</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Cobuild</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Cobuild Default LLM Configuration</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Administrators must configure default LLM settings for Cobuild (agent-building tools) upon activation of AI Assistants, including defaultEmbeddingLLMId, defaultLLMId, and defaultImageGenerationLLMId under agentBuildingSettings; if unset, Cobuild's building-agent tools will fail and instruct users to contact an administrator.</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Configure default embedding, LLM, and image-generation models for Cobuild agent building.</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>general-settings.json &gt; aiDrivenAnalyticsSettings.agentBuildingSettings.{defaultEmbeddingLLMId, defaultLLMId, defaultImageGenerationLLMId}</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>exists</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>all three fields populated with valid LLM IDs</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>agentBuildingSettings block shows non-empty defaultEmbeddingLLMId, defaultLLMId, and defaultImageGenerationLLMId values.</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>One or more of these fields is missing or empty while Cobuild/AI Assistants is enabled.</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>If aiDrivenAnalyticsSettings is absent from the diagnosis, flag needs_manual_review to confirm whether Cobuild/AI Assistants is enabled for this customer.</t>
-        </is>
-      </c>
-      <c r="P3" s="3" t="n"/>
-      <c r="Q3" s="3" t="inlineStr">
-        <is>
-          <t>Cobuild, AI Assistants, Agent building</t>
-        </is>
-      </c>
-      <c r="R3" s="3" t="inlineStr">
-        <is>
-          <t>generative_ai_acceleration</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="inlineStr">
-        <is>
-          <t>7, 8, 9</t>
-        </is>
-      </c>
-      <c r="T3" s="3" t="inlineStr">
-        <is>
-          <t>Cobuild; Cobuild; Instance Diags / DiagParser3</t>
-        </is>
-      </c>
-      <c r="U3" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="V3" s="3" t="n"/>
-      <c r="W3" s="3" t="n"/>
-      <c r="X3" s="3" t="n"/>
-      <c r="Y3" s="3" t="n"/>
-      <c r="Z3" s="3" t="n"/>
-      <c r="AA3" s="3" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>GENAI-009</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>nice_to_have</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>qualitative_practice</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Agent Hub</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Agent Hub Deployment Required Permissions</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Before a user can deploy an Agent Hub instance, they must have permissions for writing project content in the hosting project, writing isolated code execution, WebApp impersonation, and (if Quick agents are enabled) create projects; alternatively the user could be a DSS administrator, though a dedicated service account is preferred.</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Grant Agent Hub deployers write project content, isolated code execution, and webapp impersonation permissions.</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>Administration &gt; Security &gt; Groups shows the Agent Hub deployer's group granted 'Write project content', 'Write isolated code execution', and 'WebApp impersonation' permissions (plus 'Create projects' if Quick agents are enabled), or the deployer is a DSS admin/service account.</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>The deployer's group lacks one or more of these permissions and is not an admin/service account, or logs show 'Not authorized' errors when creating the Agent Hub WebApp.</t>
-        </is>
-      </c>
-      <c r="O4" s="3" t="inlineStr">
-        <is>
-          <t>If the diagnosis file lacks per-user/group permission detail, flag needs_manual_review and recommend checking Administration &gt; Security &gt; Groups directly.</t>
-        </is>
-      </c>
-      <c r="P4" s="3" t="inlineStr">
-        <is>
-          <t>Missing permissions cause deployment failures such as 'Not authorized' errors when creating the Agent Hub WebApp.</t>
-        </is>
-      </c>
-      <c r="Q4" s="3" t="inlineStr">
-        <is>
-          <t>Agent Hub, Permissions, Groups, WebApp</t>
-        </is>
-      </c>
-      <c r="R4" s="3" t="inlineStr">
-        <is>
-          <t>generative_ai_acceleration</t>
-        </is>
-      </c>
-      <c r="S4" s="3" t="inlineStr">
-        <is>
-          <t>10, 11, 12</t>
-        </is>
-      </c>
-      <c r="T4" s="3" t="inlineStr">
-        <is>
-          <t>Agent Hub NICE TO HAVE:; Writing isolated code execution; WebApp impersonation</t>
-        </is>
-      </c>
-      <c r="U4" s="3" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="V4" s="3" t="inlineStr">
-        <is>
-          <t>Although the parent topic is tagged NICE TO HAVE, the described permission requirements are phrased as mandatory ('must have permissions') for successful deployment; classification follows the explicit heading tag.</t>
-        </is>
-      </c>
-      <c r="W4" s="3" t="n"/>
-      <c r="X4" s="3" t="n"/>
-      <c r="Y4" s="3" t="n"/>
-      <c r="Z4" s="3" t="n"/>
-      <c r="AA4" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Release 0.30.0: reader 0.12.0 (sanity_check), SCALE-006 calibration (present = Pass, missing or empty = Fail), fixtures and tests
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/checklists/eval_checklist.xlsx
+++ b/tests/fixtures/checklists/eval_checklist.xlsx
@@ -3029,7 +3029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA10"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3625,12 +3625,12 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>SCALE-007</t>
+          <t>SCALE-006</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -3640,22 +3640,22 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Log Monitoring</t>
+          <t>Instance Sanity Check</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Backend.log Error Review</t>
+          <t>Usage of Instance Sanity Check</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Review recent backend.log files (including rotated/zipped logs) for ERROR or FATAL level entries indicating systemic issues such as repeating stack traces, connection failures, or plugin crashes; investigate patterns that recur frequently even without explicit user complaints.</t>
+          <t>Verify that the Instance Sanity Check feature is used to detect instance configuration problems, accessible via Administration &gt; Maintenance &gt; Instance Sanity Check.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Review backend.log for recurring ERROR/FATAL entries indicating systemic stability issues.</t>
+          <t>Use Instance Sanity Check periodically to detect instance configuration problems.</t>
         </is>
       </c>
       <c r="H6" s="3" t="n"/>
@@ -3665,27 +3665,27 @@
       <c r="L6" s="3" t="n"/>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>backend.log and rotated logs show few or no ERROR/FATAL entries, or only isolated non-recurring errors; AI Log Analysis in DiagParser3 shows no systemic issue flagged.</t>
+          <t>Evidence that the customer has run the Instance Sanity Check periodically and addressed reported issues (e.g., DiagParser3 sanity check output showing no unresolved critical issues).</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>Frequent recurring ERROR/FATAL entries (e.g., the same stack trace dozens of times per day), repeated connection failures, or plugin crashes.</t>
+          <t>No record of Instance Sanity Check usage, or reported issues left unresolved for extended periods.</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>If logs aren't included or available in the diagnosis bundle, flag needs_manual_review and request the backend.log files directly.</t>
+          <t>If the diagnosis doesn't include sanity check results, flag needs_manual_review and check DiagParser3 or the Administration UI directly.</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>A high volume of repeated errors often points to a systemic issue that needs to be addressed before it impacts instance stability.</t>
+          <t>Regular use helps proactively detect instance configuration issues before they cause problems.</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>backend.log, AI Log Analysis, DiagParser3</t>
+          <t>Instance Sanity Check</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
@@ -3695,17 +3695,17 @@
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>6, 7</t>
+          <t>5, 6</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>Backend.log Errors | MUST HAVE; Backend.log Errors | MUST HAVE</t>
+          <t>Usage of Instance Sanity Check | NICE TO HAVE; Usage of Instance Sanity Check | NICE TO HAVE</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="V6" s="3" t="n"/>
@@ -3718,7 +3718,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>SCALE-008</t>
+          <t>SCALE-007</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -3728,77 +3728,57 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>specific_setting</t>
+          <t>qualitative_practice</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Memory Sizing</t>
+          <t>Log Monitoring</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Backend Xmx Sizing</t>
+          <t>Backend.log Error Review</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>backend.xmx must be appropriately sized for the deployment based on system memory (Cloud Stacks heuristic: 4g for &gt;12GB RAM, 8g for &gt;30GB RAM, 16g for &gt;95GB RAM, more for larger deployments), and should be at least 3x the size of the configuration folder. jek.xmx and fek.xmx should also be checked to ensure they haven't been oversized, and backend.log should be checked for OutOfMemoryError entries.</t>
+          <t>Review recent backend.log files (including rotated/zipped logs) for ERROR or FATAL level entries indicating systemic issues such as repeating stack traces, connection failures, or plugin crashes; investigate patterns that recur frequently even without explicit user complaints.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Size backend.xmx per the memory heuristic, at least 3x the config folder size.</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>install.ini &gt; backend.xmx</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>greater_than_or_equal</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>per Cloud Stacks heuristic tier (4g/8g/16g based on system RAM) and &gt;=3x config folder size</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t>Also verify jek.xmx/fek.xmx are not oversized, and that xmx avoids the 32GB&lt;=xmx&lt;48GB dead zone (jump to 48GB instead) due to Java Ordinary Object Pointer behavior.</t>
-        </is>
-      </c>
+          <t>Review backend.log for recurring ERROR/FATAL entries indicating systemic stability issues.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>install.ini backend.xmx matches or exceeds the recommended tier for system memory, is &gt;=3x config folder size, and avoids the 32-48GB dead zone; no OutOfMemoryError entries in backend.log.</t>
+          <t>backend.log and rotated logs show few or no ERROR/FATAL entries, or only isolated non-recurring errors; AI Log Analysis in DiagParser3 shows no systemic issue flagged.</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>backend.xmx set below the recommended heuristic, falls in the 32GB-48GB dead zone, or backend.log shows recurring 'OutOfMemoryError: Java heap space' / 'OutOfMemoryError: GC Overhead limit exceeded' entries.</t>
+          <t>Frequent recurring ERROR/FATAL entries (e.g., the same stack trace dozens of times per day), repeated connection failures, or plugin crashes.</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>If install.ini or system memory info is not present in the diagnosis, flag needs_manual_review and request system specs and install.ini contents.</t>
+          <t>If logs aren't included or available in the diagnosis bundle, flag needs_manual_review and request the backend.log files directly.</t>
         </is>
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>Insufficient or misconfigured heap sizing leads to OutOfMemory errors and instability; oversizing into the 32-48GB range paradoxically reduces available memory due to JVM pointer compression behavior.</t>
+          <t>A high volume of repeated errors often points to a systemic issue that needs to be addressed before it impacts instance stability.</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>backend.xmx, jek.xmx, fek.xmx, JVM memory, OutOfMemoryError</t>
+          <t>backend.log, AI Log Analysis, DiagParser3</t>
         </is>
       </c>
       <c r="R7" s="3" t="inlineStr">
@@ -3808,12 +3788,12 @@
       </c>
       <c r="S7" s="3" t="inlineStr">
         <is>
-          <t>7, 8</t>
+          <t>6, 7</t>
         </is>
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>Backend Xmx | MUST HAVE; Backend Xmx | MUST HAVE</t>
+          <t>Backend.log Errors | MUST HAVE; Backend.log Errors | MUST HAVE</t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr">
@@ -3831,7 +3811,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>SCALE-009</t>
+          <t>SCALE-008</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -3846,68 +3826,72 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Flow Parallelism Limits</t>
+          <t>Memory Sizing</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Flow Limits Sizing (Max Jobs, Max Activities)</t>
+          <t>Backend Xmx Sizing</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Configure Flow concurrency limits using the 5-step sizing framework: reserve OS/backend.xmx memory, allocate roughly 70% of remaining memory to CGroups (less if offloading heavy workloads to EKS/Kubernetes), size Max Jobs from the remaining JEK memory, set the global Max Activities limit (30-50) as a backstop above Max Jobs, and leave Max Activities per Job at the default of 5. Max Jobs must never be set to 0, as this disables the limit entirely and risks crashing the instance via OOM.</t>
+          <t>backend.xmx must be appropriately sized for the deployment based on system memory (Cloud Stacks heuristic: 4g for &gt;12GB RAM, 8g for &gt;30GB RAM, 16g for &gt;95GB RAM, more for larger deployments), and should be at least 3x the size of the configuration folder. jek.xmx and fek.xmx should also be checked to ensure they haven't been oversized, and backend.log should be checked for OutOfMemoryError entries.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Size Max Jobs and Max Activities via the memory framework; never set Max Jobs to zero.</t>
+          <t>Size backend.xmx per the memory heuristic, at least 3x the config folder size.</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; maxRunningJobs</t>
+          <t>install.ini &gt; backend.xmx</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>not_equals</t>
+          <t>greater_than_or_equal</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="n"/>
+          <t>per Cloud Stacks heuristic tier (4g/8g/16g based on system RAM) and &gt;=3x config folder size</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>Also verify general-settings.json &gt; maxRunningActivities falls within 30-50, and maxRunningActivitiesPerJob is at the default of 5 unless justified. Front-end equivalent: Administration &gt; Settings &gt; Resources control &gt; Concurrent Activities.</t>
+          <t>Also verify jek.xmx/fek.xmx are not oversized, and that xmx avoids the 32GB&lt;=xmx&lt;48GB dead zone (jump to 48GB instead) due to Java Ordinary Object Pointer behavior.</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>maxRunningJobs set to a positive nonzero value derived from the 5-step memory sizing framework; maxRunningActivities within 30-50; maxRunningActivitiesPerJob at 5 (or a justified alternative).</t>
+          <t>install.ini backend.xmx matches or exceeds the recommended tier for system memory, is &gt;=3x config folder size, and avoids the 32-48GB dead zone; no OutOfMemoryError entries in backend.log.</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>maxRunningJobs is 0 or blank (critical stability risk); maxRunningActivities is outside 30-50 without justification; sizing doesn't account for available host memory, risking OOM.</t>
+          <t>backend.xmx set below the recommended heuristic, falls in the 32GB-48GB dead zone, or backend.log shows recurring 'OutOfMemoryError: Java heap space' / 'OutOfMemoryError: GC Overhead limit exceeded' entries.</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>If these general-settings.json values are missing from the diagnosis, flag needs_manual_review and check the Administration &gt; Settings &gt; Resources control UI directly.</t>
+          <t>If install.ini or system memory info is not present in the diagnosis, flag needs_manual_review and request system specs and install.ini contents.</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>Improperly sized flow limits risk instance-wide Out-Of-Memory crashes; Max Jobs=0 disables protection entirely.</t>
+          <t>Insufficient or misconfigured heap sizing leads to OutOfMemory errors and instability; oversizing into the 32-48GB range paradoxically reduces available memory due to JVM pointer compression behavior.</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>Flow limits, Max Jobs, Max Activities, CGroups, JEK, memory sizing</t>
+          <t>backend.xmx, jek.xmx, fek.xmx, JVM memory, OutOfMemoryError</t>
         </is>
       </c>
       <c r="R8" s="3" t="inlineStr">
@@ -3917,12 +3901,12 @@
       </c>
       <c r="S8" s="3" t="inlineStr">
         <is>
-          <t>8, 9, 10, 11</t>
+          <t>7, 8</t>
         </is>
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>Flow parallelism | MUST HAVE; Flow parallelism | MUST HAVE; Flow parallelism | MUST HAVE; Flow parallelism | MUST HAVE</t>
+          <t>Backend Xmx | MUST HAVE; Backend Xmx | MUST HAVE</t>
         </is>
       </c>
       <c r="U8" s="3" t="inlineStr">
@@ -3940,12 +3924,12 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>SCALE-010</t>
+          <t>SCALE-009</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>nice_to_have</t>
+          <t>must_have</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -3955,68 +3939,68 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Default Connection &amp; Engine Preferences</t>
+          <t>Flow Parallelism Limits</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Preferred Connections and Engines Settings</t>
+          <t>Flow Limits Sizing (Max Jobs, Max Activities)</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Default dataset creation settings and recipe engine preferences (preferedConnection, forcedPreferedConnection, preferedUploadConnection, preferedStorageFormats) are blank by default and should remain so unless a specific use case justifies setting them; in particular, preferred engine should almost always be left blank for v12+ instances since altering it can cause breaking changes.</t>
+          <t>Configure Flow concurrency limits using the 5-step sizing framework: reserve OS/backend.xmx memory, allocate roughly 70% of remaining memory to CGroups (less if offloading heavy workloads to EKS/Kubernetes), size Max Jobs from the remaining JEK memory, set the global Max Activities limit (30-50) as a backstop above Max Jobs, and leave Max Activities per Job at the default of 5. Max Jobs must never be set to 0, as this disables the limit entirely and risks crashing the instance via OOM.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Leave default connection and engine preferences blank unless a specific use case justifies them.</t>
+          <t>Size Max Jobs and Max Activities via the memory framework; never set Max Jobs to zero.</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; defaultDatasetCreationSettings / recipeEnginesPreferences (preferedConnection, forcedPreferedConnection, preferedUploadConnection, preferedStorageFormats)</t>
+          <t>general-settings.json &gt; maxRunningJobs</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>equals</t>
+          <t>not_equals</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>unset/blank unless justified specific use case</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K9" s="3" t="n"/>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>These keys may be entirely absent from general-settings.json if left blank, which is the expected default state.</t>
+          <t>Also verify general-settings.json &gt; maxRunningActivities falls within 30-50, and maxRunningActivitiesPerJob is at the default of 5 unless justified. Front-end equivalent: Administration &gt; Settings &gt; Resources control &gt; Concurrent Activities.</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>Keys absent or blank in general-settings.json, or if set, a documented specific use case justifies the value (e.g., not forcing storage to a local server).</t>
+          <t>maxRunningJobs set to a positive nonzero value derived from the 5-step memory sizing framework; maxRunningActivities within 30-50; maxRunningActivitiesPerJob at 5 (or a justified alternative).</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>preferedConnection/forcedPreferedConnection set to force local server storage, or preferred engine changed without clear justification, especially on v12+ instances.</t>
+          <t>maxRunningJobs is 0 or blank (critical stability risk); maxRunningActivities is outside 30-50 without justification; sizing doesn't account for available host memory, risking OOM.</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>If this section of general-settings.json is missing from the diagnosis, flag needs_manual_review and check the Administration &gt; Settings &gt; Engines &amp; connections UI.</t>
+          <t>If these general-settings.json values are missing from the diagnosis, flag needs_manual_review and check the Administration &gt; Settings &gt; Resources control UI directly.</t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>These settings default to blank for good reason; forcing values can cause breaking changes or performance issues (e.g., forcing local storage).</t>
+          <t>Improperly sized flow limits risk instance-wide Out-Of-Memory crashes; Max Jobs=0 disables protection entirely.</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>default dataset creation, recipe engine preferences, connections</t>
+          <t>Flow limits, Max Jobs, Max Activities, CGroups, JEK, memory sizing</t>
         </is>
       </c>
       <c r="R9" s="3" t="inlineStr">
@@ -4026,24 +4010,20 @@
       </c>
       <c r="S9" s="3" t="inlineStr">
         <is>
-          <t>12, 13, 14</t>
+          <t>8, 9, 10, 11</t>
         </is>
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>Preferreds and Defaults | NICE TO HAVE; Preferreds and Defaults | NICE TO HAVE; Preferreds and Defaults | NICE TO HAVE</t>
+          <t>Flow parallelism | MUST HAVE; Flow parallelism | MUST HAVE; Flow parallelism | MUST HAVE; Flow parallelism | MUST HAVE</t>
         </is>
       </c>
       <c r="U9" s="3" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="V9" s="3" t="inlineStr">
-        <is>
-          <t>Expected value is contextual ('reasonable values' if set), not a fixed constant, so the check requires judgment.</t>
-        </is>
-      </c>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V9" s="3" t="n"/>
       <c r="W9" s="3" t="n"/>
       <c r="X9" s="3" t="n"/>
       <c r="Y9" s="3" t="n"/>
@@ -4053,12 +4033,12 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>SCALE-011</t>
+          <t>SCALE-010</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -4068,68 +4048,68 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Connections Hygiene</t>
+          <t>Default Connection &amp; Engine Preferences</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Remove filesystem_root Connection</t>
+          <t>Preferred Connections and Engines Settings</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>The default filesystem_root connection pointing to the server's root filesystem should be removed unless actively used by a project; if in use, propose a dedicated scoped connection to the specific path before removing filesystem_root.</t>
+          <t>Default dataset creation settings and recipe engine preferences (preferedConnection, forcedPreferedConnection, preferedUploadConnection, preferedStorageFormats) are blank by default and should remain so unless a specific use case justifies setting them; in particular, preferred engine should almost always be left blank for v12+ instances since altering it can cause breaking changes.</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Remove the filesystem_root connection unless actively used, replacing it with a scoped connection.</t>
+          <t>Leave default connection and engine preferences blank unless a specific use case justifies them.</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>connections.json &gt; filesystem_root</t>
+          <t>general-settings.json &gt; defaultDatasetCreationSettings / recipeEnginesPreferences (preferedConnection, forcedPreferedConnection, preferedUploadConnection, preferedStorageFormats)</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>not_exists</t>
+          <t>equals</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>removed (unless replaced by a scoped connection after confirming no active project usage)</t>
+          <t>unset/blank unless justified specific use case</t>
         </is>
       </c>
       <c r="K10" s="3" t="n"/>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>Check usage via Administration -&gt; Monitoring before deletion.</t>
+          <t>These keys may be entirely absent from general-settings.json if left blank, which is the expected default state.</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>filesystem_root connection absent from the connections list, or confirmed unused and removed; if it was in use, a dedicated scoped connection was created to replace it.</t>
+          <t>Keys absent or blank in general-settings.json, or if set, a documented specific use case justifies the value (e.g., not forcing storage to a local server).</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>filesystem_root connection still present and either unused (should have been deleted) or in use without a safer scoped replacement.</t>
+          <t>preferedConnection/forcedPreferedConnection set to force local server storage, or preferred engine changed without clear justification, especially on v12+ instances.</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>If the connections list isn't in the diagnosis, flag needs_manual_review and check the Administration &gt; Connections UI directly.</t>
+          <t>If this section of general-settings.json is missing from the diagnosis, flag needs_manual_review and check the Administration &gt; Settings &gt; Engines &amp; connections UI.</t>
         </is>
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>The filesystem_root connection exposes the entire server filesystem, posing a security and stability risk.</t>
+          <t>These settings default to blank for good reason; forcing values can cause breaking changes or performance issues (e.g., forcing local storage).</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>connections, filesystem_root, security</t>
+          <t>default dataset creation, recipe engine preferences, connections</t>
         </is>
       </c>
       <c r="R10" s="3" t="inlineStr">
@@ -4139,25 +4119,138 @@
       </c>
       <c r="S10" s="3" t="inlineStr">
         <is>
-          <t>14, 15</t>
+          <t>12, 13, 14</t>
         </is>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>Remove filesystem_root connection | MUST HAVE; Remove filesystem_root connection | MUST HAVE</t>
+          <t>Preferreds and Defaults | NICE TO HAVE; Preferreds and Defaults | NICE TO HAVE; Preferreds and Defaults | NICE TO HAVE</t>
         </is>
       </c>
       <c r="U10" s="3" t="inlineStr">
         <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="V10" s="3" t="n"/>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V10" s="3" t="inlineStr">
+        <is>
+          <t>Expected value is contextual ('reasonable values' if set), not a fixed constant, so the check requires judgment.</t>
+        </is>
+      </c>
       <c r="W10" s="3" t="n"/>
       <c r="X10" s="3" t="n"/>
       <c r="Y10" s="3" t="n"/>
       <c r="Z10" s="3" t="n"/>
       <c r="AA10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>SCALE-011</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Connections Hygiene</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Remove filesystem_root Connection</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>The default filesystem_root connection pointing to the server's root filesystem should be removed unless actively used by a project; if in use, propose a dedicated scoped connection to the specific path before removing filesystem_root.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Remove the filesystem_root connection unless actively used, replacing it with a scoped connection.</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>connections.json &gt; filesystem_root</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>not_exists</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>removed (unless replaced by a scoped connection after confirming no active project usage)</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="n"/>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>Check usage via Administration -&gt; Monitoring before deletion.</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>filesystem_root connection absent from the connections list, or confirmed unused and removed; if it was in use, a dedicated scoped connection was created to replace it.</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>filesystem_root connection still present and either unused (should have been deleted) or in use without a safer scoped replacement.</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>If the connections list isn't in the diagnosis, flag needs_manual_review and check the Administration &gt; Connections UI directly.</t>
+        </is>
+      </c>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>The filesystem_root connection exposes the entire server filesystem, posing a security and stability risk.</t>
+        </is>
+      </c>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>connections, filesystem_root, security</t>
+        </is>
+      </c>
+      <c r="R11" s="3" t="inlineStr">
+        <is>
+          <t>scalable_performance_ops</t>
+        </is>
+      </c>
+      <c r="S11" s="3" t="inlineStr">
+        <is>
+          <t>14, 15</t>
+        </is>
+      </c>
+      <c r="T11" s="3" t="inlineStr">
+        <is>
+          <t>Remove filesystem_root connection | MUST HAVE; Remove filesystem_root connection | MUST HAVE</t>
+        </is>
+      </c>
+      <c r="U11" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V11" s="3" t="n"/>
+      <c r="W11" s="3" t="n"/>
+      <c r="X11" s="3" t="n"/>
+      <c r="Y11" s="3" t="n"/>
+      <c r="Z11" s="3" t="n"/>
+      <c r="AA11" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Release 0.36.0: verdicts Batch 4b (GENAI-001/003/004/005/006/007/009), reader 0.17.0
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/checklists/eval_checklist.xlsx
+++ b/tests/fixtures/checklists/eval_checklist.xlsx
@@ -2332,7 +2332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA6"/>
+  <dimension ref="A1:AA8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2613,7 +2613,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>GENAI-005</t>
+          <t>GENAI-003</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -2628,27 +2628,27 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Bring Your Own LLM Mode</t>
+          <t>Trace Explorer</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Bring Your Own LLM Mode - Reference Project &amp; Main Model</t>
+          <t>Trace Explorer Default Configuration</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>When Bring Your Own LLM mode is active, a Reference project key must be set (used for LLM Mesh requests running outside a DSS project, e.g. AI Search) and a main LLM model must be configured; if unset, requests will fail.</t>
+          <t>Configure Trace Explorer via Administration &gt; Settings &gt; Other &gt; LLM Mesh &gt; Configuration &gt; Trace by setting a default Project and Trace Explorer webapp instance, so the 'view traces' shortcut is functional from Prompt Studio, Agents, and Retrieval-Augmented LLMs.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Set a Reference project key and main LLM model when using Bring Your Own LLM.</t>
+          <t>Set a default project and webapp for Trace Explorer so view traces works.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; localAIServerSettings.referenceProjectKey / mainLLMId</t>
+          <t>general-settings.json &gt; generativeAISettings &gt; llmTraceSettings.traceExplorerDefaultWebApp</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -2658,30 +2658,34 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>non-empty values set for both fields</t>
+          <t>projectKey and webAppId both set to non-empty values</t>
         </is>
       </c>
       <c r="K3" s="3" t="n"/>
       <c r="L3" s="3" t="n"/>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>localAIServerSettings.useLocalServer=true with referenceProjectKey and mainLLMId populated (e.g., 'openai:openai-adrissi:gpt-5.5').</t>
+          <t>generativeAISettings.llmTraceSettings.traceExplorerDefaultWebApp present in general-settings.json with non-empty projectKey and webAppId fields.</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>useLocalServer=true but referenceProjectKey or mainLLMId missing or empty.</t>
+          <t>llmTraceSettings missing entirely, or traceExplorerDefaultWebApp present but empty/null.</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>If localAIServerSettings is absent from the diagnosis, flag needs_manual_review to confirm whether Bring Your Own LLM mode is in use.</t>
-        </is>
-      </c>
-      <c r="P3" s="3" t="n"/>
+          <t>If general-settings.json content isn't captured in the diagnosis, flag needs_manual_review to verify via the UI.</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>Without this default configuration, the trace-viewing shortcut from Prompt Studio/Agents/RAG LLMs will not function.</t>
+        </is>
+      </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>Bring Your Own LLM, AI Services, LLM Mesh</t>
+          <t>Trace Explorer, LLM Mesh, Agents</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
@@ -2691,12 +2695,12 @@
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
-          <t>5, 6</t>
+          <t>3, 4</t>
         </is>
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>Bring your own LLM Mode; Instance Diags / DiagParser3</t>
+          <t>Trace Explorer MUST HAVE:; Instance Diags / DiagParser3</t>
         </is>
       </c>
       <c r="U3" s="3" t="inlineStr">
@@ -2714,7 +2718,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>GENAI-006</t>
+          <t>GENAI-004</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -2729,68 +2733,64 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Bring Your Own LLM Mode</t>
+          <t>AI Services</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Bring Your Own LLM - Recommended Model Versions</t>
+          <t>AI Services Terms of Use Acceptance &amp; Enablement</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>If the customer has activated Bring Your Own LLM Mode for AI Assistants, verify they are using recommended model versions (minimum OpenAI ChatGPT 5.2) and avoid unsupported ones (e.g., ChatGPT 5.1, which will not provide good results).</t>
+          <t>Verify that the customer has accepted the Dataiku AI Services Terms of Use and that AI Services are enabled by the admin in Administration &gt; AI Services. Confirm outbound internet connectivity to https://ai-gateway.api-services.dataiku.io, required in both 'Operated by Dataiku' and 'Bring your own LLM' modes.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Use at least ChatGPT 5.2 for Bring Your Own LLM; avoid version 5.1.</t>
+          <t>Confirm AI Services Terms of Use are accepted and AI Services are enabled.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; localAIServerSettings.mainLLMId (and responseFormatAwareLLMId/fastLightLLMId)</t>
+          <t>general-settings.json &gt; dataikuAIServicesTermsOfUseAccepted / enabled</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>not_equals</t>
+          <t>equals</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>ChatGPT 5.1 or earlier / unsupported model versions</t>
+          <t>true</t>
         </is>
       </c>
       <c r="K4" s="3" t="n"/>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>Exact version comparison against the recommended minimum (ChatGPT 5.2) may require manual judgment; refer to https://doc.dataiku.com/dss/latest/ai-assistants/setup.html#bring-your-own-llm-mode.</t>
+          <t>Also check byoTermsOfUseAccepted for Bring-your-own-LLM mode. Internet whitelisting of ai-gateway.api-services.dataiku.io is not verifiable from diagnosis JSON alone.</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>mainLLMId/related LLM IDs reference gpt-5.2 or later.</t>
+          <t>general-settings.json shows dataikuAIServicesTermsOfUseAccepted=true and enabled=true.</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>mainLLMId/related LLM IDs reference gpt-5.1 or an older/unsupported model.</t>
+          <t>enabled=false or Terms of Use not accepted while AI Services usage is expected/observed.</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>If the model identifier is ambiguous, non-OpenAI, or version cannot be determined, flag needs_manual_review and reference the setup documentation.</t>
-        </is>
-      </c>
-      <c r="P4" s="3" t="inlineStr">
-        <is>
-          <t>Using unsupported model versions is stated to produce poor results.</t>
-        </is>
-      </c>
+          <t>If AI Services keys are absent from the diagnosis, treat as not enabled and flag needs_manual_review to confirm with the customer whether AI Services usage is intended.</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="n"/>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Bring Your Own LLM, Model selection, AI Assistants</t>
+          <t>AI Services, Terms of Use, LLM Mesh</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
@@ -2800,17 +2800,17 @@
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>6, 7</t>
+          <t>4, 5</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>Bring your own LLM Mode; Bring your own LLM Mode</t>
+          <t>AI Services NICE TO HAVE:; Instance Diags / DiagParser3</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="V4" s="3" t="n"/>
@@ -2823,7 +2823,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>GENAI-007</t>
+          <t>GENAI-005</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -2838,27 +2838,27 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Cobuild</t>
+          <t>Bring Your Own LLM Mode</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Cobuild Default LLM Configuration</t>
+          <t>Bring Your Own LLM Mode - Reference Project &amp; Main Model</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Administrators must configure default LLM settings for Cobuild (agent-building tools) upon activation of AI Assistants, including defaultEmbeddingLLMId, defaultLLMId, and defaultImageGenerationLLMId under agentBuildingSettings; if unset, Cobuild's building-agent tools will fail and instruct users to contact an administrator.</t>
+          <t>When Bring Your Own LLM mode is active, a Reference project key must be set (used for LLM Mesh requests running outside a DSS project, e.g. AI Search) and a main LLM model must be configured; if unset, requests will fail.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Configure default embedding, LLM, and image-generation models for Cobuild agent building.</t>
+          <t>Set a Reference project key and main LLM model when using Bring Your Own LLM.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; aiDrivenAnalyticsSettings.agentBuildingSettings.{defaultEmbeddingLLMId, defaultLLMId, defaultImageGenerationLLMId}</t>
+          <t>general-settings.json &gt; localAIServerSettings.referenceProjectKey / mainLLMId</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -2868,30 +2868,30 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>all three fields populated with valid LLM IDs</t>
+          <t>non-empty values set for both fields</t>
         </is>
       </c>
       <c r="K5" s="3" t="n"/>
       <c r="L5" s="3" t="n"/>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>agentBuildingSettings block shows non-empty defaultEmbeddingLLMId, defaultLLMId, and defaultImageGenerationLLMId values.</t>
+          <t>localAIServerSettings.useLocalServer=true with referenceProjectKey and mainLLMId populated (e.g., 'openai:openai-adrissi:gpt-5.5').</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>One or more of these fields is missing or empty while Cobuild/AI Assistants is enabled.</t>
+          <t>useLocalServer=true but referenceProjectKey or mainLLMId missing or empty.</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>If aiDrivenAnalyticsSettings is absent from the diagnosis, flag needs_manual_review to confirm whether Cobuild/AI Assistants is enabled for this customer.</t>
+          <t>If localAIServerSettings is absent from the diagnosis, flag needs_manual_review to confirm whether Bring Your Own LLM mode is in use.</t>
         </is>
       </c>
       <c r="P5" s="3" t="n"/>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>Cobuild, AI Assistants, Agent building</t>
+          <t>Bring Your Own LLM, AI Services, LLM Mesh</t>
         </is>
       </c>
       <c r="R5" s="3" t="inlineStr">
@@ -2901,12 +2901,12 @@
       </c>
       <c r="S5" s="3" t="inlineStr">
         <is>
-          <t>7, 8, 9</t>
+          <t>5, 6</t>
         </is>
       </c>
       <c r="T5" s="3" t="inlineStr">
         <is>
-          <t>Cobuild; Cobuild; Instance Diags / DiagParser3</t>
+          <t>Bring your own LLM Mode; Instance Diags / DiagParser3</t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr">
@@ -2924,7 +2924,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>GENAI-009</t>
+          <t>GENAI-006</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -2934,57 +2934,73 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>qualitative_practice</t>
+          <t>specific_setting</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Agent Hub</t>
+          <t>Bring Your Own LLM Mode</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Agent Hub Deployment Required Permissions</t>
+          <t>Bring Your Own LLM - Recommended Model Versions</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Before a user can deploy an Agent Hub instance, they must have permissions for writing project content in the hosting project, writing isolated code execution, WebApp impersonation, and (if Quick agents are enabled) create projects; alternatively the user could be a DSS administrator, though a dedicated service account is preferred.</t>
+          <t>If the customer has activated Bring Your Own LLM Mode for AI Assistants, verify they are using recommended model versions (minimum OpenAI ChatGPT 5.2) and avoid unsupported ones (e.g., ChatGPT 5.1, which will not provide good results).</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Grant Agent Hub deployers write project content, isolated code execution, and webapp impersonation permissions.</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
+          <t>Use at least ChatGPT 5.2 for Bring Your Own LLM; avoid version 5.1.</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; localAIServerSettings.mainLLMId (and responseFormatAwareLLMId/fastLightLLMId)</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>not_equals</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>ChatGPT 5.1 or earlier / unsupported model versions</t>
+        </is>
+      </c>
       <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Exact version comparison against the recommended minimum (ChatGPT 5.2) may require manual judgment; refer to https://doc.dataiku.com/dss/latest/ai-assistants/setup.html#bring-your-own-llm-mode.</t>
+        </is>
+      </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>Administration &gt; Security &gt; Groups shows the Agent Hub deployer's group granted 'Write project content', 'Write isolated code execution', and 'WebApp impersonation' permissions (plus 'Create projects' if Quick agents are enabled), or the deployer is a DSS admin/service account.</t>
+          <t>mainLLMId/related LLM IDs reference gpt-5.2 or later.</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>The deployer's group lacks one or more of these permissions and is not an admin/service account, or logs show 'Not authorized' errors when creating the Agent Hub WebApp.</t>
+          <t>mainLLMId/related LLM IDs reference gpt-5.1 or an older/unsupported model.</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file lacks per-user/group permission detail, flag needs_manual_review and recommend checking Administration &gt; Security &gt; Groups directly.</t>
+          <t>If the model identifier is ambiguous, non-OpenAI, or version cannot be determined, flag needs_manual_review and reference the setup documentation.</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>Missing permissions cause deployment failures such as 'Not authorized' errors when creating the Agent Hub WebApp.</t>
+          <t>Using unsupported model versions is stated to produce poor results.</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>Agent Hub, Permissions, Groups, WebApp</t>
+          <t>Bring Your Own LLM, Model selection, AI Assistants</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
@@ -2994,12 +3010,12 @@
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>10, 11, 12</t>
+          <t>6, 7</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>Agent Hub NICE TO HAVE:; Writing isolated code execution; WebApp impersonation</t>
+          <t>Bring your own LLM Mode; Bring your own LLM Mode</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
@@ -3007,16 +3023,210 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="V6" s="3" t="inlineStr">
-        <is>
-          <t>Although the parent topic is tagged NICE TO HAVE, the described permission requirements are phrased as mandatory ('must have permissions') for successful deployment; classification follows the explicit heading tag.</t>
-        </is>
-      </c>
+      <c r="V6" s="3" t="n"/>
       <c r="W6" s="3" t="n"/>
       <c r="X6" s="3" t="n"/>
       <c r="Y6" s="3" t="n"/>
       <c r="Z6" s="3" t="n"/>
       <c r="AA6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>GENAI-007</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Cobuild</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Cobuild Default LLM Configuration</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Administrators must configure default LLM settings for Cobuild (agent-building tools) upon activation of AI Assistants, including defaultEmbeddingLLMId, defaultLLMId, and defaultImageGenerationLLMId under agentBuildingSettings; if unset, Cobuild's building-agent tools will fail and instruct users to contact an administrator.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Configure default embedding, LLM, and image-generation models for Cobuild agent building.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; aiDrivenAnalyticsSettings.agentBuildingSettings.{defaultEmbeddingLLMId, defaultLLMId, defaultImageGenerationLLMId}</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>exists</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>all three fields populated with valid LLM IDs</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>agentBuildingSettings block shows non-empty defaultEmbeddingLLMId, defaultLLMId, and defaultImageGenerationLLMId values.</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>One or more of these fields is missing or empty while Cobuild/AI Assistants is enabled.</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>If aiDrivenAnalyticsSettings is absent from the diagnosis, flag needs_manual_review to confirm whether Cobuild/AI Assistants is enabled for this customer.</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="n"/>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>Cobuild, AI Assistants, Agent building</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>generative_ai_acceleration</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>7, 8, 9</t>
+        </is>
+      </c>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>Cobuild; Cobuild; Instance Diags / DiagParser3</t>
+        </is>
+      </c>
+      <c r="U7" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V7" s="3" t="n"/>
+      <c r="W7" s="3" t="n"/>
+      <c r="X7" s="3" t="n"/>
+      <c r="Y7" s="3" t="n"/>
+      <c r="Z7" s="3" t="n"/>
+      <c r="AA7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>GENAI-009</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>nice_to_have</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>qualitative_practice</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub Deployment Required Permissions</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Before a user can deploy an Agent Hub instance, they must have permissions for writing project content in the hosting project, writing isolated code execution, WebApp impersonation, and (if Quick agents are enabled) create projects; alternatively the user could be a DSS administrator, though a dedicated service account is preferred.</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Grant Agent Hub deployers write project content, isolated code execution, and webapp impersonation permissions.</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="n"/>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="n"/>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="n"/>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>Administration &gt; Security &gt; Groups shows the Agent Hub deployer's group granted 'Write project content', 'Write isolated code execution', and 'WebApp impersonation' permissions (plus 'Create projects' if Quick agents are enabled), or the deployer is a DSS admin/service account.</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>The deployer's group lacks one or more of these permissions and is not an admin/service account, or logs show 'Not authorized' errors when creating the Agent Hub WebApp.</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file lacks per-user/group permission detail, flag needs_manual_review and recommend checking Administration &gt; Security &gt; Groups directly.</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>Missing permissions cause deployment failures such as 'Not authorized' errors when creating the Agent Hub WebApp.</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub, Permissions, Groups, WebApp</t>
+        </is>
+      </c>
+      <c r="R8" s="3" t="inlineStr">
+        <is>
+          <t>generative_ai_acceleration</t>
+        </is>
+      </c>
+      <c r="S8" s="3" t="inlineStr">
+        <is>
+          <t>10, 11, 12</t>
+        </is>
+      </c>
+      <c r="T8" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub NICE TO HAVE:; Writing isolated code execution; WebApp impersonation</t>
+        </is>
+      </c>
+      <c r="U8" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V8" s="3" t="inlineStr">
+        <is>
+          <t>Although the parent topic is tagged NICE TO HAVE, the described permission requirements are phrased as mandatory ('must have permissions') for successful deployment; classification follows the explicit heading tag.</t>
+        </is>
+      </c>
+      <c r="W8" s="3" t="n"/>
+      <c r="X8" s="3" t="n"/>
+      <c r="Y8" s="3" t="n"/>
+      <c r="Z8" s="3" t="n"/>
+      <c r="AA8" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Release 0.38.0: verdicts Batch 4a (ARCH-005/006/007/010/011/013/016/017), reader 0.19.0
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/checklists/eval_checklist.xlsx
+++ b/tests/fixtures/checklists/eval_checklist.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA9"/>
+  <dimension ref="A1:AA14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -985,12 +985,12 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>ARCH-006</t>
+          <t>ARCH-005</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>nice_to_have</t>
+          <t>must_have</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -1005,63 +1005,63 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Baseline Spark Configuration Set (High/Standard/Large-memory/High I/O)</t>
+          <t>Valid Spark Configuration for Spark Jobs</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Dataiku recommends defining multiple named Spark configurations as a tunable baseline: a default Standard config for recipes and notebooks, a High config for higher parallelism, a Large memory config for the largest jobs, and an optional High I/O config for read/write-heavy workloads with a high cores-to-memory ratio.</t>
+          <t>Environments that run Spark jobs must have a valid Spark configuration set (general-settings.json under sparkSettings, or via Administration &gt; Settings &gt; Spark); the specific example values Dataiku provides are only a baseline, not a strict requirement, but a workable config must exist wherever Spark is used.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Define Standard, High, Large-memory, and optional High I/O Spark configurations as a baseline.</t>
+          <t>Configure a valid Spark configuration in sparkSettings wherever Spark jobs run.</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; sparkSettings (named spark configs)</t>
+          <t>general-settings.json &gt; sparkSettings</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>one_of</t>
+          <t>exists</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Standard/High/Large-memory baseline configs, plus optional High I/O config, as documented</t>
+          <t>valid spark configuration present</t>
         </is>
       </c>
       <c r="K6" s="3" t="n"/>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>Baseline reference values: Standard config - spark.executor.instances=4, spark.executor.memory=6g, spark.executor.cores=2, spark.kubernetes.memoryOverheadFactor=0.4, spark.driver.memory=1g, spark.sql.shuffle.partitions=40, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. High config - spark.executor.instances=12, spark.executor.memory=6g, spark.executor.cores=2, spark.kubernetes.memoryOverheadFactor=0.4, spark.driver.memory=1g, spark.sql.shuffle.partitions=80, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. Large memory config - spark.executor.instances=4, spark.executor.memory=12g, spark.executor.cores=2, spark.kubernetes.memoryOverheadFactor=0.6, spark.driver.memory=3g, spark.sql.shuffle.partitions=80, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. Optional High I/O config (only if there is a use case for it) - spark.executor.instances=2, spark.executor.memory=16g, spark.executor.cores=8, spark.kubernetes.memoryOverheadFactor=0.4, spark.driver.memory=3g, spark.sql.shuffle.partitions=40, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. These values are guidance, not a requirement.</t>
+          <t>Required only if the environment executes Spark jobs; the specific parameter values shown by Dataiku are illustrative, not mandatory.</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>sparkSettings contains multiple named configs roughly matching these purposes (default/high-parallelism/large-memory, and optionally high I/O).</t>
+          <t>sparkSettings block is present and non-empty in general-settings.json, consistent with evidence of successful Spark job execution elsewhere in the diagnosis.</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>Only a single undifferentiated spark config exists despite varied workload needs (e.g., both lightweight recipes and large jobs run identically).</t>
+          <t>sparkSettings is missing or empty while the instance shows evidence of Spark recipes/jobs being used.</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not list multiple sparkSettings configs or describe workload diversity, flag needs_manual_review and ask about workload variety.</t>
+          <t>If the diagnosis file does not indicate whether Spark is used at all, flag needs_manual_review to confirm with the customer whether Spark jobs are run.</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>Different Spark workloads (lightweight recipes vs. large jobs vs. I/O-heavy jobs) benefit from different executor sizing and parallelism trade-offs.</t>
+          <t>Without a valid Spark config, Spark jobs cannot execute at all.</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>Spark executor, Spark configuration, Kubernetes</t>
+          <t>Spark, general-settings.json, sparkSettings</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
@@ -1071,12 +1071,12 @@
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>4, 5</t>
+          <t>3, 4</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>Define three spark configs - NICE TO HAVE; Special spark configs (only if there's use case for it)</t>
+          <t>Spark runtime configurations | MUST HAVE if running spark jobs; Spark runtime configurations | MUST HAVE if running spark jobs</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
@@ -1094,67 +1094,83 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>ARCH-008</t>
+          <t>ARCH-006</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>qualitative_practice</t>
+          <t>specific_setting</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Spark Validation</t>
+          <t>Spark Configuration</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Functional Validation of Spark Execution (Recipe &amp; Notebook)</t>
+          <t>Baseline Spark Configuration Set (High/Standard/Large-memory/High I/O)</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Reviewers should functionally validate Spark execution: run a Spark-engine recipe on Kubernetes in a test project (should succeed), and separately launch a Python/R/Scala notebook with starter Spark code and run it locally (should succeed, with Spark executor pods visible in the cluster while the code runs).</t>
+          <t>Dataiku recommends defining multiple named Spark configurations as a tunable baseline: a default Standard config for recipes and notebooks, a High config for higher parallelism, a Large memory config for the largest jobs, and an optional High I/O config for read/write-heavy workloads with a high cores-to-memory ratio.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Validate Spark execution by successfully running a test Spark recipe and notebook.</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
+          <t>Define Standard, High, Large-memory, and optional High I/O Spark configurations as a baseline.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; sparkSettings (named spark configs)</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>one_of</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Standard/High/Large-memory baseline configs, plus optional High I/O config, as documented</t>
+        </is>
+      </c>
       <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Baseline reference values: Standard config - spark.executor.instances=4, spark.executor.memory=6g, spark.executor.cores=2, spark.kubernetes.memoryOverheadFactor=0.4, spark.driver.memory=1g, spark.sql.shuffle.partitions=40, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. High config - spark.executor.instances=12, spark.executor.memory=6g, spark.executor.cores=2, spark.kubernetes.memoryOverheadFactor=0.4, spark.driver.memory=1g, spark.sql.shuffle.partitions=80, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. Large memory config - spark.executor.instances=4, spark.executor.memory=12g, spark.executor.cores=2, spark.kubernetes.memoryOverheadFactor=0.6, spark.driver.memory=3g, spark.sql.shuffle.partitions=80, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. Optional High I/O config (only if there is a use case for it) - spark.executor.instances=2, spark.executor.memory=16g, spark.executor.cores=8, spark.kubernetes.memoryOverheadFactor=0.4, spark.driver.memory=3g, spark.sql.shuffle.partitions=40, spark.sql.broadcastTimeout=3600, spark.port.maxRetries=200, spark.driver.host=&lt;DSS host IP&gt;. These values are guidance, not a requirement.</t>
+        </is>
+      </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>Job/notebook execution logs show successful completion of a Spark recipe and a Spark notebook session, and cluster monitoring shows executor pods created during notebook execution.</t>
+          <t>sparkSettings contains multiple named configs roughly matching these purposes (default/high-parallelism/large-memory, and optionally high I/O).</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>The Spark recipe or notebook execution fails, hangs, or no executor pods ever appear in the cluster.</t>
+          <t>Only a single undifferentiated spark config exists despite varied workload needs (e.g., both lightweight recipes and large jobs run identically).</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file lacks job/notebook execution logs or cluster pod visibility, flag needs_manual_review and recommend running these test steps manually.</t>
+          <t>If the diagnosis file does not list multiple sparkSettings configs or describe workload diversity, flag needs_manual_review and ask about workload variety.</t>
         </is>
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>Confirms Spark integration works end-to-end, beyond just having a syntactically valid configuration.</t>
+          <t>Different Spark workloads (lightweight recipes vs. large jobs vs. I/O-heavy jobs) benefit from different executor sizing and parallelism trade-offs.</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>Spark recipe, Spark notebook, Kubernetes executor pods</t>
+          <t>Spark executor, Spark configuration, Kubernetes</t>
         </is>
       </c>
       <c r="R7" s="3" t="inlineStr">
@@ -1164,12 +1180,12 @@
       </c>
       <c r="S7" s="3" t="inlineStr">
         <is>
-          <t>5, 6, 7</t>
+          <t>4, 5</t>
         </is>
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>Additional Spark testing; Spark on Notebook MUST HAVE; Spark on Notebook MUST HAVE</t>
+          <t>Define three spark configs - NICE TO HAVE; Special spark configs (only if there's use case for it)</t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr">
@@ -1177,11 +1193,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="V7" s="3" t="inlineStr">
-        <is>
-          <t>Worded for Spark on Kubernetes (executor pods). If no Kubernetes cluster is attached and Spark runs on YARN/Hadoop, the pod-based checks do not apply.</t>
-        </is>
-      </c>
+      <c r="V7" s="3" t="n"/>
       <c r="W7" s="3" t="n"/>
       <c r="X7" s="3" t="n"/>
       <c r="Y7" s="3" t="n"/>
@@ -1191,12 +1203,12 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>ARCH-010</t>
+          <t>ARCH-007</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -1206,68 +1218,68 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Containerized Execution</t>
+          <t>Spark Configuration</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Valid Containerized Execution Configuration</t>
+          <t>Kubernetes Namespace and Auth Recommendations for Spark</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Environments using Elastic Compute (Kubernetes) must have at least one valid containerized execution configuration set up (general-settings.json &gt; containerSettings, or Administration &gt; Settings &gt; Containerized execution); as with Spark, the specific example values are only a baseline, not a strict requirement.</t>
+          <t>For Spark-on-Kubernetes, Dataiku recommends one Kubernetes namespace per user (e.g. dss-ns-${dssUserLogin}), auto-creating namespaces, ensuring namespace names are Kubernetes-compliant, and dynamically creating service accounts for authentication mode.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Configure at least one valid containerized execution config when using Elastic Compute.</t>
+          <t>Use one Kubernetes namespace per user with auto-created, dynamically authenticated service accounts for Spark.</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; containerSettings</t>
+          <t>general-settings.json &gt; sparkSettings (Kubernetes namespace/authentication settings)</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>exists</t>
+          <t>equals</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>valid containerized execution configuration present</t>
+          <t>one namespace per user (dss-ns-${dssUserLogin}), auto-create namespaces enabled, K8s-compliant naming, dynamic service account creation</t>
         </is>
       </c>
       <c r="K8" s="3" t="n"/>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>Required only when the customer uses Elastic Compute/Kubernetes for offloaded workloads.</t>
+          <t>No single literal diag field was given for this sub-setting; pointer is a best-effort conceptual location within sparkSettings/Kubernetes settings.</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>containerSettings block is present with at least one named config with reasonable memory requests/limits.</t>
+          <t>Namespace naming pattern and auto-create/dynamic service account settings match the recommendation.</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>containerSettings is missing or empty while the instance shows evidence of Kubernetes-based execution elsewhere in the diagnosis.</t>
+          <t>A single shared namespace is used for all users, or service accounts are managed manually rather than dynamically.</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not clarify whether Elastic Compute is used, flag needs_manual_review.</t>
+          <t>If the diagnosis file does not expose namespace or authentication configuration for Spark-on-Kubernetes, flag needs_manual_review.</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>A valid container exec config is required to run workloads in Kubernetes.</t>
+          <t>Per-user namespace isolation improves security boundaries and resource tracking on Kubernetes.</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>Containerized execution, containerSettings, Elastic Compute</t>
+          <t>Kubernetes namespace, Service account, Spark on Kubernetes</t>
         </is>
       </c>
       <c r="R8" s="3" t="inlineStr">
@@ -1277,17 +1289,17 @@
       </c>
       <c r="S8" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>Containerized execution configs | MUST HAVE if using Elastic Compute</t>
+          <t>Recommended Settings NICE TO HAVE</t>
         </is>
       </c>
       <c r="U8" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="V8" s="3" t="n"/>
@@ -1300,7 +1312,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>ARCH-013</t>
+          <t>ARCH-008</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1310,69 +1322,57 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>specific_setting</t>
+          <t>qualitative_practice</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Cluster Configuration</t>
+          <t>Spark Validation</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Valid Cluster Configuration for Elastic Compute</t>
+          <t>Functional Validation of Spark Execution (Recipe &amp; Notebook)</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Environments using Elastic Compute must have at least one valid cluster configured (found under {DATADIR}/config/clusters or Administration &gt; Clusters); Dataiku does not mandate the specific example configuration, only that a workable cluster exists.</t>
+          <t>Reviewers should functionally validate Spark execution: run a Spark-engine recipe on Kubernetes in a test project (should succeed), and separately launch a Python/R/Scala notebook with starter Spark code and run it locally (should succeed, with Spark executor pods visible in the cluster while the code runs).</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Configure at least one valid Kubernetes cluster when using Elastic Compute.</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>{DATADIR}/config/clusters</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>exists</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>at least one valid cluster configuration present</t>
-        </is>
-      </c>
+          <t>Validate Spark execution by successfully running a test Spark recipe and notebook.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="n"/>
       <c r="K9" s="3" t="n"/>
       <c r="L9" s="3" t="n"/>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>The clusters config/directory contains at least one properly defined cluster, consistent with other evidence of elastic-compute usage (spark/container jobs running on Kubernetes).</t>
+          <t>Job/notebook execution logs show successful completion of a Spark recipe and a Spark notebook session, and cluster monitoring shows executor pods created during notebook execution.</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>No cluster configuration is present despite evidence of Kubernetes-based workloads elsewhere in the diagnosis.</t>
+          <t>The Spark recipe or notebook execution fails, hangs, or no executor pods ever appear in the cluster.</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not clarify whether Elastic Compute is used at all, flag needs_manual_review.</t>
+          <t>If the diagnosis file lacks job/notebook execution logs or cluster pod visibility, flag needs_manual_review and recommend running these test steps manually.</t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>A valid cluster is required to offload computation to Kubernetes.</t>
+          <t>Confirms Spark integration works end-to-end, beyond just having a syntactically valid configuration.</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>Cluster, Managed cluster, Unmanaged cluster, Elastic AI</t>
+          <t>Spark recipe, Spark notebook, Kubernetes executor pods</t>
         </is>
       </c>
       <c r="R9" s="3" t="inlineStr">
@@ -1382,12 +1382,12 @@
       </c>
       <c r="S9" s="3" t="inlineStr">
         <is>
-          <t>12, 13</t>
+          <t>5, 6, 7</t>
         </is>
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>Cluster configurations | MUST HAVE if using Elastic Compute; Cluster configurations | MUST HAVE if using Elastic Compute</t>
+          <t>Additional Spark testing; Spark on Notebook MUST HAVE; Spark on Notebook MUST HAVE</t>
         </is>
       </c>
       <c r="U9" s="3" t="inlineStr">
@@ -1395,12 +1395,553 @@
           <t>high</t>
         </is>
       </c>
-      <c r="V9" s="3" t="n"/>
+      <c r="V9" s="3" t="inlineStr">
+        <is>
+          <t>Worded for Spark on Kubernetes (executor pods). If no Kubernetes cluster is attached and Spark runs on YARN/Hadoop, the pod-based checks do not apply.</t>
+        </is>
+      </c>
       <c r="W9" s="3" t="n"/>
       <c r="X9" s="3" t="n"/>
       <c r="Y9" s="3" t="n"/>
       <c r="Z9" s="3" t="n"/>
       <c r="AA9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-010</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Containerized Execution</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Valid Containerized Execution Configuration</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Environments using Elastic Compute (Kubernetes) must have at least one valid containerized execution configuration set up (general-settings.json &gt; containerSettings, or Administration &gt; Settings &gt; Containerized execution); as with Spark, the specific example values are only a baseline, not a strict requirement.</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Configure at least one valid containerized execution config when using Elastic Compute.</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; containerSettings</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>exists</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>valid containerized execution configuration present</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>Required only when the customer uses Elastic Compute/Kubernetes for offloaded workloads.</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>containerSettings block is present with at least one named config with reasonable memory requests/limits.</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>containerSettings is missing or empty while the instance shows evidence of Kubernetes-based execution elsewhere in the diagnosis.</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not clarify whether Elastic Compute is used, flag needs_manual_review.</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>A valid container exec config is required to run workloads in Kubernetes.</t>
+        </is>
+      </c>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>Containerized execution, containerSettings, Elastic Compute</t>
+        </is>
+      </c>
+      <c r="R10" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S10" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="T10" s="3" t="inlineStr">
+        <is>
+          <t>Containerized execution configs | MUST HAVE if using Elastic Compute</t>
+        </is>
+      </c>
+      <c r="U10" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V10" s="3" t="n"/>
+      <c r="W10" s="3" t="n"/>
+      <c r="X10" s="3" t="n"/>
+      <c r="Y10" s="3" t="n"/>
+      <c r="Z10" s="3" t="n"/>
+      <c r="AA10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-011</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>nice_to_have</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Containerized Execution</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Baseline Container Execution Configs (Standard, Webapp) and Namespace Settings</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Dataiku recommends at least two named containerized execution configs as a baseline - a Standard config for notebooks/recipes/ML (memory request 200MB, memory limit 16000MB) and a Webapp config for webapps (memory request 500MB, memory limit 500MB) - plus per-user Kubernetes namespaces (dss-ns-${dssUserLogin}) with K8s-compliant naming and auto-creation, and using the Webapp config for virtual webapp backends run in containers.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Define Standard and Webapp container execution configs plus per-user Kubernetes namespaces.</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; containerSettings (named container exec configs)</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>one_of</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Standard config (memory request 200MB / limit 16000MB) and Webapp config (memory request 500MB / limit 500MB)</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>Additional recommended settings: one Kubernetes namespace per user (dss-ns-${dssUserLogin}), K8s-compliant namespace names, auto-create namespaces, and virtual webapps configured to run in a container using the Webapp config.</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>containerSettings includes configs resembling the Standard and Webapp purposes with comparable memory request/limit values, and namespace settings follow a per-user pattern.</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>A single undifferentiated container config is used for both interactive workloads and webapps, or all users share one namespace.</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not list named container configs or namespace settings, flag needs_manual_review.</t>
+        </is>
+      </c>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
+          <t>Separating configs by workload type avoids over- or under-provisioning; per-user namespaces aid isolation and cost tracking.</t>
+        </is>
+      </c>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>Containerized execution, Kubernetes namespace, Webapp backend</t>
+        </is>
+      </c>
+      <c r="R11" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S11" s="3" t="inlineStr">
+        <is>
+          <t>8, 9</t>
+        </is>
+      </c>
+      <c r="T11" s="3" t="inlineStr">
+        <is>
+          <t>Recommendations NICE TO HAVE; Recommended Settings</t>
+        </is>
+      </c>
+      <c r="U11" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V11" s="3" t="n"/>
+      <c r="W11" s="3" t="n"/>
+      <c r="X11" s="3" t="n"/>
+      <c r="Y11" s="3" t="n"/>
+      <c r="Z11" s="3" t="n"/>
+      <c r="AA11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-013</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Cluster Configuration</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Valid Cluster Configuration for Elastic Compute</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Environments using Elastic Compute must have at least one valid cluster configured (found under {DATADIR}/config/clusters or Administration &gt; Clusters); Dataiku does not mandate the specific example configuration, only that a workable cluster exists.</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Configure at least one valid Kubernetes cluster when using Elastic Compute.</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>{DATADIR}/config/clusters</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>exists</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>at least one valid cluster configuration present</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="3" t="n"/>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>The clusters config/directory contains at least one properly defined cluster, consistent with other evidence of elastic-compute usage (spark/container jobs running on Kubernetes).</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>No cluster configuration is present despite evidence of Kubernetes-based workloads elsewhere in the diagnosis.</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not clarify whether Elastic Compute is used at all, flag needs_manual_review.</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>A valid cluster is required to offload computation to Kubernetes.</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>Cluster, Managed cluster, Unmanaged cluster, Elastic AI</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>12, 13</t>
+        </is>
+      </c>
+      <c r="T12" s="3" t="inlineStr">
+        <is>
+          <t>Cluster configurations | MUST HAVE if using Elastic Compute; Cluster configurations | MUST HAVE if using Elastic Compute</t>
+        </is>
+      </c>
+      <c r="U12" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V12" s="3" t="n"/>
+      <c r="W12" s="3" t="n"/>
+      <c r="X12" s="3" t="n"/>
+      <c r="Y12" s="3" t="n"/>
+      <c r="Z12" s="3" t="n"/>
+      <c r="AA12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-016</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Default Compute Settings</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Global Default Cluster and Default Execution Config Set (if Elastic AI used)</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>If the customer intends to offload most or all recipes to Kubernetes, a default cluster (general-settings.json &gt; defaultK8sClusterId) and a default containerized execution config (general-settings.json &gt; defaultExecutionConfig) should be set globally rather than configured per-recipe or per-project; if this global default is set, the associated execution config must have properly configured resource requests/limits rather than being a resource-hogging default.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Set a global default cluster and execution config with proper resource limits when offloading broadly.</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; defaultK8sClusterId and general-settings.json &gt; defaultExecutionConfig</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>exists</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>both set to valid, non-resource-hogging values when Elastic AI/offloading is used broadly</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="n"/>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>Both defaultK8sClusterId and defaultExecutionConfig are set to valid values, and the referenced execution config has reasonable memory/CPU requests and limits.</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>These fields are unset despite most recipes being offloaded to Kubernetes, or the default execution config lacks resource limits/requests (resource-hogging risk).</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not clarify the proportion of recipes offloaded to Kubernetes, flag needs_manual_review to confirm intended usage pattern with the customer.</t>
+        </is>
+      </c>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>Setting a global default simplifies configuration management and avoids inconsistent per-recipe settings; an unset or misconfigured default risks uncontrolled resource usage.</t>
+        </is>
+      </c>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>defaultK8sClusterId, defaultExecutionConfig, Containerized execution, Elastic AI</t>
+        </is>
+      </c>
+      <c r="R13" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S13" s="3" t="inlineStr">
+        <is>
+          <t>15, 16</t>
+        </is>
+      </c>
+      <c r="T13" s="3" t="inlineStr">
+        <is>
+          <t>Default Cluster &amp; Default Containerized Execution Config | MUST HAVE if Elastic AI is used; Default Cluster &amp; Default Containerized Execution Config | MUST HAVE if Elastic AI is used</t>
+        </is>
+      </c>
+      <c r="U13" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V13" s="3" t="n"/>
+      <c r="W13" s="3" t="n"/>
+      <c r="X13" s="3" t="n"/>
+      <c r="Y13" s="3" t="n"/>
+      <c r="Z13" s="3" t="n"/>
+      <c r="AA13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-017</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>nice_to_have</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Containerized Visual Recipes</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Containerized Visual Recipes (CDE) Enabled and Base Image Built</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>If the customer intends to offload visual recipes to Kubernetes, CDE should be enabled (general-settings.json &gt; cdeEnabled) and its base image built via Administration &gt; Settings &gt; Containerized Execution &gt; Build image for containerized visual recipes; a default execution config for visual recipe workloads (general-settings.json &gt; defaultExecutionConfigForVisualRecipesWorkloads) should also be set, validated by confirming a simple recipe (e.g. a sync recipe) shows Engine: DSS (containerized).</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Enable CDE and build its base image to offload visual recipes to Kubernetes.</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; cdeEnabled and general-settings.json &gt; defaultExecutionConfigForVisualRecipesWorkloads</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>equals</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>cdeEnabled=true and defaultExecutionConfigForVisualRecipesWorkloads set to a valid execution config</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="n"/>
+      <c r="L14" s="3" t="n"/>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>cdeEnabled is true, base CDE image build evidence exists, defaultExecutionConfigForVisualRecipesWorkloads is set, and a sample visual recipe shows Engine: DSS (containerized).</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>cdeEnabled is false or unset while the customer relies on Kubernetes offloading for visual recipes, or a visual recipe fails to show the containerized engine.</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not indicate whether visual recipe offloading to Kubernetes is desired, flag needs_manual_review.</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>Ensures visual recipes can actually be executed on the cluster with an appropriate base image and default resource config.</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>CDE, cdeEnabled, Visual recipes, Containerized execution</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>16, 17, 18</t>
+        </is>
+      </c>
+      <c r="T14" s="3" t="inlineStr">
+        <is>
+          <t>Containerized Visual Recipes (CDE) | NICE TO HAVE; Containerized Visual Recipes (CDE) | NICE TO HAVE; Containerized Visual Recipes (CDE) | NICE TO HAVE</t>
+        </is>
+      </c>
+      <c r="U14" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V14" s="3" t="n"/>
+      <c r="W14" s="3" t="n"/>
+      <c r="X14" s="3" t="n"/>
+      <c r="Y14" s="3" t="n"/>
+      <c r="Z14" s="3" t="n"/>
+      <c r="AA14" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Release 0.38.2: rules for 16 more checks (62 of 67), reader 0.20.0, ADVSEC policy notes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/checklists/eval_checklist.xlsx
+++ b/tests/fixtures/checklists/eval_checklist.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA14"/>
+  <dimension ref="A1:AA16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1736,12 +1736,12 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>ARCH-016</t>
+          <t>ARCH-014</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1751,64 +1751,68 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Default Compute Settings</t>
+          <t>Cluster Configuration</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Global Default Cluster and Default Execution Config Set (if Elastic AI used)</t>
+          <t>Recommended Cluster Topology (Single Managed Cluster, Node Groups, Autoscaling)</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>If the customer intends to offload most or all recipes to Kubernetes, a default cluster (general-settings.json &gt; defaultK8sClusterId) and a default containerized execution config (general-settings.json &gt; defaultExecutionConfig) should be set globally rather than configured per-recipe or per-project; if this global default is set, the associated execution config must have properly configured resource requests/limits rather than being a resource-hogging default.</t>
+          <t>Dataiku recommends a single managed cluster with one CPU node group serving containerized execution, ML, Spark, webapp, and API workloads, adding a separate GPU node group only if needed, and enabling a metrics server plus cluster autoscaling.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Set a global default cluster and execution config with proper resource limits when offloading broadly.</t>
+          <t>Use a single managed cluster with one CPU node group and autoscaling enabled.</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; defaultK8sClusterId and general-settings.json &gt; defaultExecutionConfig</t>
+          <t>{DATADIR}/config/clusters (cluster topology / node group / autoscaling settings)</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>exists</t>
+          <t>equals</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>both set to valid, non-resource-hogging values when Elastic AI/offloading is used broadly</t>
+          <t>single managed cluster, one CPU node group for all standard workloads, optional GPU node group only if needed, metrics server installed, autoscaling enabled</t>
         </is>
       </c>
       <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="n"/>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>No literal single field was given for this recommendation; pointer is a best-effort conceptual location within the clusters config.</t>
+        </is>
+      </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>Both defaultK8sClusterId and defaultExecutionConfig are set to valid values, and the referenced execution config has reasonable memory/CPU requests and limits.</t>
+          <t>Cluster configuration shows one managed cluster with a shared CPU node group, autoscaling enabled, metrics server installed, and a GPU node group only present when GPU workloads exist.</t>
         </is>
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>These fields are unset despite most recipes being offloaded to Kubernetes, or the default execution config lacks resource limits/requests (resource-hogging risk).</t>
+          <t>Multiple redundant clusters/node groups without clear justification, no autoscaling enabled, or a GPU node group present without any GPU workload evidence.</t>
         </is>
       </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not clarify the proportion of recipes offloaded to Kubernetes, flag needs_manual_review to confirm intended usage pattern with the customer.</t>
+          <t>If the diagnosis file does not detail node groups or autoscaling settings, flag needs_manual_review.</t>
         </is>
       </c>
       <c r="P13" s="3" t="inlineStr">
         <is>
-          <t>Setting a global default simplifies configuration management and avoids inconsistent per-recipe settings; an unset or misconfigured default risks uncontrolled resource usage.</t>
+          <t>Simplifies management and reduces cost while retaining elasticity for varying workloads.</t>
         </is>
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>defaultK8sClusterId, defaultExecutionConfig, Containerized execution, Elastic AI</t>
+          <t>Managed cluster, Node group, Autoscaling, Metrics server</t>
         </is>
       </c>
       <c r="R13" s="3" t="inlineStr">
@@ -1818,17 +1822,17 @@
       </c>
       <c r="S13" s="3" t="inlineStr">
         <is>
-          <t>15, 16</t>
+          <t>14</t>
         </is>
       </c>
       <c r="T13" s="3" t="inlineStr">
         <is>
-          <t>Default Cluster &amp; Default Containerized Execution Config | MUST HAVE if Elastic AI is used; Default Cluster &amp; Default Containerized Execution Config | MUST HAVE if Elastic AI is used</t>
+          <t>Recommended settings NICE TO HAVE</t>
         </is>
       </c>
       <c r="U13" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="V13" s="3" t="n"/>
@@ -1841,12 +1845,12 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>ARCH-017</t>
+          <t>ARCH-015</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>nice_to_have</t>
+          <t>must_have</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1856,64 +1860,72 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Containerized Visual Recipes</t>
+          <t>Cluster Sizing</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Containerized Visual Recipes (CDE) Enabled and Base Image Built</t>
+          <t>Appropriate Cluster Sizing</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>If the customer intends to offload visual recipes to Kubernetes, CDE should be enabled (general-settings.json &gt; cdeEnabled) and its base image built via Administration &gt; Settings &gt; Containerized Execution &gt; Build image for containerized visual recipes; a default execution config for visual recipe workloads (general-settings.json &gt; defaultExecutionConfigForVisualRecipesWorkloads) should also be set, validated by confirming a simple recipe (e.g. a sync recipe) shows Engine: DSS (containerized).</t>
+          <t>The Kubernetes cluster must be sized appropriately for the customer's workloads - large enough to avoid resource exhaustion but not so large as to waste resources. Dataiku's memory/disk calculation is only an illustrative baseline (not a mandatory formula), derived from Spark settings (general-settings.json &gt; sparkSettings), container exec settings (general-settings.json &gt; containerSettings), and global flow concurrency (general-settings.json &gt; maxRunningActivities).</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Enable CDE and build its base image to offload visual recipes to Kubernetes.</t>
+          <t>Size the Kubernetes cluster appropriately for workloads, avoiding under- or over-provisioning.</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; cdeEnabled and general-settings.json &gt; defaultExecutionConfigForVisualRecipesWorkloads</t>
+          <t>general-settings.json &gt; sparkSettings, general-settings.json &gt; containerSettings, general-settings.json &gt; maxRunningActivities (used to estimate cluster memory/disk sizing)</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>equals</t>
+          <t>greater_than_or_equal</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>cdeEnabled=true and defaultExecutionConfigForVisualRecipesWorkloads set to a valid execution config</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="n"/>
+          <t>cluster capacity &gt;= estimated total_memory and disk needs derived from the formulas in notes</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>Illustrative sizing formulas provided by Dataiku, reproduced in full: spark_recipes_memory = global flow concurrency*spark.executor.instances*spark.executor.memory*(1+spark.kubernetes.memoryOverheadFactor) [based on the largest spark config]. spark_notebooks_memory = 30%_DSS_users*spark.executor.instances*spark.executor.memory*(1+spark.kubernetes.memoryOverheadFactor) [using associated spark config]. jupyter_notebooks_memory = 30%_DSS_users * container exec memory limit [using associated container exec config]. total_memory = spark_recipes_memory + spark_notebooks_memory + jupyter_notebooks_memory. DISK = 25GB * spark.executor.instances. Recommended instance sizing: 64 GB &lt; worker size &lt; 128 GB. These are baselines/examples; the cluster need not match this exact calculation, but must be appropriately sized for the customer's workloads based on evidence, and should not be resized without evidence of resource exhaustion.</t>
+        </is>
+      </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>cdeEnabled is true, base CDE image build evidence exists, defaultExecutionConfigForVisualRecipesWorkloads is set, and a sample visual recipe shows Engine: DSS (containerized).</t>
+          <t>Cluster memory/CPU capacity is consistent with or exceeds the estimated total_memory/disk needs given current spark/container/concurrency settings, with no signs of chronic resource exhaustion (OOM kills, pending pods) or gross over-provisioning.</t>
         </is>
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>cdeEnabled is false or unset while the customer relies on Kubernetes offloading for visual recipes, or a visual recipe fails to show the containerized engine.</t>
+          <t>Cluster capacity is far below estimated needs (frequent OOM kills/evictions) or drastically oversized relative to workload with no growth justification.</t>
         </is>
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not indicate whether visual recipe offloading to Kubernetes is desired, flag needs_manual_review.</t>
+          <t>If the diagnosis file lacks cluster capacity metrics or the underlying spark/container/concurrency settings needed to compute the estimate, flag needs_manual_review and recommend gathering these values.</t>
         </is>
       </c>
       <c r="P14" s="3" t="inlineStr">
         <is>
-          <t>Ensures visual recipes can actually be executed on the cluster with an appropriate base image and default resource config.</t>
+          <t>Prevents both instability/performance degradation from under-sizing and cost waste from over-sizing.</t>
         </is>
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>CDE, cdeEnabled, Visual recipes, Containerized execution</t>
+          <t>Cluster sizing, Spark executor memory, Container exec memory limit, maxRunningActivities, Global flow concurrency</t>
         </is>
       </c>
       <c r="R14" s="3" t="inlineStr">
@@ -1923,12 +1935,12 @@
       </c>
       <c r="S14" s="3" t="inlineStr">
         <is>
-          <t>16, 17, 18</t>
+          <t>14, 15</t>
         </is>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>Containerized Visual Recipes (CDE) | NICE TO HAVE; Containerized Visual Recipes (CDE) | NICE TO HAVE; Containerized Visual Recipes (CDE) | NICE TO HAVE</t>
+          <t>Cluster sizing | MUST HAVE; Cluster sizing | MUST HAVE</t>
         </is>
       </c>
       <c r="U14" s="3" t="inlineStr">
@@ -1942,6 +1954,216 @@
       <c r="Y14" s="3" t="n"/>
       <c r="Z14" s="3" t="n"/>
       <c r="AA14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-016</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Default Compute Settings</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Global Default Cluster and Default Execution Config Set (if Elastic AI used)</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>If the customer intends to offload most or all recipes to Kubernetes, a default cluster (general-settings.json &gt; defaultK8sClusterId) and a default containerized execution config (general-settings.json &gt; defaultExecutionConfig) should be set globally rather than configured per-recipe or per-project; if this global default is set, the associated execution config must have properly configured resource requests/limits rather than being a resource-hogging default.</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Set a global default cluster and execution config with proper resource limits when offloading broadly.</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; defaultK8sClusterId and general-settings.json &gt; defaultExecutionConfig</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>exists</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>both set to valid, non-resource-hogging values when Elastic AI/offloading is used broadly</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="3" t="n"/>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>Both defaultK8sClusterId and defaultExecutionConfig are set to valid values, and the referenced execution config has reasonable memory/CPU requests and limits.</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>These fields are unset despite most recipes being offloaded to Kubernetes, or the default execution config lacks resource limits/requests (resource-hogging risk).</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not clarify the proportion of recipes offloaded to Kubernetes, flag needs_manual_review to confirm intended usage pattern with the customer.</t>
+        </is>
+      </c>
+      <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t>Setting a global default simplifies configuration management and avoids inconsistent per-recipe settings; an unset or misconfigured default risks uncontrolled resource usage.</t>
+        </is>
+      </c>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>defaultK8sClusterId, defaultExecutionConfig, Containerized execution, Elastic AI</t>
+        </is>
+      </c>
+      <c r="R15" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S15" s="3" t="inlineStr">
+        <is>
+          <t>15, 16</t>
+        </is>
+      </c>
+      <c r="T15" s="3" t="inlineStr">
+        <is>
+          <t>Default Cluster &amp; Default Containerized Execution Config | MUST HAVE if Elastic AI is used; Default Cluster &amp; Default Containerized Execution Config | MUST HAVE if Elastic AI is used</t>
+        </is>
+      </c>
+      <c r="U15" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V15" s="3" t="n"/>
+      <c r="W15" s="3" t="n"/>
+      <c r="X15" s="3" t="n"/>
+      <c r="Y15" s="3" t="n"/>
+      <c r="Z15" s="3" t="n"/>
+      <c r="AA15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-017</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>nice_to_have</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Containerized Visual Recipes</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Containerized Visual Recipes (CDE) Enabled and Base Image Built</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>If the customer intends to offload visual recipes to Kubernetes, CDE should be enabled (general-settings.json &gt; cdeEnabled) and its base image built via Administration &gt; Settings &gt; Containerized Execution &gt; Build image for containerized visual recipes; a default execution config for visual recipe workloads (general-settings.json &gt; defaultExecutionConfigForVisualRecipesWorkloads) should also be set, validated by confirming a simple recipe (e.g. a sync recipe) shows Engine: DSS (containerized).</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Enable CDE and build its base image to offload visual recipes to Kubernetes.</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; cdeEnabled and general-settings.json &gt; defaultExecutionConfigForVisualRecipesWorkloads</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>equals</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>cdeEnabled=true and defaultExecutionConfigForVisualRecipesWorkloads set to a valid execution config</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="n"/>
+      <c r="L16" s="3" t="n"/>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>cdeEnabled is true, base CDE image build evidence exists, defaultExecutionConfigForVisualRecipesWorkloads is set, and a sample visual recipe shows Engine: DSS (containerized).</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>cdeEnabled is false or unset while the customer relies on Kubernetes offloading for visual recipes, or a visual recipe fails to show the containerized engine.</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not indicate whether visual recipe offloading to Kubernetes is desired, flag needs_manual_review.</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>Ensures visual recipes can actually be executed on the cluster with an appropriate base image and default resource config.</t>
+        </is>
+      </c>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>CDE, cdeEnabled, Visual recipes, Containerized execution</t>
+        </is>
+      </c>
+      <c r="R16" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S16" s="3" t="inlineStr">
+        <is>
+          <t>16, 17, 18</t>
+        </is>
+      </c>
+      <c r="T16" s="3" t="inlineStr">
+        <is>
+          <t>Containerized Visual Recipes (CDE) | NICE TO HAVE; Containerized Visual Recipes (CDE) | NICE TO HAVE; Containerized Visual Recipes (CDE) | NICE TO HAVE</t>
+        </is>
+      </c>
+      <c r="U16" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V16" s="3" t="n"/>
+      <c r="W16" s="3" t="n"/>
+      <c r="X16" s="3" t="n"/>
+      <c r="Y16" s="3" t="n"/>
+      <c r="Z16" s="3" t="n"/>
+      <c r="AA16" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2873,7 +3095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA8"/>
+  <dimension ref="A1:AA9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3675,12 +3897,12 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>GENAI-009</t>
+          <t>GENAI-008</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>nice_to_have</t>
+          <t>must_have</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -3690,22 +3912,22 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Agent Hub</t>
+          <t>AI Assistants Diagnostics</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Agent Hub Deployment Required Permissions</t>
+          <t>Include AI Assistant Debug Data in Instance Diagnostics</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Before a user can deploy an Agent Hub instance, they must have permissions for writing project content in the hosting project, writing isolated code execution, WebApp impersonation, and (if Quick agents are enabled) create projects; alternatively the user could be a DSS administrator, though a dedicated service account is preferred.</t>
+          <t>To access AI Assistant Logs (ui.json, runtime.json, traces per project) in an Instance Diagnostic (V14.7+), an administrator must explicitly select the option to include these logs when generating a diagnostic via Administration &gt; Maintenance &gt; Instance Diagnostic.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Grant Agent Hub deployers write project content, isolated code execution, and webapp impersonation permissions.</t>
+          <t>Select the option to include AI Assistant debug logs when generating instance diagnostics.</t>
         </is>
       </c>
       <c r="H8" s="3" t="n"/>
@@ -3715,27 +3937,27 @@
       <c r="L8" s="3" t="n"/>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>Administration &gt; Security &gt; Groups shows the Agent Hub deployer's group granted 'Write project content', 'Write isolated code execution', and 'WebApp impersonation' permissions (plus 'Create projects' if Quick agents are enabled), or the deployer is a DSS admin/service account.</t>
+          <t>The diagnostic bundle includes an 'AI Assistants debug data' section organized by project with ui.json, runtime.json, and traces files.</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>The deployer's group lacks one or more of these permissions and is not an admin/service account, or logs show 'Not authorized' errors when creating the Agent Hub WebApp.</t>
+          <t>Diagnostic bundle lacks these files despite AI Assistants being actively used on the instance.</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file lacks per-user/group permission detail, flag needs_manual_review and recommend checking Administration &gt; Security &gt; Groups directly.</t>
+          <t>If the diagnostic was generated on a version prior to 14.7, or the inclusion option's state can't be determined, flag needs_manual_review and note reviewers should confirm the option was selected during diagnostic generation.</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>Missing permissions cause deployment failures such as 'Not authorized' errors when creating the Agent Hub WebApp.</t>
+          <t>Without selecting this option, AI Assistant logs are not captured, limiting the reviewer's ability to diagnose LLM Mesh/agent-building issues.</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>Agent Hub, Permissions, Groups, WebApp</t>
+          <t>Instance Diagnostic, AI Assistants, Logging</t>
         </is>
       </c>
       <c r="R8" s="3" t="inlineStr">
@@ -3745,22 +3967,22 @@
       </c>
       <c r="S8" s="3" t="inlineStr">
         <is>
-          <t>10, 11, 12</t>
+          <t>9, 10</t>
         </is>
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>Agent Hub NICE TO HAVE:; Writing isolated code execution; WebApp impersonation</t>
+          <t>Instance Diags / DiagParser3; Instance Diags / DiagParser3</t>
         </is>
       </c>
       <c r="U8" s="3" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="V8" s="3" t="inlineStr">
         <is>
-          <t>Although the parent topic is tagged NICE TO HAVE, the described permission requirements are phrased as mandatory ('must have permissions') for successful deployment; classification follows the explicit heading tag.</t>
+          <t>This is more a diagnostic-generation process note than a platform configuration state, so evaluability from a static diagnosis file is limited.</t>
         </is>
       </c>
       <c r="W8" s="3" t="n"/>
@@ -3768,6 +3990,103 @@
       <c r="Y8" s="3" t="n"/>
       <c r="Z8" s="3" t="n"/>
       <c r="AA8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>GENAI-009</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>nice_to_have</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>qualitative_practice</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub Deployment Required Permissions</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Before a user can deploy an Agent Hub instance, they must have permissions for writing project content in the hosting project, writing isolated code execution, WebApp impersonation, and (if Quick agents are enabled) create projects; alternatively the user could be a DSS administrator, though a dedicated service account is preferred.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Grant Agent Hub deployers write project content, isolated code execution, and webapp impersonation permissions.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="n"/>
+      <c r="K9" s="3" t="n"/>
+      <c r="L9" s="3" t="n"/>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>Administration &gt; Security &gt; Groups shows the Agent Hub deployer's group granted 'Write project content', 'Write isolated code execution', and 'WebApp impersonation' permissions (plus 'Create projects' if Quick agents are enabled), or the deployer is a DSS admin/service account.</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>The deployer's group lacks one or more of these permissions and is not an admin/service account, or logs show 'Not authorized' errors when creating the Agent Hub WebApp.</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file lacks per-user/group permission detail, flag needs_manual_review and recommend checking Administration &gt; Security &gt; Groups directly.</t>
+        </is>
+      </c>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>Missing permissions cause deployment failures such as 'Not authorized' errors when creating the Agent Hub WebApp.</t>
+        </is>
+      </c>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub, Permissions, Groups, WebApp</t>
+        </is>
+      </c>
+      <c r="R9" s="3" t="inlineStr">
+        <is>
+          <t>generative_ai_acceleration</t>
+        </is>
+      </c>
+      <c r="S9" s="3" t="inlineStr">
+        <is>
+          <t>10, 11, 12</t>
+        </is>
+      </c>
+      <c r="T9" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub NICE TO HAVE:; Writing isolated code execution; WebApp impersonation</t>
+        </is>
+      </c>
+      <c r="U9" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V9" s="3" t="inlineStr">
+        <is>
+          <t>Although the parent topic is tagged NICE TO HAVE, the described permission requirements are phrased as mandatory ('must have permissions') for successful deployment; classification follows the explicit heading tag.</t>
+        </is>
+      </c>
+      <c r="W9" s="3" t="n"/>
+      <c r="X9" s="3" t="n"/>
+      <c r="Y9" s="3" t="n"/>
+      <c r="Z9" s="3" t="n"/>
+      <c r="AA9" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3780,7 +4099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA11"/>
+  <dimension ref="A1:AA15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5002,6 +5321,442 @@
       <c r="Y11" s="3" t="n"/>
       <c r="Z11" s="3" t="n"/>
       <c r="AA11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>SCALE-012</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Cloud Storage Connections</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Cloud Object Storage Configuration (Details Readable By, HDFS Interface)</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>For S3/Azure Blob/GCS connections, enable 'Details readable by' to allow compute engines (Spark, Snowflake, Databricks) direct/parallel access instead of funneling through the DSS node, and set the appropriate HDFS interface per cloud/storage type (S3: S3A off-EMR or EMRFS on-EMR; Azure Blob: ABFS if Hierarchical namespace enabled else WASB; GCS: GS). Consider S3 VPC endpoints if custom VPC egress routing impacts performance, though this should be a recommendation rather than a mandatory fix.</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Enable Details readable by and set the correct HDFS interface for cloud storage connections.</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>cloud storage connection settings &gt; detailsReadableBy</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>equals</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>Also verify HDFS interface setting matches the cloud storage type mapping (S3A/EMRFS for S3, ABFS/WASB for Azure Blob, GS for GCS).</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>Cloud storage connections show 'Details readable by' enabled and the correct HDFS interface configured per the platform/type mapping.</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>'Details readable by' disabled, forcing all traffic through the DSS node (performance bottleneck), or a mismatched/incorrect HDFS interface for the cloud storage type.</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>If connection details aren't in the diagnosis, flag needs_manual_review and check Administration &gt; Connections for each cloud storage connection.</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>Without 'Details readable by', all data traffic funnels through the single DSS node creating a performance bottleneck; correct HDFS interface ensures compatibility with distributed compute engines.</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>cloud storage connections, details readable by, HDFS interface, S3, Azure Blob, GCS</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>scalable_performance_ops</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>15, 16</t>
+        </is>
+      </c>
+      <c r="T12" s="3" t="inlineStr">
+        <is>
+          <t>Cloud Object Storage | MUST HAVE; Cloud Object Storage | MUST HAVE</t>
+        </is>
+      </c>
+      <c r="U12" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V12" s="3" t="n"/>
+      <c r="W12" s="3" t="n"/>
+      <c r="X12" s="3" t="n"/>
+      <c r="Y12" s="3" t="n"/>
+      <c r="Z12" s="3" t="n"/>
+      <c r="AA12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>SCALE-013</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Cloud Data Warehouse Connections</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Snowflake Connection Configuration</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>For Snowflake connections, confirm the cloud storage connection's authentication is compatible with Automatic fast-write, and enable Spark native integration, UDF support, and Automatic fast-write. 'Details readable by' on the cloud storage connection is required for Snowpark and Spark Native integration; without it, users are limited to Visual and SQL recipes.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Enable Automatic fast-write, Spark native integration, and UDF support for Snowflake connections.</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Snowflake connection settings &gt; enableAutomaticFastWrite / enableSparkNativeIntegration / enableUDF, and cloud storage connection &gt; detailsReadableBy</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>equals</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>Cloud storage connection authentication must also meet the Automatic fast-write requirements per Dataiku documentation.</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>Snowflake connection shows Automatic fast-write, Spark native integration, and UDF enabled where applicable, and the cloud storage connection has 'Details readable by' enabled with compatible auth.</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>These settings disabled without justification, or cloud storage auth incompatible with fast-write requirements, limiting functionality (e.g., no Snowpark/Spark native access).</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>If Snowflake connection settings aren't present in the diagnosis, flag needs_manual_review and check Administration &gt; Connections for the Snowflake connection.</t>
+        </is>
+      </c>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>These settings enable performant, parallel data movement and advanced compute integration (Snowpark, Spark) rather than slow single-threaded funneling.</t>
+        </is>
+      </c>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>Snowflake, Automatic fast-write, Spark native integration, details readable by</t>
+        </is>
+      </c>
+      <c r="R13" s="3" t="inlineStr">
+        <is>
+          <t>scalable_performance_ops</t>
+        </is>
+      </c>
+      <c r="S13" s="3" t="inlineStr">
+        <is>
+          <t>16, 17</t>
+        </is>
+      </c>
+      <c r="T13" s="3" t="inlineStr">
+        <is>
+          <t>Snowflake | MUST HAVE; Snowflake | MUST HAVE</t>
+        </is>
+      </c>
+      <c r="U13" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V13" s="3" t="n"/>
+      <c r="W13" s="3" t="n"/>
+      <c r="X13" s="3" t="n"/>
+      <c r="Y13" s="3" t="n"/>
+      <c r="Z13" s="3" t="n"/>
+      <c r="AA13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>SCALE-014</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Cloud Data Warehouse Connections</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Databricks Connection Configuration</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>For Databricks connections, confirm the cloud storage connection's authentication is compatible with Automatic fast-write, and enable both Automatic fast-write and 'Details readable by' on the cloud storage connection.</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Enable Automatic fast-write and Details readable by for Databricks connections.</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Databricks connection settings &gt; enableAutomaticFastWrite, and cloud storage connection &gt; detailsReadableBy</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>equals</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="n"/>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>Cloud storage connection authentication must also meet the Automatic fast-write requirements per Dataiku documentation.</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>Databricks connection shows Automatic fast-write enabled, and the cloud storage connection has 'Details readable by' enabled with compatible auth.</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>Automatic fast-write or 'Details readable by' disabled, or cloud storage auth incompatible with fast-write requirements.</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>If Databricks connection settings aren't present in the diagnosis, flag needs_manual_review and check Administration &gt; Connections for the Databricks connection.</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>These settings enable performant, parallel data movement between DSS and Databricks rather than slow single-threaded funneling.</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>Databricks, Automatic fast-write, details readable by</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="inlineStr">
+        <is>
+          <t>scalable_performance_ops</t>
+        </is>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>17, 18</t>
+        </is>
+      </c>
+      <c r="T14" s="3" t="inlineStr">
+        <is>
+          <t>Databricks | MUST HAVE; Databricks | MUST HAVE</t>
+        </is>
+      </c>
+      <c r="U14" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V14" s="3" t="n"/>
+      <c r="W14" s="3" t="n"/>
+      <c r="X14" s="3" t="n"/>
+      <c r="Y14" s="3" t="n"/>
+      <c r="Z14" s="3" t="n"/>
+      <c r="AA14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>SCALE-015</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Cloud Data Warehouse Connections</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Amazon Redshift, Google BigQuery, Azure Synapse Connection Configuration</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>For Redshift, BigQuery, and Synapse connections, confirm the cloud storage connection's authentication is compatible with Automatic fast-write, and enable Automatic fast-write. Note that for Redshift, the Fast Path only applies to writing to Redshift, not to unload operations.</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Enable Automatic fast-write for Redshift, BigQuery, and Synapse connections.</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Redshift/BigQuery/Synapse connection settings &gt; enableAutomaticFastWrite</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>equals</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>Cloud storage connection authentication must also meet the Automatic fast-write requirements per Dataiku documentation; Redshift Fast Path is write-only and does not apply to unload.</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>Redshift/BigQuery/Synapse connection shows Automatic fast-write enabled and compatible cloud storage authentication.</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>Automatic fast-write disabled, or cloud storage auth incompatible with fast-write requirements.</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>If these connection settings aren't present in the diagnosis, flag needs_manual_review and check Administration &gt; Connections for the relevant connection.</t>
+        </is>
+      </c>
+      <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t>Automatic fast-write enables performant, parallel data movement rather than slow single-threaded funneling.</t>
+        </is>
+      </c>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>Redshift, BigQuery, Synapse, Automatic fast-write</t>
+        </is>
+      </c>
+      <c r="R15" s="3" t="inlineStr">
+        <is>
+          <t>scalable_performance_ops</t>
+        </is>
+      </c>
+      <c r="S15" s="3" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="T15" s="3" t="inlineStr">
+        <is>
+          <t>Amazon Redshift, Google BigQuery, Azure Synapse | MUST HAVE</t>
+        </is>
+      </c>
+      <c r="U15" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V15" s="3" t="n"/>
+      <c r="W15" s="3" t="n"/>
+      <c r="X15" s="3" t="n"/>
+      <c r="Y15" s="3" t="n"/>
+      <c r="Z15" s="3" t="n"/>
+      <c r="AA15" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Release 0.38.3: GENAI-002, GENAI-011, SEC-003 ruled (65 of 67); ARCH-002/003 stay with the model
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/checklists/eval_checklist.xlsx
+++ b/tests/fixtures/checklists/eval_checklist.xlsx
@@ -3095,7 +3095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA9"/>
+  <dimension ref="A1:AA10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3376,7 +3376,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>GENAI-003</t>
+          <t>GENAI-002</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -3391,27 +3391,27 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Trace Explorer</t>
+          <t>LLM Mesh and Agents</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Trace Explorer Default Configuration</t>
+          <t>Hugging Face Local LLM Enablement (Conditional)</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Configure Trace Explorer via Administration &gt; Settings &gt; Other &gt; LLM Mesh &gt; Configuration &gt; Trace by setting a default Project and Trace Explorer webapp instance, so the 'view traces' shortcut is functional from Prompt Studio, Agents, and Retrieval-Augmented LLMs.</t>
+          <t>When the customer uses Hugging Face local LLMs, ensure the INTERNAL_huggingface_local_v1 code env is installed and that technical prerequisites are met: a running Elastic AI Kubernetes cluster with NVIDIA GPUs (compute capability &gt;= 7.0, driver compatible with CUDA 12.8), Almalinux 9 base images, and Python 3.11.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Set a default project and webapp for Trace Explorer so view traces works.</t>
+          <t>Install the Hugging Face code env and verify GPU cluster prerequisites when used.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; generativeAISettings &gt; llmTraceSettings.traceExplorerDefaultWebApp</t>
+          <t>Administration &gt; Code-envs &gt; INTERNAL_huggingface_local_v1 (installed)</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -3421,34 +3421,38 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>projectKey and webAppId both set to non-empty values</t>
+          <t>installed and configured</t>
         </is>
       </c>
       <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>No literal diag JSON field was given in the source for this check; infrastructure prerequisites (GPU compute capability, CUDA/driver version, Python 3.11, Almalinux 9) are not verifiable from a diagnosis JSON alone and require manual/infra review.</t>
+        </is>
+      </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>generativeAISettings.llmTraceSettings.traceExplorerDefaultWebApp present in general-settings.json with non-empty projectKey and webAppId fields.</t>
+          <t>Code-env listing shows INTERNAL_huggingface_local_v1 present and in use; Elastic AI cluster configuration references GPU-enabled nodes.</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>llmTraceSettings missing entirely, or traceExplorerDefaultWebApp present but empty/null.</t>
+          <t>Env missing, or Hugging Face local LLM feature is referenced in use without a corresponding GPU-enabled Elastic AI cluster.</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>If general-settings.json content isn't captured in the diagnosis, flag needs_manual_review to verify via the UI.</t>
+          <t>If the diagnosis doesn't reference Hugging Face local LLM usage, treat as not applicable; if usage is confirmed elsewhere but infra details aren't in the diagnosis, flag needs_manual_review.</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>Without this default configuration, the trace-viewing shortcut from Prompt Studio/Agents/RAG LLMs will not function.</t>
+          <t>Without the correct GPU cluster, driver/CUDA compatibility, base image, and Python version, local Hugging Face LLMs will not function.</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>Trace Explorer, LLM Mesh, Agents</t>
+          <t>Hugging Face, Elastic AI, Kubernetes, GPU, code environments</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
@@ -3458,20 +3462,24 @@
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
-          <t>3, 4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>Trace Explorer MUST HAVE:; Instance Diags / DiagParser3</t>
+          <t>Hugging face local LLMs (only if applicable)</t>
         </is>
       </c>
       <c r="U3" s="3" t="inlineStr">
         <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="V3" s="3" t="n"/>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>Conditional feature ('only if applicable'); priority applies only when the customer has opted to use this capability.</t>
+        </is>
+      </c>
       <c r="W3" s="3" t="n"/>
       <c r="X3" s="3" t="n"/>
       <c r="Y3" s="3" t="n"/>
@@ -3481,12 +3489,12 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>GENAI-004</t>
+          <t>GENAI-003</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>nice_to_have</t>
+          <t>must_have</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -3496,64 +3504,64 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>AI Services</t>
+          <t>Trace Explorer</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>AI Services Terms of Use Acceptance &amp; Enablement</t>
+          <t>Trace Explorer Default Configuration</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Verify that the customer has accepted the Dataiku AI Services Terms of Use and that AI Services are enabled by the admin in Administration &gt; AI Services. Confirm outbound internet connectivity to https://ai-gateway.api-services.dataiku.io, required in both 'Operated by Dataiku' and 'Bring your own LLM' modes.</t>
+          <t>Configure Trace Explorer via Administration &gt; Settings &gt; Other &gt; LLM Mesh &gt; Configuration &gt; Trace by setting a default Project and Trace Explorer webapp instance, so the 'view traces' shortcut is functional from Prompt Studio, Agents, and Retrieval-Augmented LLMs.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Confirm AI Services Terms of Use are accepted and AI Services are enabled.</t>
+          <t>Set a default project and webapp for Trace Explorer so view traces works.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; dataikuAIServicesTermsOfUseAccepted / enabled</t>
+          <t>general-settings.json &gt; generativeAISettings &gt; llmTraceSettings.traceExplorerDefaultWebApp</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>equals</t>
+          <t>exists</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>projectKey and webAppId both set to non-empty values</t>
         </is>
       </c>
       <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>Also check byoTermsOfUseAccepted for Bring-your-own-LLM mode. Internet whitelisting of ai-gateway.api-services.dataiku.io is not verifiable from diagnosis JSON alone.</t>
-        </is>
-      </c>
+      <c r="L4" s="3" t="n"/>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json shows dataikuAIServicesTermsOfUseAccepted=true and enabled=true.</t>
+          <t>generativeAISettings.llmTraceSettings.traceExplorerDefaultWebApp present in general-settings.json with non-empty projectKey and webAppId fields.</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>enabled=false or Terms of Use not accepted while AI Services usage is expected/observed.</t>
+          <t>llmTraceSettings missing entirely, or traceExplorerDefaultWebApp present but empty/null.</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>If AI Services keys are absent from the diagnosis, treat as not enabled and flag needs_manual_review to confirm with the customer whether AI Services usage is intended.</t>
-        </is>
-      </c>
-      <c r="P4" s="3" t="n"/>
+          <t>If general-settings.json content isn't captured in the diagnosis, flag needs_manual_review to verify via the UI.</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>Without this default configuration, the trace-viewing shortcut from Prompt Studio/Agents/RAG LLMs will not function.</t>
+        </is>
+      </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>AI Services, Terms of Use, LLM Mesh</t>
+          <t>Trace Explorer, LLM Mesh, Agents</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
@@ -3563,12 +3571,12 @@
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>4, 5</t>
+          <t>3, 4</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>AI Services NICE TO HAVE:; Instance Diags / DiagParser3</t>
+          <t>Trace Explorer MUST HAVE:; Instance Diags / DiagParser3</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
@@ -3586,12 +3594,12 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>GENAI-005</t>
+          <t>GENAI-004</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -3601,60 +3609,64 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Bring Your Own LLM Mode</t>
+          <t>AI Services</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Bring Your Own LLM Mode - Reference Project &amp; Main Model</t>
+          <t>AI Services Terms of Use Acceptance &amp; Enablement</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>When Bring Your Own LLM mode is active, a Reference project key must be set (used for LLM Mesh requests running outside a DSS project, e.g. AI Search) and a main LLM model must be configured; if unset, requests will fail.</t>
+          <t>Verify that the customer has accepted the Dataiku AI Services Terms of Use and that AI Services are enabled by the admin in Administration &gt; AI Services. Confirm outbound internet connectivity to https://ai-gateway.api-services.dataiku.io, required in both 'Operated by Dataiku' and 'Bring your own LLM' modes.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Set a Reference project key and main LLM model when using Bring Your Own LLM.</t>
+          <t>Confirm AI Services Terms of Use are accepted and AI Services are enabled.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; localAIServerSettings.referenceProjectKey / mainLLMId</t>
+          <t>general-settings.json &gt; dataikuAIServicesTermsOfUseAccepted / enabled</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>exists</t>
+          <t>equals</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>non-empty values set for both fields</t>
+          <t>true</t>
         </is>
       </c>
       <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Also check byoTermsOfUseAccepted for Bring-your-own-LLM mode. Internet whitelisting of ai-gateway.api-services.dataiku.io is not verifiable from diagnosis JSON alone.</t>
+        </is>
+      </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>localAIServerSettings.useLocalServer=true with referenceProjectKey and mainLLMId populated (e.g., 'openai:openai-adrissi:gpt-5.5').</t>
+          <t>general-settings.json shows dataikuAIServicesTermsOfUseAccepted=true and enabled=true.</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>useLocalServer=true but referenceProjectKey or mainLLMId missing or empty.</t>
+          <t>enabled=false or Terms of Use not accepted while AI Services usage is expected/observed.</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>If localAIServerSettings is absent from the diagnosis, flag needs_manual_review to confirm whether Bring Your Own LLM mode is in use.</t>
+          <t>If AI Services keys are absent from the diagnosis, treat as not enabled and flag needs_manual_review to confirm with the customer whether AI Services usage is intended.</t>
         </is>
       </c>
       <c r="P5" s="3" t="n"/>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>Bring Your Own LLM, AI Services, LLM Mesh</t>
+          <t>AI Services, Terms of Use, LLM Mesh</t>
         </is>
       </c>
       <c r="R5" s="3" t="inlineStr">
@@ -3664,12 +3676,12 @@
       </c>
       <c r="S5" s="3" t="inlineStr">
         <is>
-          <t>5, 6</t>
+          <t>4, 5</t>
         </is>
       </c>
       <c r="T5" s="3" t="inlineStr">
         <is>
-          <t>Bring your own LLM Mode; Instance Diags / DiagParser3</t>
+          <t>AI Services NICE TO HAVE:; Instance Diags / DiagParser3</t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr">
@@ -3687,12 +3699,12 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>GENAI-006</t>
+          <t>GENAI-005</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>nice_to_have</t>
+          <t>must_have</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -3707,63 +3719,55 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Bring Your Own LLM - Recommended Model Versions</t>
+          <t>Bring Your Own LLM Mode - Reference Project &amp; Main Model</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>If the customer has activated Bring Your Own LLM Mode for AI Assistants, verify they are using recommended model versions (minimum OpenAI ChatGPT 5.2) and avoid unsupported ones (e.g., ChatGPT 5.1, which will not provide good results).</t>
+          <t>When Bring Your Own LLM mode is active, a Reference project key must be set (used for LLM Mesh requests running outside a DSS project, e.g. AI Search) and a main LLM model must be configured; if unset, requests will fail.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Use at least ChatGPT 5.2 for Bring Your Own LLM; avoid version 5.1.</t>
+          <t>Set a Reference project key and main LLM model when using Bring Your Own LLM.</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; localAIServerSettings.mainLLMId (and responseFormatAwareLLMId/fastLightLLMId)</t>
+          <t>general-settings.json &gt; localAIServerSettings.referenceProjectKey / mainLLMId</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>not_equals</t>
+          <t>exists</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>ChatGPT 5.1 or earlier / unsupported model versions</t>
+          <t>non-empty values set for both fields</t>
         </is>
       </c>
       <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>Exact version comparison against the recommended minimum (ChatGPT 5.2) may require manual judgment; refer to https://doc.dataiku.com/dss/latest/ai-assistants/setup.html#bring-your-own-llm-mode.</t>
-        </is>
-      </c>
+      <c r="L6" s="3" t="n"/>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>mainLLMId/related LLM IDs reference gpt-5.2 or later.</t>
+          <t>localAIServerSettings.useLocalServer=true with referenceProjectKey and mainLLMId populated (e.g., 'openai:openai-adrissi:gpt-5.5').</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>mainLLMId/related LLM IDs reference gpt-5.1 or an older/unsupported model.</t>
+          <t>useLocalServer=true but referenceProjectKey or mainLLMId missing or empty.</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>If the model identifier is ambiguous, non-OpenAI, or version cannot be determined, flag needs_manual_review and reference the setup documentation.</t>
-        </is>
-      </c>
-      <c r="P6" s="3" t="inlineStr">
-        <is>
-          <t>Using unsupported model versions is stated to produce poor results.</t>
-        </is>
-      </c>
+          <t>If localAIServerSettings is absent from the diagnosis, flag needs_manual_review to confirm whether Bring Your Own LLM mode is in use.</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="n"/>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>Bring Your Own LLM, Model selection, AI Assistants</t>
+          <t>Bring Your Own LLM, AI Services, LLM Mesh</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
@@ -3773,17 +3777,17 @@
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>6, 7</t>
+          <t>5, 6</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>Bring your own LLM Mode; Bring your own LLM Mode</t>
+          <t>Bring your own LLM Mode; Instance Diags / DiagParser3</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="V6" s="3" t="n"/>
@@ -3796,12 +3800,12 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>GENAI-007</t>
+          <t>GENAI-006</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -3811,60 +3815,68 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Cobuild</t>
+          <t>Bring Your Own LLM Mode</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Cobuild Default LLM Configuration</t>
+          <t>Bring Your Own LLM - Recommended Model Versions</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Administrators must configure default LLM settings for Cobuild (agent-building tools) upon activation of AI Assistants, including defaultEmbeddingLLMId, defaultLLMId, and defaultImageGenerationLLMId under agentBuildingSettings; if unset, Cobuild's building-agent tools will fail and instruct users to contact an administrator.</t>
+          <t>If the customer has activated Bring Your Own LLM Mode for AI Assistants, verify they are using recommended model versions (minimum OpenAI ChatGPT 5.2) and avoid unsupported ones (e.g., ChatGPT 5.1, which will not provide good results).</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Configure default embedding, LLM, and image-generation models for Cobuild agent building.</t>
+          <t>Use at least ChatGPT 5.2 for Bring Your Own LLM; avoid version 5.1.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; aiDrivenAnalyticsSettings.agentBuildingSettings.{defaultEmbeddingLLMId, defaultLLMId, defaultImageGenerationLLMId}</t>
+          <t>general-settings.json &gt; localAIServerSettings.mainLLMId (and responseFormatAwareLLMId/fastLightLLMId)</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>exists</t>
+          <t>not_equals</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>all three fields populated with valid LLM IDs</t>
+          <t>ChatGPT 5.1 or earlier / unsupported model versions</t>
         </is>
       </c>
       <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Exact version comparison against the recommended minimum (ChatGPT 5.2) may require manual judgment; refer to https://doc.dataiku.com/dss/latest/ai-assistants/setup.html#bring-your-own-llm-mode.</t>
+        </is>
+      </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>agentBuildingSettings block shows non-empty defaultEmbeddingLLMId, defaultLLMId, and defaultImageGenerationLLMId values.</t>
+          <t>mainLLMId/related LLM IDs reference gpt-5.2 or later.</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>One or more of these fields is missing or empty while Cobuild/AI Assistants is enabled.</t>
+          <t>mainLLMId/related LLM IDs reference gpt-5.1 or an older/unsupported model.</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>If aiDrivenAnalyticsSettings is absent from the diagnosis, flag needs_manual_review to confirm whether Cobuild/AI Assistants is enabled for this customer.</t>
-        </is>
-      </c>
-      <c r="P7" s="3" t="n"/>
+          <t>If the model identifier is ambiguous, non-OpenAI, or version cannot be determined, flag needs_manual_review and reference the setup documentation.</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>Using unsupported model versions is stated to produce poor results.</t>
+        </is>
+      </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>Cobuild, AI Assistants, Agent building</t>
+          <t>Bring Your Own LLM, Model selection, AI Assistants</t>
         </is>
       </c>
       <c r="R7" s="3" t="inlineStr">
@@ -3874,17 +3886,17 @@
       </c>
       <c r="S7" s="3" t="inlineStr">
         <is>
-          <t>7, 8, 9</t>
+          <t>6, 7</t>
         </is>
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>Cobuild; Cobuild; Instance Diags / DiagParser3</t>
+          <t>Bring your own LLM Mode; Bring your own LLM Mode</t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="V7" s="3" t="n"/>
@@ -3897,7 +3909,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>GENAI-008</t>
+          <t>GENAI-007</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -3907,57 +3919,65 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>qualitative_practice</t>
+          <t>specific_setting</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>AI Assistants Diagnostics</t>
+          <t>Cobuild</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Include AI Assistant Debug Data in Instance Diagnostics</t>
+          <t>Cobuild Default LLM Configuration</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>To access AI Assistant Logs (ui.json, runtime.json, traces per project) in an Instance Diagnostic (V14.7+), an administrator must explicitly select the option to include these logs when generating a diagnostic via Administration &gt; Maintenance &gt; Instance Diagnostic.</t>
+          <t>Administrators must configure default LLM settings for Cobuild (agent-building tools) upon activation of AI Assistants, including defaultEmbeddingLLMId, defaultLLMId, and defaultImageGenerationLLMId under agentBuildingSettings; if unset, Cobuild's building-agent tools will fail and instruct users to contact an administrator.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Select the option to include AI Assistant debug logs when generating instance diagnostics.</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="n"/>
+          <t>Configure default embedding, LLM, and image-generation models for Cobuild agent building.</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; aiDrivenAnalyticsSettings.agentBuildingSettings.{defaultEmbeddingLLMId, defaultLLMId, defaultImageGenerationLLMId}</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>exists</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>all three fields populated with valid LLM IDs</t>
+        </is>
+      </c>
       <c r="K8" s="3" t="n"/>
       <c r="L8" s="3" t="n"/>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>The diagnostic bundle includes an 'AI Assistants debug data' section organized by project with ui.json, runtime.json, and traces files.</t>
+          <t>agentBuildingSettings block shows non-empty defaultEmbeddingLLMId, defaultLLMId, and defaultImageGenerationLLMId values.</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>Diagnostic bundle lacks these files despite AI Assistants being actively used on the instance.</t>
+          <t>One or more of these fields is missing or empty while Cobuild/AI Assistants is enabled.</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>If the diagnostic was generated on a version prior to 14.7, or the inclusion option's state can't be determined, flag needs_manual_review and note reviewers should confirm the option was selected during diagnostic generation.</t>
-        </is>
-      </c>
-      <c r="P8" s="3" t="inlineStr">
-        <is>
-          <t>Without selecting this option, AI Assistant logs are not captured, limiting the reviewer's ability to diagnose LLM Mesh/agent-building issues.</t>
-        </is>
-      </c>
+          <t>If aiDrivenAnalyticsSettings is absent from the diagnosis, flag needs_manual_review to confirm whether Cobuild/AI Assistants is enabled for this customer.</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="n"/>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>Instance Diagnostic, AI Assistants, Logging</t>
+          <t>Cobuild, AI Assistants, Agent building</t>
         </is>
       </c>
       <c r="R8" s="3" t="inlineStr">
@@ -3967,24 +3987,20 @@
       </c>
       <c r="S8" s="3" t="inlineStr">
         <is>
-          <t>9, 10</t>
+          <t>7, 8, 9</t>
         </is>
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>Instance Diags / DiagParser3; Instance Diags / DiagParser3</t>
+          <t>Cobuild; Cobuild; Instance Diags / DiagParser3</t>
         </is>
       </c>
       <c r="U8" s="3" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="V8" s="3" t="inlineStr">
-        <is>
-          <t>This is more a diagnostic-generation process note than a platform configuration state, so evaluability from a static diagnosis file is limited.</t>
-        </is>
-      </c>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V8" s="3" t="n"/>
       <c r="W8" s="3" t="n"/>
       <c r="X8" s="3" t="n"/>
       <c r="Y8" s="3" t="n"/>
@@ -3994,12 +4010,12 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>GENAI-009</t>
+          <t>GENAI-008</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>nice_to_have</t>
+          <t>must_have</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -4009,22 +4025,22 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Agent Hub</t>
+          <t>AI Assistants Diagnostics</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Agent Hub Deployment Required Permissions</t>
+          <t>Include AI Assistant Debug Data in Instance Diagnostics</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Before a user can deploy an Agent Hub instance, they must have permissions for writing project content in the hosting project, writing isolated code execution, WebApp impersonation, and (if Quick agents are enabled) create projects; alternatively the user could be a DSS administrator, though a dedicated service account is preferred.</t>
+          <t>To access AI Assistant Logs (ui.json, runtime.json, traces per project) in an Instance Diagnostic (V14.7+), an administrator must explicitly select the option to include these logs when generating a diagnostic via Administration &gt; Maintenance &gt; Instance Diagnostic.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Grant Agent Hub deployers write project content, isolated code execution, and webapp impersonation permissions.</t>
+          <t>Select the option to include AI Assistant debug logs when generating instance diagnostics.</t>
         </is>
       </c>
       <c r="H9" s="3" t="n"/>
@@ -4034,27 +4050,27 @@
       <c r="L9" s="3" t="n"/>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>Administration &gt; Security &gt; Groups shows the Agent Hub deployer's group granted 'Write project content', 'Write isolated code execution', and 'WebApp impersonation' permissions (plus 'Create projects' if Quick agents are enabled), or the deployer is a DSS admin/service account.</t>
+          <t>The diagnostic bundle includes an 'AI Assistants debug data' section organized by project with ui.json, runtime.json, and traces files.</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>The deployer's group lacks one or more of these permissions and is not an admin/service account, or logs show 'Not authorized' errors when creating the Agent Hub WebApp.</t>
+          <t>Diagnostic bundle lacks these files despite AI Assistants being actively used on the instance.</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file lacks per-user/group permission detail, flag needs_manual_review and recommend checking Administration &gt; Security &gt; Groups directly.</t>
+          <t>If the diagnostic was generated on a version prior to 14.7, or the inclusion option's state can't be determined, flag needs_manual_review and note reviewers should confirm the option was selected during diagnostic generation.</t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>Missing permissions cause deployment failures such as 'Not authorized' errors when creating the Agent Hub WebApp.</t>
+          <t>Without selecting this option, AI Assistant logs are not captured, limiting the reviewer's ability to diagnose LLM Mesh/agent-building issues.</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>Agent Hub, Permissions, Groups, WebApp</t>
+          <t>Instance Diagnostic, AI Assistants, Logging</t>
         </is>
       </c>
       <c r="R9" s="3" t="inlineStr">
@@ -4064,22 +4080,22 @@
       </c>
       <c r="S9" s="3" t="inlineStr">
         <is>
-          <t>10, 11, 12</t>
+          <t>9, 10</t>
         </is>
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>Agent Hub NICE TO HAVE:; Writing isolated code execution; WebApp impersonation</t>
+          <t>Instance Diags / DiagParser3; Instance Diags / DiagParser3</t>
         </is>
       </c>
       <c r="U9" s="3" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="V9" s="3" t="inlineStr">
         <is>
-          <t>Although the parent topic is tagged NICE TO HAVE, the described permission requirements are phrased as mandatory ('must have permissions') for successful deployment; classification follows the explicit heading tag.</t>
+          <t>This is more a diagnostic-generation process note than a platform configuration state, so evaluability from a static diagnosis file is limited.</t>
         </is>
       </c>
       <c r="W9" s="3" t="n"/>
@@ -4087,6 +4103,103 @@
       <c r="Y9" s="3" t="n"/>
       <c r="Z9" s="3" t="n"/>
       <c r="AA9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>GENAI-009</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>nice_to_have</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>qualitative_practice</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub Deployment Required Permissions</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Before a user can deploy an Agent Hub instance, they must have permissions for writing project content in the hosting project, writing isolated code execution, WebApp impersonation, and (if Quick agents are enabled) create projects; alternatively the user could be a DSS administrator, though a dedicated service account is preferred.</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Grant Agent Hub deployers write project content, isolated code execution, and webapp impersonation permissions.</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="n"/>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="n"/>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>Administration &gt; Security &gt; Groups shows the Agent Hub deployer's group granted 'Write project content', 'Write isolated code execution', and 'WebApp impersonation' permissions (plus 'Create projects' if Quick agents are enabled), or the deployer is a DSS admin/service account.</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>The deployer's group lacks one or more of these permissions and is not an admin/service account, or logs show 'Not authorized' errors when creating the Agent Hub WebApp.</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file lacks per-user/group permission detail, flag needs_manual_review and recommend checking Administration &gt; Security &gt; Groups directly.</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>Missing permissions cause deployment failures such as 'Not authorized' errors when creating the Agent Hub WebApp.</t>
+        </is>
+      </c>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub, Permissions, Groups, WebApp</t>
+        </is>
+      </c>
+      <c r="R10" s="3" t="inlineStr">
+        <is>
+          <t>generative_ai_acceleration</t>
+        </is>
+      </c>
+      <c r="S10" s="3" t="inlineStr">
+        <is>
+          <t>10, 11, 12</t>
+        </is>
+      </c>
+      <c r="T10" s="3" t="inlineStr">
+        <is>
+          <t>Agent Hub NICE TO HAVE:; Writing isolated code execution; WebApp impersonation</t>
+        </is>
+      </c>
+      <c r="U10" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="V10" s="3" t="inlineStr">
+        <is>
+          <t>Although the parent topic is tagged NICE TO HAVE, the described permission requirements are phrased as mandatory ('must have permissions') for successful deployment; classification follows the explicit heading tag.</t>
+        </is>
+      </c>
+      <c r="W10" s="3" t="n"/>
+      <c r="X10" s="3" t="n"/>
+      <c r="Y10" s="3" t="n"/>
+      <c r="Z10" s="3" t="n"/>
+      <c r="AA10" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
ARCH-009/012: Not Applicable with no cluster attached, else Needs Review (moved from rules_review.py to rules_k8s.py)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/checklists/eval_checklist.xlsx
+++ b/tests/fixtures/checklists/eval_checklist.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA16"/>
+  <dimension ref="A1:AA18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1409,7 +1409,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>ARCH-010</t>
+          <t>ARCH-009</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1419,73 +1419,57 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>specific_setting</t>
+          <t>qualitative_practice</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Containerized Execution</t>
+          <t>Network Connectivity</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Valid Containerized Execution Configuration</t>
+          <t>Bidirectional Network Connectivity Between DSS and Elastic AI Cluster</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Environments using Elastic Compute (Kubernetes) must have at least one valid containerized execution configuration set up (general-settings.json &gt; containerSettings, or Administration &gt; Settings &gt; Containerized execution); as with Spark, the specific example values are only a baseline, not a strict requirement.</t>
+          <t>Full bidirectional network connectivity between DSS and the Kubernetes/Elastic AI cluster is mandatory: workers must be able to reach Dataiku (required for Spark to start and for any container execution), and Dataiku must be able to reach workers (required for operations that bring data back to the driver, e.g. toPandas/collect/head/show/broadcast join). This should be validated by running a pySpark recipe that pulls data back to the driver and confirming success via the Main Activity Log.</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Configure at least one valid containerized execution config when using Elastic Compute.</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>general-settings.json &gt; containerSettings</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>exists</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>valid containerized execution configuration present</t>
-        </is>
-      </c>
+          <t>Ensure full bidirectional network connectivity between DSS and the Elastic AI cluster.</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="n"/>
       <c r="K10" s="3" t="n"/>
-      <c r="L10" s="3" t="inlineStr">
-        <is>
-          <t>Required only when the customer uses Elastic Compute/Kubernetes for offloaded workloads.</t>
-        </is>
-      </c>
+      <c r="L10" s="3" t="n"/>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>containerSettings block is present with at least one named config with reasonable memory requests/limits.</t>
+          <t>A pySpark recipe using collect/head/show/toPandas completes successfully, with a corresponding HEAD operation visible in the Main Activity Log, and no worker-to-DSS or DSS-to-worker connectivity errors appear in logs.</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>containerSettings is missing or empty while the instance shows evidence of Kubernetes-based execution elsewhere in the diagnosis.</t>
+          <t>Connection timeouts or errors between workers and the DSS host in logs, or driver-return operations failing/hanging.</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not clarify whether Elastic Compute is used, flag needs_manual_review.</t>
+          <t>If the diagnosis file lacks job logs or network topology details, flag needs_manual_review and recommend running the described test recipe.</t>
         </is>
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>A valid container exec config is required to run workloads in Kubernetes.</t>
+          <t>Both directions of connectivity are mandatory prerequisites for Spark to start and for common data-return operations to work.</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>Containerized execution, containerSettings, Elastic Compute</t>
+          <t>Spark driver, Spark workers, Network connectivity, Kubernetes</t>
         </is>
       </c>
       <c r="R10" s="3" t="inlineStr">
@@ -1495,12 +1479,12 @@
       </c>
       <c r="S10" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>Containerized execution configs | MUST HAVE if using Elastic Compute</t>
+          <t>Connectivity between Dataiku and Elastic AI must be fully open MUST HAVE</t>
         </is>
       </c>
       <c r="U10" s="3" t="inlineStr">
@@ -1518,12 +1502,12 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>ARCH-011</t>
+          <t>ARCH-010</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>nice_to_have</t>
+          <t>must_have</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1538,67 +1522,63 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Baseline Container Execution Configs (Standard, Webapp) and Namespace Settings</t>
+          <t>Valid Containerized Execution Configuration</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Dataiku recommends at least two named containerized execution configs as a baseline - a Standard config for notebooks/recipes/ML (memory request 200MB, memory limit 16000MB) and a Webapp config for webapps (memory request 500MB, memory limit 500MB) - plus per-user Kubernetes namespaces (dss-ns-${dssUserLogin}) with K8s-compliant naming and auto-creation, and using the Webapp config for virtual webapp backends run in containers.</t>
+          <t>Environments using Elastic Compute (Kubernetes) must have at least one valid containerized execution configuration set up (general-settings.json &gt; containerSettings, or Administration &gt; Settings &gt; Containerized execution); as with Spark, the specific example values are only a baseline, not a strict requirement.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Define Standard and Webapp container execution configs plus per-user Kubernetes namespaces.</t>
+          <t>Configure at least one valid containerized execution config when using Elastic Compute.</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; containerSettings (named container exec configs)</t>
+          <t>general-settings.json &gt; containerSettings</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>one_of</t>
+          <t>exists</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Standard config (memory request 200MB / limit 16000MB) and Webapp config (memory request 500MB / limit 500MB)</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>MB</t>
-        </is>
-      </c>
+          <t>valid containerized execution configuration present</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="n"/>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>Additional recommended settings: one Kubernetes namespace per user (dss-ns-${dssUserLogin}), K8s-compliant namespace names, auto-create namespaces, and virtual webapps configured to run in a container using the Webapp config.</t>
+          <t>Required only when the customer uses Elastic Compute/Kubernetes for offloaded workloads.</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>containerSettings includes configs resembling the Standard and Webapp purposes with comparable memory request/limit values, and namespace settings follow a per-user pattern.</t>
+          <t>containerSettings block is present with at least one named config with reasonable memory requests/limits.</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>A single undifferentiated container config is used for both interactive workloads and webapps, or all users share one namespace.</t>
+          <t>containerSettings is missing or empty while the instance shows evidence of Kubernetes-based execution elsewhere in the diagnosis.</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not list named container configs or namespace settings, flag needs_manual_review.</t>
+          <t>If the diagnosis file does not clarify whether Elastic Compute is used, flag needs_manual_review.</t>
         </is>
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>Separating configs by workload type avoids over- or under-provisioning; per-user namespaces aid isolation and cost tracking.</t>
+          <t>A valid container exec config is required to run workloads in Kubernetes.</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>Containerized execution, Kubernetes namespace, Webapp backend</t>
+          <t>Containerized execution, containerSettings, Elastic Compute</t>
         </is>
       </c>
       <c r="R11" s="3" t="inlineStr">
@@ -1608,12 +1588,12 @@
       </c>
       <c r="S11" s="3" t="inlineStr">
         <is>
-          <t>8, 9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="T11" s="3" t="inlineStr">
         <is>
-          <t>Recommendations NICE TO HAVE; Recommended Settings</t>
+          <t>Containerized execution configs | MUST HAVE if using Elastic Compute</t>
         </is>
       </c>
       <c r="U11" s="3" t="inlineStr">
@@ -1631,12 +1611,12 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>ARCH-013</t>
+          <t>ARCH-011</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1646,64 +1626,72 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Cluster Configuration</t>
+          <t>Containerized Execution</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Valid Cluster Configuration for Elastic Compute</t>
+          <t>Baseline Container Execution Configs (Standard, Webapp) and Namespace Settings</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Environments using Elastic Compute must have at least one valid cluster configured (found under {DATADIR}/config/clusters or Administration &gt; Clusters); Dataiku does not mandate the specific example configuration, only that a workable cluster exists.</t>
+          <t>Dataiku recommends at least two named containerized execution configs as a baseline - a Standard config for notebooks/recipes/ML (memory request 200MB, memory limit 16000MB) and a Webapp config for webapps (memory request 500MB, memory limit 500MB) - plus per-user Kubernetes namespaces (dss-ns-${dssUserLogin}) with K8s-compliant naming and auto-creation, and using the Webapp config for virtual webapp backends run in containers.</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Configure at least one valid Kubernetes cluster when using Elastic Compute.</t>
+          <t>Define Standard and Webapp container execution configs plus per-user Kubernetes namespaces.</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>{DATADIR}/config/clusters</t>
+          <t>general-settings.json &gt; containerSettings (named container exec configs)</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>exists</t>
+          <t>one_of</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>at least one valid cluster configuration present</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="n"/>
-      <c r="L12" s="3" t="n"/>
+          <t>Standard config (memory request 200MB / limit 16000MB) and Webapp config (memory request 500MB / limit 500MB)</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>Additional recommended settings: one Kubernetes namespace per user (dss-ns-${dssUserLogin}), K8s-compliant namespace names, auto-create namespaces, and virtual webapps configured to run in a container using the Webapp config.</t>
+        </is>
+      </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>The clusters config/directory contains at least one properly defined cluster, consistent with other evidence of elastic-compute usage (spark/container jobs running on Kubernetes).</t>
+          <t>containerSettings includes configs resembling the Standard and Webapp purposes with comparable memory request/limit values, and namespace settings follow a per-user pattern.</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>No cluster configuration is present despite evidence of Kubernetes-based workloads elsewhere in the diagnosis.</t>
+          <t>A single undifferentiated container config is used for both interactive workloads and webapps, or all users share one namespace.</t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not clarify whether Elastic Compute is used at all, flag needs_manual_review.</t>
+          <t>If the diagnosis file does not list named container configs or namespace settings, flag needs_manual_review.</t>
         </is>
       </c>
       <c r="P12" s="3" t="inlineStr">
         <is>
-          <t>A valid cluster is required to offload computation to Kubernetes.</t>
+          <t>Separating configs by workload type avoids over- or under-provisioning; per-user namespaces aid isolation and cost tracking.</t>
         </is>
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>Cluster, Managed cluster, Unmanaged cluster, Elastic AI</t>
+          <t>Containerized execution, Kubernetes namespace, Webapp backend</t>
         </is>
       </c>
       <c r="R12" s="3" t="inlineStr">
@@ -1713,12 +1701,12 @@
       </c>
       <c r="S12" s="3" t="inlineStr">
         <is>
-          <t>12, 13</t>
+          <t>8, 9</t>
         </is>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>Cluster configurations | MUST HAVE if using Elastic Compute; Cluster configurations | MUST HAVE if using Elastic Compute</t>
+          <t>Recommendations NICE TO HAVE; Recommended Settings</t>
         </is>
       </c>
       <c r="U12" s="3" t="inlineStr">
@@ -1736,83 +1724,67 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>ARCH-014</t>
+          <t>ARCH-012</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>nice_to_have</t>
+          <t>must_have</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>specific_setting</t>
+          <t>qualitative_practice</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Cluster Configuration</t>
+          <t>Containerized Execution Validation</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Recommended Cluster Topology (Single Managed Cluster, Node Groups, Autoscaling)</t>
+          <t>Functional Validation of Containerized Execution Across Recipe, Notebook, Webapp, and API</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Dataiku recommends a single managed cluster with one CPU node group serving containerized execution, ML, Spark, webapp, and API workloads, adding a separate GPU node group only if needed, and enabling a metrics server plus cluster autoscaling.</t>
+          <t>Reviewers should validate containerized execution end-to-end: execute a recipe in Kubernetes, launch a notebook in the cluster (pod visible in Cluster Monitoring UI), create a test webapp configured with a container backend (deployment visible in Cluster Monitoring UI), and deploy an API service to Kubernetes via the API Deployer (deployment visible in Cluster Monitoring UI and callable via sample code).</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Use a single managed cluster with one CPU node group and autoscaling enabled.</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>{DATADIR}/config/clusters (cluster topology / node group / autoscaling settings)</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>equals</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>single managed cluster, one CPU node group for all standard workloads, optional GPU node group only if needed, metrics server installed, autoscaling enabled</t>
-        </is>
-      </c>
+          <t>Validate containerized execution works for recipes, notebooks, webapps, and API deployments.</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="n"/>
+      <c r="J13" s="3" t="n"/>
       <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="inlineStr">
-        <is>
-          <t>No literal single field was given for this recommendation; pointer is a best-effort conceptual location within the clusters config.</t>
-        </is>
-      </c>
+      <c r="L13" s="3" t="n"/>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>Cluster configuration shows one managed cluster with a shared CPU node group, autoscaling enabled, metrics server installed, and a GPU node group only present when GPU workloads exist.</t>
+          <t>Cluster monitoring evidence or reviewer test logs show successful recipe execution, a notebook pod, a webapp deployment, and an API deployment all running in Kubernetes, with the API additionally callable via sample code.</t>
         </is>
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>Multiple redundant clusters/node groups without clear justification, no autoscaling enabled, or a GPU node group present without any GPU workload evidence.</t>
+          <t>Any of the four (recipe, notebook, webapp, API) fails to launch, or no corresponding pods/deployments ever appear in Cluster Monitoring.</t>
         </is>
       </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not detail node groups or autoscaling settings, flag needs_manual_review.</t>
+          <t>If the diagnosis file does not include cluster monitoring or job execution evidence for these workload types, flag needs_manual_review and recommend running these four test steps manually.</t>
         </is>
       </c>
       <c r="P13" s="3" t="inlineStr">
         <is>
-          <t>Simplifies management and reduces cost while retaining elasticity for varying workloads.</t>
+          <t>Confirms containerized execution actually works for all major workload types, not merely that configuration exists.</t>
         </is>
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>Managed cluster, Node group, Autoscaling, Metrics server</t>
+          <t>Kubernetes, Recipe, Notebook, Webapp, API Deployer, Cluster Monitoring</t>
         </is>
       </c>
       <c r="R13" s="3" t="inlineStr">
@@ -1822,17 +1794,17 @@
       </c>
       <c r="S13" s="3" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>9, 10, 11, 12</t>
         </is>
       </c>
       <c r="T13" s="3" t="inlineStr">
         <is>
-          <t>Recommended settings NICE TO HAVE</t>
+          <t>Additional container execution testing; Webapp MUST HAVE; API MUST HAVE; API MUST HAVE</t>
         </is>
       </c>
       <c r="U13" s="3" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="V13" s="3" t="n"/>
@@ -1845,7 +1817,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>ARCH-015</t>
+          <t>ARCH-013</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1860,72 +1832,64 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Cluster Sizing</t>
+          <t>Cluster Configuration</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Appropriate Cluster Sizing</t>
+          <t>Valid Cluster Configuration for Elastic Compute</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>The Kubernetes cluster must be sized appropriately for the customer's workloads - large enough to avoid resource exhaustion but not so large as to waste resources. Dataiku's memory/disk calculation is only an illustrative baseline (not a mandatory formula), derived from Spark settings (general-settings.json &gt; sparkSettings), container exec settings (general-settings.json &gt; containerSettings), and global flow concurrency (general-settings.json &gt; maxRunningActivities).</t>
+          <t>Environments using Elastic Compute must have at least one valid cluster configured (found under {DATADIR}/config/clusters or Administration &gt; Clusters); Dataiku does not mandate the specific example configuration, only that a workable cluster exists.</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Size the Kubernetes cluster appropriately for workloads, avoiding under- or over-provisioning.</t>
+          <t>Configure at least one valid Kubernetes cluster when using Elastic Compute.</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; sparkSettings, general-settings.json &gt; containerSettings, general-settings.json &gt; maxRunningActivities (used to estimate cluster memory/disk sizing)</t>
+          <t>{DATADIR}/config/clusters</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>greater_than_or_equal</t>
+          <t>exists</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>cluster capacity &gt;= estimated total_memory and disk needs derived from the formulas in notes</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="L14" s="3" t="inlineStr">
-        <is>
-          <t>Illustrative sizing formulas provided by Dataiku, reproduced in full: spark_recipes_memory = global flow concurrency*spark.executor.instances*spark.executor.memory*(1+spark.kubernetes.memoryOverheadFactor) [based on the largest spark config]. spark_notebooks_memory = 30%_DSS_users*spark.executor.instances*spark.executor.memory*(1+spark.kubernetes.memoryOverheadFactor) [using associated spark config]. jupyter_notebooks_memory = 30%_DSS_users * container exec memory limit [using associated container exec config]. total_memory = spark_recipes_memory + spark_notebooks_memory + jupyter_notebooks_memory. DISK = 25GB * spark.executor.instances. Recommended instance sizing: 64 GB &lt; worker size &lt; 128 GB. These are baselines/examples; the cluster need not match this exact calculation, but must be appropriately sized for the customer's workloads based on evidence, and should not be resized without evidence of resource exhaustion.</t>
-        </is>
-      </c>
+          <t>at least one valid cluster configuration present</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="n"/>
+      <c r="L14" s="3" t="n"/>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>Cluster memory/CPU capacity is consistent with or exceeds the estimated total_memory/disk needs given current spark/container/concurrency settings, with no signs of chronic resource exhaustion (OOM kills, pending pods) or gross over-provisioning.</t>
+          <t>The clusters config/directory contains at least one properly defined cluster, consistent with other evidence of elastic-compute usage (spark/container jobs running on Kubernetes).</t>
         </is>
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>Cluster capacity is far below estimated needs (frequent OOM kills/evictions) or drastically oversized relative to workload with no growth justification.</t>
+          <t>No cluster configuration is present despite evidence of Kubernetes-based workloads elsewhere in the diagnosis.</t>
         </is>
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file lacks cluster capacity metrics or the underlying spark/container/concurrency settings needed to compute the estimate, flag needs_manual_review and recommend gathering these values.</t>
+          <t>If the diagnosis file does not clarify whether Elastic Compute is used at all, flag needs_manual_review.</t>
         </is>
       </c>
       <c r="P14" s="3" t="inlineStr">
         <is>
-          <t>Prevents both instability/performance degradation from under-sizing and cost waste from over-sizing.</t>
+          <t>A valid cluster is required to offload computation to Kubernetes.</t>
         </is>
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>Cluster sizing, Spark executor memory, Container exec memory limit, maxRunningActivities, Global flow concurrency</t>
+          <t>Cluster, Managed cluster, Unmanaged cluster, Elastic AI</t>
         </is>
       </c>
       <c r="R14" s="3" t="inlineStr">
@@ -1935,12 +1899,12 @@
       </c>
       <c r="S14" s="3" t="inlineStr">
         <is>
-          <t>14, 15</t>
+          <t>12, 13</t>
         </is>
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>Cluster sizing | MUST HAVE; Cluster sizing | MUST HAVE</t>
+          <t>Cluster configurations | MUST HAVE if using Elastic Compute; Cluster configurations | MUST HAVE if using Elastic Compute</t>
         </is>
       </c>
       <c r="U14" s="3" t="inlineStr">
@@ -1958,12 +1922,12 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>ARCH-016</t>
+          <t>ARCH-014</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>must_have</t>
+          <t>nice_to_have</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1973,64 +1937,68 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Default Compute Settings</t>
+          <t>Cluster Configuration</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Global Default Cluster and Default Execution Config Set (if Elastic AI used)</t>
+          <t>Recommended Cluster Topology (Single Managed Cluster, Node Groups, Autoscaling)</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>If the customer intends to offload most or all recipes to Kubernetes, a default cluster (general-settings.json &gt; defaultK8sClusterId) and a default containerized execution config (general-settings.json &gt; defaultExecutionConfig) should be set globally rather than configured per-recipe or per-project; if this global default is set, the associated execution config must have properly configured resource requests/limits rather than being a resource-hogging default.</t>
+          <t>Dataiku recommends a single managed cluster with one CPU node group serving containerized execution, ML, Spark, webapp, and API workloads, adding a separate GPU node group only if needed, and enabling a metrics server plus cluster autoscaling.</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Set a global default cluster and execution config with proper resource limits when offloading broadly.</t>
+          <t>Use a single managed cluster with one CPU node group and autoscaling enabled.</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; defaultK8sClusterId and general-settings.json &gt; defaultExecutionConfig</t>
+          <t>{DATADIR}/config/clusters (cluster topology / node group / autoscaling settings)</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>exists</t>
+          <t>equals</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>both set to valid, non-resource-hogging values when Elastic AI/offloading is used broadly</t>
+          <t>single managed cluster, one CPU node group for all standard workloads, optional GPU node group only if needed, metrics server installed, autoscaling enabled</t>
         </is>
       </c>
       <c r="K15" s="3" t="n"/>
-      <c r="L15" s="3" t="n"/>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>No literal single field was given for this recommendation; pointer is a best-effort conceptual location within the clusters config.</t>
+        </is>
+      </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>Both defaultK8sClusterId and defaultExecutionConfig are set to valid values, and the referenced execution config has reasonable memory/CPU requests and limits.</t>
+          <t>Cluster configuration shows one managed cluster with a shared CPU node group, autoscaling enabled, metrics server installed, and a GPU node group only present when GPU workloads exist.</t>
         </is>
       </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>These fields are unset despite most recipes being offloaded to Kubernetes, or the default execution config lacks resource limits/requests (resource-hogging risk).</t>
+          <t>Multiple redundant clusters/node groups without clear justification, no autoscaling enabled, or a GPU node group present without any GPU workload evidence.</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not clarify the proportion of recipes offloaded to Kubernetes, flag needs_manual_review to confirm intended usage pattern with the customer.</t>
+          <t>If the diagnosis file does not detail node groups or autoscaling settings, flag needs_manual_review.</t>
         </is>
       </c>
       <c r="P15" s="3" t="inlineStr">
         <is>
-          <t>Setting a global default simplifies configuration management and avoids inconsistent per-recipe settings; an unset or misconfigured default risks uncontrolled resource usage.</t>
+          <t>Simplifies management and reduces cost while retaining elasticity for varying workloads.</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>defaultK8sClusterId, defaultExecutionConfig, Containerized execution, Elastic AI</t>
+          <t>Managed cluster, Node group, Autoscaling, Metrics server</t>
         </is>
       </c>
       <c r="R15" s="3" t="inlineStr">
@@ -2040,17 +2008,17 @@
       </c>
       <c r="S15" s="3" t="inlineStr">
         <is>
-          <t>15, 16</t>
+          <t>14</t>
         </is>
       </c>
       <c r="T15" s="3" t="inlineStr">
         <is>
-          <t>Default Cluster &amp; Default Containerized Execution Config | MUST HAVE if Elastic AI is used; Default Cluster &amp; Default Containerized Execution Config | MUST HAVE if Elastic AI is used</t>
+          <t>Recommended settings NICE TO HAVE</t>
         </is>
       </c>
       <c r="U15" s="3" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="V15" s="3" t="n"/>
@@ -2063,12 +2031,12 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>ARCH-017</t>
+          <t>ARCH-015</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>nice_to_have</t>
+          <t>must_have</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -2078,64 +2046,72 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Containerized Visual Recipes</t>
+          <t>Cluster Sizing</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Containerized Visual Recipes (CDE) Enabled and Base Image Built</t>
+          <t>Appropriate Cluster Sizing</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>If the customer intends to offload visual recipes to Kubernetes, CDE should be enabled (general-settings.json &gt; cdeEnabled) and its base image built via Administration &gt; Settings &gt; Containerized Execution &gt; Build image for containerized visual recipes; a default execution config for visual recipe workloads (general-settings.json &gt; defaultExecutionConfigForVisualRecipesWorkloads) should also be set, validated by confirming a simple recipe (e.g. a sync recipe) shows Engine: DSS (containerized).</t>
+          <t>The Kubernetes cluster must be sized appropriately for the customer's workloads - large enough to avoid resource exhaustion but not so large as to waste resources. Dataiku's memory/disk calculation is only an illustrative baseline (not a mandatory formula), derived from Spark settings (general-settings.json &gt; sparkSettings), container exec settings (general-settings.json &gt; containerSettings), and global flow concurrency (general-settings.json &gt; maxRunningActivities).</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Enable CDE and build its base image to offload visual recipes to Kubernetes.</t>
+          <t>Size the Kubernetes cluster appropriately for workloads, avoiding under- or over-provisioning.</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>general-settings.json &gt; cdeEnabled and general-settings.json &gt; defaultExecutionConfigForVisualRecipesWorkloads</t>
+          <t>general-settings.json &gt; sparkSettings, general-settings.json &gt; containerSettings, general-settings.json &gt; maxRunningActivities (used to estimate cluster memory/disk sizing)</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>equals</t>
+          <t>greater_than_or_equal</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>cdeEnabled=true and defaultExecutionConfigForVisualRecipesWorkloads set to a valid execution config</t>
-        </is>
-      </c>
-      <c r="K16" s="3" t="n"/>
-      <c r="L16" s="3" t="n"/>
+          <t>cluster capacity &gt;= estimated total_memory and disk needs derived from the formulas in notes</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>Illustrative sizing formulas provided by Dataiku, reproduced in full: spark_recipes_memory = global flow concurrency*spark.executor.instances*spark.executor.memory*(1+spark.kubernetes.memoryOverheadFactor) [based on the largest spark config]. spark_notebooks_memory = 30%_DSS_users*spark.executor.instances*spark.executor.memory*(1+spark.kubernetes.memoryOverheadFactor) [using associated spark config]. jupyter_notebooks_memory = 30%_DSS_users * container exec memory limit [using associated container exec config]. total_memory = spark_recipes_memory + spark_notebooks_memory + jupyter_notebooks_memory. DISK = 25GB * spark.executor.instances. Recommended instance sizing: 64 GB &lt; worker size &lt; 128 GB. These are baselines/examples; the cluster need not match this exact calculation, but must be appropriately sized for the customer's workloads based on evidence, and should not be resized without evidence of resource exhaustion.</t>
+        </is>
+      </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>cdeEnabled is true, base CDE image build evidence exists, defaultExecutionConfigForVisualRecipesWorkloads is set, and a sample visual recipe shows Engine: DSS (containerized).</t>
+          <t>Cluster memory/CPU capacity is consistent with or exceeds the estimated total_memory/disk needs given current spark/container/concurrency settings, with no signs of chronic resource exhaustion (OOM kills, pending pods) or gross over-provisioning.</t>
         </is>
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t>cdeEnabled is false or unset while the customer relies on Kubernetes offloading for visual recipes, or a visual recipe fails to show the containerized engine.</t>
+          <t>Cluster capacity is far below estimated needs (frequent OOM kills/evictions) or drastically oversized relative to workload with no growth justification.</t>
         </is>
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t>If the diagnosis file does not indicate whether visual recipe offloading to Kubernetes is desired, flag needs_manual_review.</t>
+          <t>If the diagnosis file lacks cluster capacity metrics or the underlying spark/container/concurrency settings needed to compute the estimate, flag needs_manual_review and recommend gathering these values.</t>
         </is>
       </c>
       <c r="P16" s="3" t="inlineStr">
         <is>
-          <t>Ensures visual recipes can actually be executed on the cluster with an appropriate base image and default resource config.</t>
+          <t>Prevents both instability/performance degradation from under-sizing and cost waste from over-sizing.</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>CDE, cdeEnabled, Visual recipes, Containerized execution</t>
+          <t>Cluster sizing, Spark executor memory, Container exec memory limit, maxRunningActivities, Global flow concurrency</t>
         </is>
       </c>
       <c r="R16" s="3" t="inlineStr">
@@ -2145,12 +2121,12 @@
       </c>
       <c r="S16" s="3" t="inlineStr">
         <is>
-          <t>16, 17, 18</t>
+          <t>14, 15</t>
         </is>
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>Containerized Visual Recipes (CDE) | NICE TO HAVE; Containerized Visual Recipes (CDE) | NICE TO HAVE; Containerized Visual Recipes (CDE) | NICE TO HAVE</t>
+          <t>Cluster sizing | MUST HAVE; Cluster sizing | MUST HAVE</t>
         </is>
       </c>
       <c r="U16" s="3" t="inlineStr">
@@ -2164,6 +2140,216 @@
       <c r="Y16" s="3" t="n"/>
       <c r="Z16" s="3" t="n"/>
       <c r="AA16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-016</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>must_have</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Default Compute Settings</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Global Default Cluster and Default Execution Config Set (if Elastic AI used)</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>If the customer intends to offload most or all recipes to Kubernetes, a default cluster (general-settings.json &gt; defaultK8sClusterId) and a default containerized execution config (general-settings.json &gt; defaultExecutionConfig) should be set globally rather than configured per-recipe or per-project; if this global default is set, the associated execution config must have properly configured resource requests/limits rather than being a resource-hogging default.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Set a global default cluster and execution config with proper resource limits when offloading broadly.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; defaultK8sClusterId and general-settings.json &gt; defaultExecutionConfig</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>exists</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>both set to valid, non-resource-hogging values when Elastic AI/offloading is used broadly</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="3" t="n"/>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>Both defaultK8sClusterId and defaultExecutionConfig are set to valid values, and the referenced execution config has reasonable memory/CPU requests and limits.</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>These fields are unset despite most recipes being offloaded to Kubernetes, or the default execution config lacks resource limits/requests (resource-hogging risk).</t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not clarify the proportion of recipes offloaded to Kubernetes, flag needs_manual_review to confirm intended usage pattern with the customer.</t>
+        </is>
+      </c>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>Setting a global default simplifies configuration management and avoids inconsistent per-recipe settings; an unset or misconfigured default risks uncontrolled resource usage.</t>
+        </is>
+      </c>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>defaultK8sClusterId, defaultExecutionConfig, Containerized execution, Elastic AI</t>
+        </is>
+      </c>
+      <c r="R17" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S17" s="3" t="inlineStr">
+        <is>
+          <t>15, 16</t>
+        </is>
+      </c>
+      <c r="T17" s="3" t="inlineStr">
+        <is>
+          <t>Default Cluster &amp; Default Containerized Execution Config | MUST HAVE if Elastic AI is used; Default Cluster &amp; Default Containerized Execution Config | MUST HAVE if Elastic AI is used</t>
+        </is>
+      </c>
+      <c r="U17" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V17" s="3" t="n"/>
+      <c r="W17" s="3" t="n"/>
+      <c r="X17" s="3" t="n"/>
+      <c r="Y17" s="3" t="n"/>
+      <c r="Z17" s="3" t="n"/>
+      <c r="AA17" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>ARCH-017</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>nice_to_have</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>specific_setting</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Containerized Visual Recipes</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Containerized Visual Recipes (CDE) Enabled and Base Image Built</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>If the customer intends to offload visual recipes to Kubernetes, CDE should be enabled (general-settings.json &gt; cdeEnabled) and its base image built via Administration &gt; Settings &gt; Containerized Execution &gt; Build image for containerized visual recipes; a default execution config for visual recipe workloads (general-settings.json &gt; defaultExecutionConfigForVisualRecipesWorkloads) should also be set, validated by confirming a simple recipe (e.g. a sync recipe) shows Engine: DSS (containerized).</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Enable CDE and build its base image to offload visual recipes to Kubernetes.</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>general-settings.json &gt; cdeEnabled and general-settings.json &gt; defaultExecutionConfigForVisualRecipesWorkloads</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>equals</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>cdeEnabled=true and defaultExecutionConfigForVisualRecipesWorkloads set to a valid execution config</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="n"/>
+      <c r="L18" s="3" t="n"/>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>cdeEnabled is true, base CDE image build evidence exists, defaultExecutionConfigForVisualRecipesWorkloads is set, and a sample visual recipe shows Engine: DSS (containerized).</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>cdeEnabled is false or unset while the customer relies on Kubernetes offloading for visual recipes, or a visual recipe fails to show the containerized engine.</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>If the diagnosis file does not indicate whether visual recipe offloading to Kubernetes is desired, flag needs_manual_review.</t>
+        </is>
+      </c>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>Ensures visual recipes can actually be executed on the cluster with an appropriate base image and default resource config.</t>
+        </is>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>CDE, cdeEnabled, Visual recipes, Containerized execution</t>
+        </is>
+      </c>
+      <c r="R18" s="3" t="inlineStr">
+        <is>
+          <t>architecture_compute_cost</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>16, 17, 18</t>
+        </is>
+      </c>
+      <c r="T18" s="3" t="inlineStr">
+        <is>
+          <t>Containerized Visual Recipes (CDE) | NICE TO HAVE; Containerized Visual Recipes (CDE) | NICE TO HAVE; Containerized Visual Recipes (CDE) | NICE TO HAVE</t>
+        </is>
+      </c>
+      <c r="U18" s="3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="V18" s="3" t="n"/>
+      <c r="W18" s="3" t="n"/>
+      <c r="X18" s="3" t="n"/>
+      <c r="Y18" s="3" t="n"/>
+      <c r="Z18" s="3" t="n"/>
+      <c r="AA18" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>